<commit_message>
Module 2: fill Detail Data actuals from SEC 10-Ks and forecasts from FactSet (S8), add data pull note, verification form, and financials.js
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BxJkWqH3wcE5wkAQrnr3qC
</commit_message>
<xml_diff>
--- a/workbook/QD-HSY.xlsx
+++ b/workbook/QD-HSY.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chrislester/Documents/GitHub/HSY-valuation/workbook/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FCB9D10-3725-DC4E-A664-EDB3473EE0FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBEB0C49-7238-6143-BBD4-31006369D13E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="660" windowWidth="28800" windowHeight="15740" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="15740" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FrontPage" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
     <definedName name="MLNKa7775792bf444a4785f8ed5c82461a24" localSheetId="2" hidden="1">#REF!</definedName>
     <definedName name="MLNKa7775792bf444a4785f8ed5c82461a24" hidden="1">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -2867,6 +2867,7 @@
     <xf numFmtId="194" fontId="46" fillId="13" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="194" fontId="46" fillId="13" borderId="12" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="185" fontId="46" fillId="13" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2951,7 +2952,6 @@
     <xf numFmtId="194" fontId="46" fillId="13" borderId="46" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -3157,10 +3157,10 @@
                 <c:formatCode>#,##0.00_);\(#,##0.00\)</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>-1.8128026589484418E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>-1.8128026589484418E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>169.5</c:v>
@@ -3272,10 +3272,10 @@
                 <c:formatCode>#,##0.00_);\(#,##0.00\)</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>-1.8128026589484418E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>-1.8128026589484418E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>327.85</c:v>
@@ -3840,7 +3840,7 @@
                 <c:formatCode>"$"#,##0.00_);\("$"#,##0.00\);@_)</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>-1.8128026589484418E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -3958,7 +3958,7 @@
                 <c:formatCode>"$"#,##0.00_);\("$"#,##0.00\);@_)</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>-1.8128026589484418E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -4242,7 +4242,7 @@
                 <c:formatCode>"$"#,##0.00_);\("$"#,##0.00\);@_)</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>-1.8128026589484418E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4276,7 +4276,7 @@
                 <c:formatCode>"$"#,##0.00_);\("$"#,##0.00\);@_)</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>-1.8128026589484418E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6509,19 +6509,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="378"/>
-      <c r="B1" s="378"/>
-      <c r="C1" s="378"/>
-      <c r="D1" s="378"/>
-      <c r="E1" s="378"/>
-      <c r="F1" s="378"/>
-      <c r="G1" s="378"/>
-      <c r="H1" s="379"/>
-      <c r="I1" s="379"/>
-      <c r="J1" s="379"/>
-      <c r="K1" s="379"/>
-      <c r="L1" s="379"/>
-      <c r="M1" s="379"/>
+      <c r="A1" s="379"/>
+      <c r="B1" s="379"/>
+      <c r="C1" s="379"/>
+      <c r="D1" s="379"/>
+      <c r="E1" s="379"/>
+      <c r="F1" s="379"/>
+      <c r="G1" s="379"/>
+      <c r="H1" s="380"/>
+      <c r="I1" s="380"/>
+      <c r="J1" s="380"/>
+      <c r="K1" s="380"/>
+      <c r="L1" s="380"/>
+      <c r="M1" s="380"/>
     </row>
     <row r="2" spans="1:18" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
@@ -6533,16 +6533,16 @@
       <c r="E2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="380"/>
-      <c r="G2" s="380"/>
-      <c r="H2" s="381" t="s">
+      <c r="F2" s="381"/>
+      <c r="G2" s="381"/>
+      <c r="H2" s="382" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="381"/>
-      <c r="J2" s="381"/>
-      <c r="K2" s="381"/>
-      <c r="L2" s="381"/>
-      <c r="M2" s="381"/>
+      <c r="I2" s="382"/>
+      <c r="J2" s="382"/>
+      <c r="K2" s="382"/>
+      <c r="L2" s="382"/>
+      <c r="M2" s="382"/>
     </row>
     <row r="3" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
@@ -6554,8 +6554,8 @@
       <c r="E3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="382"/>
-      <c r="G3" s="382"/>
+      <c r="F3" s="383"/>
+      <c r="G3" s="383"/>
       <c r="H3" s="11" t="s">
         <v>5</v>
       </c>
@@ -6575,13 +6575,15 @@
         <v>7</v>
       </c>
       <c r="B4" s="15"/>
-      <c r="C4" s="16"/>
+      <c r="C4" s="16">
+        <v>46299</v>
+      </c>
       <c r="D4" s="17"/>
       <c r="E4" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="383"/>
-      <c r="G4" s="383"/>
+      <c r="F4" s="384"/>
+      <c r="G4" s="384"/>
       <c r="H4" s="19" t="s">
         <v>9</v>
       </c>
@@ -6594,7 +6596,7 @@
       <c r="L4" s="22"/>
       <c r="M4" s="23">
         <f>M3+'Detail Data'!E34-'Detail Data'!E28</f>
-        <v>0</v>
+        <v>3242.2</v>
       </c>
     </row>
     <row r="5" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -6613,15 +6615,15 @@
       <c r="G5" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="H5" s="384" t="s">
+      <c r="H5" s="385" t="s">
         <v>15</v>
       </c>
-      <c r="I5" s="384"/>
-      <c r="K5" s="385" t="s">
+      <c r="I5" s="385"/>
+      <c r="K5" s="386" t="s">
         <v>16</v>
       </c>
-      <c r="L5" s="385"/>
-      <c r="M5" s="385"/>
+      <c r="L5" s="386"/>
+      <c r="M5" s="386"/>
     </row>
     <row r="6" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="30" t="s">
@@ -6638,9 +6640,9 @@
       <c r="H6" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="I6" s="36" t="e">
+      <c r="I6" s="36">
         <f>'Detail Data'!E23</f>
-        <v>#DIV/0!</v>
+        <v>0.41118204367096334</v>
       </c>
       <c r="K6" s="35" t="s">
         <v>19</v>
@@ -6648,7 +6650,7 @@
       <c r="L6" s="37"/>
       <c r="M6" s="38">
         <f>'Detail Data'!E28</f>
-        <v>0</v>
+        <v>1451.5</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -6674,9 +6676,9 @@
       <c r="H7" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="I7" s="36" t="e">
+      <c r="I7" s="36">
         <f>AVERAGE('Detail Data'!C23,'Detail Data'!D23,'Detail Data'!E23)</f>
-        <v>#DIV/0!</v>
+        <v>0.4066217346176888</v>
       </c>
       <c r="K7" s="35" t="s">
         <v>22</v>
@@ -6708,9 +6710,9 @@
       <c r="H8" s="35" t="s">
         <v>24</v>
       </c>
-      <c r="I8" s="36" t="e">
+      <c r="I8" s="36">
         <f>'Detail Data'!E25</f>
-        <v>#DIV/0!</v>
+        <v>0.13910462326678322</v>
       </c>
       <c r="K8" s="35" t="s">
         <v>25</v>
@@ -6744,9 +6746,9 @@
       <c r="H9" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="I9" s="36" t="e">
+      <c r="I9" s="36">
         <f>AVERAGE('Detail Data'!C25,'Detail Data'!D25,'Detail Data'!E25)</f>
-        <v>#DIV/0!</v>
+        <v>0.13764294654242248</v>
       </c>
       <c r="K9" s="35" t="s">
         <v>28</v>
@@ -6758,23 +6760,23 @@
       </c>
     </row>
     <row r="10" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="386" t="s">
+      <c r="A10" s="387" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="386"/>
-      <c r="C10" s="386"/>
+      <c r="B10" s="387"/>
+      <c r="C10" s="387"/>
       <c r="D10" s="17"/>
-      <c r="E10" s="384" t="s">
+      <c r="E10" s="385" t="s">
         <v>30</v>
       </c>
-      <c r="F10" s="384"/>
-      <c r="G10" s="384"/>
+      <c r="F10" s="385"/>
+      <c r="G10" s="385"/>
       <c r="H10" s="35" t="s">
         <v>31</v>
       </c>
-      <c r="I10" s="36" t="e">
+      <c r="I10" s="36">
         <f>'Detail Data'!E26</f>
-        <v>#DIV/0!</v>
+        <v>0.2468263326962957</v>
       </c>
       <c r="K10" s="35" t="s">
         <v>32</v>
@@ -6782,25 +6784,25 @@
       <c r="L10" s="37"/>
       <c r="M10" s="38">
         <f>'Detail Data'!E34</f>
-        <v>0</v>
+        <v>4693.7</v>
       </c>
     </row>
     <row r="11" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="387"/>
-      <c r="B11" s="387"/>
-      <c r="C11" s="387"/>
+      <c r="A11" s="388"/>
+      <c r="B11" s="388"/>
+      <c r="C11" s="388"/>
       <c r="D11" s="17"/>
-      <c r="E11" s="388" t="s">
+      <c r="E11" s="389" t="s">
         <v>33</v>
       </c>
-      <c r="F11" s="388"/>
-      <c r="G11" s="388"/>
+      <c r="F11" s="389"/>
+      <c r="G11" s="389"/>
       <c r="H11" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="I11" s="52" t="e">
+      <c r="I11" s="52">
         <f>AVERAGE('Detail Data'!C26,'Detail Data'!D26,'Detail Data'!E26)</f>
-        <v>#DIV/0!</v>
+        <v>8.2275444232098566E-2</v>
       </c>
       <c r="K11" s="51" t="s">
         <v>35</v>
@@ -6812,17 +6814,17 @@
       </c>
     </row>
     <row r="12" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="387"/>
-      <c r="B12" s="387"/>
-      <c r="C12" s="387"/>
+      <c r="A12" s="388"/>
+      <c r="B12" s="388"/>
+      <c r="C12" s="388"/>
       <c r="D12" s="17"/>
-      <c r="E12" s="388"/>
-      <c r="F12" s="388"/>
-      <c r="G12" s="388"/>
-      <c r="H12" s="384" t="s">
+      <c r="E12" s="389"/>
+      <c r="F12" s="389"/>
+      <c r="G12" s="389"/>
+      <c r="H12" s="385" t="s">
         <v>36</v>
       </c>
-      <c r="I12" s="384"/>
+      <c r="I12" s="385"/>
       <c r="K12" s="55" t="s">
         <v>37</v>
       </c>
@@ -6834,19 +6836,19 @@
       </c>
     </row>
     <row r="13" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="387"/>
-      <c r="B13" s="387"/>
-      <c r="C13" s="387"/>
+      <c r="A13" s="388"/>
+      <c r="B13" s="388"/>
+      <c r="C13" s="388"/>
       <c r="D13" s="17"/>
-      <c r="E13" s="388"/>
-      <c r="F13" s="388"/>
-      <c r="G13" s="388"/>
+      <c r="E13" s="389"/>
+      <c r="F13" s="389"/>
+      <c r="G13" s="389"/>
       <c r="H13" s="58" t="s">
         <v>39</v>
       </c>
-      <c r="I13" s="59" t="e">
+      <c r="I13" s="59">
         <f>('Detail Data'!E5/'Detail Data'!D5)-1</f>
-        <v>#DIV/0!</v>
+        <v>5.1648050903990494E-2</v>
       </c>
       <c r="K13" s="60" t="s">
         <v>40</v>
@@ -6861,19 +6863,19 @@
       </c>
     </row>
     <row r="14" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="387"/>
-      <c r="B14" s="387"/>
-      <c r="C14" s="387"/>
+      <c r="A14" s="388"/>
+      <c r="B14" s="388"/>
+      <c r="C14" s="388"/>
       <c r="D14" s="17"/>
-      <c r="E14" s="388"/>
-      <c r="F14" s="388"/>
-      <c r="G14" s="388"/>
+      <c r="E14" s="389"/>
+      <c r="F14" s="389"/>
+      <c r="G14" s="389"/>
       <c r="H14" s="58" t="s">
         <v>41</v>
       </c>
-      <c r="I14" s="59" t="e">
+      <c r="I14" s="59">
         <f>'Detail Data'!F5/'Detail Data'!E5-1</f>
-        <v>#DIV/0!</v>
+        <v>2.4966453868987104E-2</v>
       </c>
       <c r="K14" s="58" t="s">
         <v>42</v>
@@ -6888,23 +6890,23 @@
       </c>
     </row>
     <row r="15" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="384" t="s">
+      <c r="A15" s="385" t="s">
         <v>43</v>
       </c>
-      <c r="B15" s="384"/>
-      <c r="C15" s="384"/>
+      <c r="B15" s="385"/>
+      <c r="C15" s="385"/>
       <c r="D15" s="17"/>
-      <c r="E15" s="384" t="s">
+      <c r="E15" s="385" t="s">
         <v>44</v>
       </c>
-      <c r="F15" s="384"/>
-      <c r="G15" s="384"/>
+      <c r="F15" s="385"/>
+      <c r="G15" s="385"/>
       <c r="H15" s="58" t="s">
         <v>45</v>
       </c>
-      <c r="I15" s="59" t="e">
+      <c r="I15" s="59">
         <f>(('Detail Data'!G5/'Detail Data'!E5)^(1/2))-1</f>
-        <v>#DIV/0!</v>
+        <v>2.551120927708328E-2</v>
       </c>
       <c r="K15" s="65" t="s">
         <v>46</v>
@@ -6919,15 +6921,15 @@
       </c>
     </row>
     <row r="16" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="389"/>
-      <c r="B16" s="389"/>
-      <c r="C16" s="389"/>
+      <c r="A16" s="390"/>
+      <c r="B16" s="390"/>
+      <c r="C16" s="390"/>
       <c r="D16" s="17"/>
-      <c r="E16" s="390" t="s">
+      <c r="E16" s="391" t="s">
         <v>47</v>
       </c>
-      <c r="F16" s="390"/>
-      <c r="G16" s="390"/>
+      <c r="F16" s="391"/>
+      <c r="G16" s="391"/>
       <c r="H16" s="58" t="s">
         <v>48</v>
       </c>
@@ -6938,9 +6940,9 @@
       <c r="K16" s="60" t="s">
         <v>49</v>
       </c>
-      <c r="L16" s="68" t="e">
+      <c r="L16" s="68">
         <f>'Detail Data'!E11</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="M16" s="62" t="e">
         <f>('Detail Data'!E11*'Detail Data'!E5)/'Detail Data'!E9</f>
@@ -6955,13 +6957,13 @@
       <c r="R16" s="72"/>
     </row>
     <row r="17" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="389"/>
-      <c r="B17" s="389"/>
-      <c r="C17" s="389"/>
+      <c r="A17" s="390"/>
+      <c r="B17" s="390"/>
+      <c r="C17" s="390"/>
       <c r="D17" s="17"/>
-      <c r="E17" s="390"/>
-      <c r="F17" s="390"/>
-      <c r="G17" s="390"/>
+      <c r="E17" s="391"/>
+      <c r="F17" s="391"/>
+      <c r="G17" s="391"/>
       <c r="H17" s="58" t="s">
         <v>51</v>
       </c>
@@ -6972,9 +6974,9 @@
       <c r="K17" s="58" t="s">
         <v>52</v>
       </c>
-      <c r="L17" s="63" t="e">
+      <c r="L17" s="63">
         <f>'Detail Data'!F11</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="M17" s="64" t="e">
         <f>('Detail Data'!E11*'Detail Data'!F5)/'Detail Data'!F9</f>
@@ -6989,13 +6991,13 @@
       <c r="R17" s="72"/>
     </row>
     <row r="18" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="389"/>
-      <c r="B18" s="389"/>
-      <c r="C18" s="389"/>
+      <c r="A18" s="390"/>
+      <c r="B18" s="390"/>
+      <c r="C18" s="390"/>
       <c r="D18" s="17"/>
-      <c r="E18" s="390"/>
-      <c r="F18" s="390"/>
-      <c r="G18" s="390"/>
+      <c r="E18" s="391"/>
+      <c r="F18" s="391"/>
+      <c r="G18" s="391"/>
       <c r="H18" s="65" t="s">
         <v>54</v>
       </c>
@@ -7006,9 +7008,9 @@
       <c r="K18" s="65" t="s">
         <v>55</v>
       </c>
-      <c r="L18" s="66" t="e">
+      <c r="L18" s="66">
         <f>'Detail Data'!G11</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="M18" s="67" t="e">
         <f>('Detail Data'!E11*'Detail Data'!G5)/'Detail Data'!G9</f>
@@ -7023,27 +7025,27 @@
       <c r="R18" s="71"/>
     </row>
     <row r="19" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="386" t="s">
+      <c r="A19" s="387" t="s">
         <v>57</v>
       </c>
-      <c r="B19" s="386"/>
-      <c r="C19" s="386"/>
+      <c r="B19" s="387"/>
+      <c r="C19" s="387"/>
       <c r="D19" s="17"/>
-      <c r="E19" s="385" t="s">
+      <c r="E19" s="386" t="s">
         <v>58</v>
       </c>
-      <c r="F19" s="385"/>
-      <c r="G19" s="385"/>
-      <c r="H19" s="384" t="s">
+      <c r="F19" s="386"/>
+      <c r="G19" s="386"/>
+      <c r="H19" s="385" t="s">
         <v>59</v>
       </c>
-      <c r="I19" s="384"/>
+      <c r="I19" s="385"/>
       <c r="K19" s="60" t="s">
         <v>60</v>
       </c>
-      <c r="L19" s="68" t="e">
+      <c r="L19" s="68">
         <f>'Detail Data'!E13</f>
-        <v>#DIV/0!</v>
+        <v>0.81035221244769529</v>
       </c>
       <c r="M19" s="62" t="e">
         <f>(('Detail Data'!E13*'Detail Data'!E21)-'Detail Data'!E34+'Detail Data'!E28)/'Detail Data'!E9</f>
@@ -7058,30 +7060,30 @@
       <c r="R19" s="74"/>
     </row>
     <row r="20" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="387" t="s">
+      <c r="A20" s="388" t="s">
         <v>62</v>
       </c>
-      <c r="B20" s="387"/>
-      <c r="C20" s="387"/>
+      <c r="B20" s="388"/>
+      <c r="C20" s="388"/>
       <c r="D20" s="17"/>
-      <c r="E20" s="391" t="s">
+      <c r="E20" s="392" t="s">
         <v>63</v>
       </c>
-      <c r="F20" s="391"/>
-      <c r="G20" s="391"/>
+      <c r="F20" s="392"/>
+      <c r="G20" s="392"/>
       <c r="H20" s="60" t="s">
         <v>64</v>
       </c>
-      <c r="I20" s="75" t="e">
+      <c r="I20" s="75">
         <f>'Detail Data'!E35/AVERAGE('Detail Data'!E30,'Detail Data'!D30)</f>
-        <v>#DIV/0!</v>
+        <v>0.34483455126494161</v>
       </c>
       <c r="K20" s="58" t="s">
         <v>65</v>
       </c>
-      <c r="L20" s="63" t="e">
+      <c r="L20" s="63">
         <f>'Detail Data'!F13</f>
-        <v>#DIV/0!</v>
+        <v>0.7247038717661618</v>
       </c>
       <c r="M20" s="64" t="e">
         <f>(('Detail Data'!E13*'Detail Data'!F21)+'Detail Data'!F28-'Detail Data'!F34)/'Detail Data'!F9</f>
@@ -7096,28 +7098,28 @@
       <c r="R20" s="74"/>
     </row>
     <row r="21" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="387"/>
-      <c r="B21" s="387"/>
-      <c r="C21" s="387"/>
+      <c r="A21" s="388"/>
+      <c r="B21" s="388"/>
+      <c r="C21" s="388"/>
       <c r="D21" s="17"/>
-      <c r="E21" s="392" t="s">
+      <c r="E21" s="393" t="s">
         <v>67</v>
       </c>
-      <c r="F21" s="392"/>
-      <c r="G21" s="392"/>
+      <c r="F21" s="393"/>
+      <c r="G21" s="393"/>
       <c r="H21" s="58" t="s">
         <v>68</v>
       </c>
-      <c r="I21" s="59" t="e">
+      <c r="I21" s="59">
         <f>'Detail Data'!E17/AVERAGE('Detail Data'!C35,'Detail Data'!D35,'Detail Data'!E35)</f>
-        <v>#DIV/0!</v>
+        <v>0.36311979450455362</v>
       </c>
       <c r="K21" s="65" t="s">
         <v>69</v>
       </c>
-      <c r="L21" s="66" t="e">
+      <c r="L21" s="66">
         <f>'Detail Data'!G13</f>
-        <v>#DIV/0!</v>
+        <v>0.69199819931348827</v>
       </c>
       <c r="M21" s="67" t="e">
         <f>(('Detail Data'!E13*'Detail Data'!G21)+'Detail Data'!G28-'Detail Data'!G34)/'Detail Data'!G9</f>
@@ -7132,21 +7134,21 @@
       <c r="R21" s="78"/>
     </row>
     <row r="22" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="387"/>
-      <c r="B22" s="387"/>
-      <c r="C22" s="387"/>
+      <c r="A22" s="388"/>
+      <c r="B22" s="388"/>
+      <c r="C22" s="388"/>
       <c r="D22" s="17"/>
-      <c r="E22" s="390" t="s">
+      <c r="E22" s="391" t="s">
         <v>71</v>
       </c>
-      <c r="F22" s="390"/>
-      <c r="G22" s="390"/>
+      <c r="F22" s="391"/>
+      <c r="G22" s="391"/>
       <c r="H22" s="58" t="s">
         <v>72</v>
       </c>
-      <c r="I22" s="59" t="e">
+      <c r="I22" s="59">
         <f>'Detail Data'!E40/AVERAGE('Detail Data'!E30,'Detail Data'!D30,'Detail Data'!C30)</f>
-        <v>#DIV/0!</v>
+        <v>3.2514168398018267E-2</v>
       </c>
       <c r="K22" s="60"/>
       <c r="L22" s="68"/>
@@ -7160,21 +7162,21 @@
       <c r="R22" s="71"/>
     </row>
     <row r="23" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="387"/>
-      <c r="B23" s="387"/>
-      <c r="C23" s="387"/>
+      <c r="A23" s="388"/>
+      <c r="B23" s="388"/>
+      <c r="C23" s="388"/>
       <c r="D23" s="17"/>
-      <c r="E23" s="393" t="s">
+      <c r="E23" s="394" t="s">
         <v>74</v>
       </c>
-      <c r="F23" s="393"/>
-      <c r="G23" s="393"/>
+      <c r="F23" s="394"/>
+      <c r="G23" s="394"/>
       <c r="H23" s="58" t="s">
         <v>75</v>
       </c>
-      <c r="I23" s="59" t="e">
+      <c r="I23" s="59">
         <f>'Detail Data'!E17/'Detail Data'!E35</f>
-        <v>#DIV/0!</v>
+        <v>0.35783021630894107</v>
       </c>
       <c r="K23" s="58"/>
       <c r="L23" s="63"/>
@@ -7188,23 +7190,23 @@
       <c r="R23" s="74"/>
     </row>
     <row r="24" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="384" t="s">
+      <c r="A24" s="385" t="s">
         <v>77</v>
       </c>
-      <c r="B24" s="384"/>
-      <c r="C24" s="384"/>
+      <c r="B24" s="385"/>
+      <c r="C24" s="385"/>
       <c r="D24" s="17"/>
-      <c r="E24" s="391" t="s">
+      <c r="E24" s="392" t="s">
         <v>63</v>
       </c>
-      <c r="F24" s="391"/>
-      <c r="G24" s="391"/>
+      <c r="F24" s="392"/>
+      <c r="G24" s="392"/>
       <c r="H24" s="58" t="s">
         <v>78</v>
       </c>
-      <c r="I24" s="59" t="e">
+      <c r="I24" s="59">
         <f>AVERAGE('Detail Data'!D30,'Detail Data'!E30)/AVERAGE('Detail Data'!D35,'Detail Data'!E35)</f>
-        <v>#DIV/0!</v>
+        <v>2.9441010937665921</v>
       </c>
       <c r="K24" s="65"/>
       <c r="L24" s="66"/>
@@ -7221,51 +7223,51 @@
       <c r="A25" s="79" t="s">
         <v>80</v>
       </c>
-      <c r="B25" s="395" t="s">
+      <c r="B25" s="396" t="s">
         <v>81</v>
       </c>
-      <c r="C25" s="395"/>
+      <c r="C25" s="396"/>
       <c r="D25" s="17"/>
-      <c r="E25" s="392" t="s">
+      <c r="E25" s="393" t="s">
         <v>67</v>
       </c>
-      <c r="F25" s="392"/>
-      <c r="G25" s="392"/>
+      <c r="F25" s="393"/>
+      <c r="G25" s="393"/>
       <c r="H25" s="58" t="s">
         <v>82</v>
       </c>
-      <c r="I25" s="59" t="e">
+      <c r="I25" s="59">
         <f>AVERAGE('Detail Data'!C30,'Detail Data'!D30,'Detail Data'!E30)/AVERAGE('Detail Data'!C35,'Detail Data'!D35,'Detail Data'!E35)</f>
-        <v>#DIV/0!</v>
+        <v>2.8780330745770146</v>
       </c>
     </row>
     <row r="26" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="79" t="s">
         <v>83</v>
       </c>
-      <c r="B26" s="396" t="s">
+      <c r="B26" s="397" t="s">
         <v>84</v>
       </c>
-      <c r="C26" s="396"/>
+      <c r="C26" s="397"/>
       <c r="D26" s="17"/>
-      <c r="E26" s="392" t="s">
+      <c r="E26" s="393" t="s">
         <v>71</v>
       </c>
-      <c r="F26" s="392"/>
-      <c r="G26" s="392"/>
+      <c r="F26" s="393"/>
+      <c r="G26" s="393"/>
       <c r="H26" s="58"/>
       <c r="I26" s="59"/>
     </row>
     <row r="27" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="394" t="s">
+      <c r="A27" s="395" t="s">
         <v>85</v>
       </c>
-      <c r="B27" s="394"/>
-      <c r="C27" s="394"/>
-      <c r="D27" s="394"/>
-      <c r="E27" s="394"/>
-      <c r="F27" s="394"/>
-      <c r="G27" s="394"/>
+      <c r="B27" s="395"/>
+      <c r="C27" s="395"/>
+      <c r="D27" s="395"/>
+      <c r="E27" s="395"/>
+      <c r="F27" s="395"/>
+      <c r="G27" s="395"/>
       <c r="H27" s="65"/>
       <c r="I27" s="54"/>
     </row>
@@ -7277,15 +7279,15 @@
       <c r="E28" s="81"/>
       <c r="F28" s="81"/>
       <c r="G28" s="83"/>
-      <c r="H28" s="384" t="s">
+      <c r="H28" s="385" t="s">
         <v>86</v>
       </c>
-      <c r="I28" s="384"/>
-      <c r="K28" s="384" t="s">
+      <c r="I28" s="385"/>
+      <c r="K28" s="385" t="s">
         <v>87</v>
       </c>
-      <c r="L28" s="384"/>
-      <c r="M28" s="384"/>
+      <c r="L28" s="385"/>
+      <c r="M28" s="385"/>
     </row>
     <row r="29" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="80"/>
@@ -7298,9 +7300,9 @@
       <c r="H29" s="58" t="s">
         <v>88</v>
       </c>
-      <c r="I29" s="59" t="e">
+      <c r="I29" s="59">
         <f>'Detail Data'!E40/'Detail Data'!E5</f>
-        <v>#DIV/0!</v>
+        <v>3.5847598910259015E-2</v>
       </c>
       <c r="K29" s="60" t="s">
         <v>89</v>
@@ -7323,17 +7325,17 @@
       <c r="H30" s="58" t="s">
         <v>90</v>
       </c>
-      <c r="I30" s="59" t="e">
+      <c r="I30" s="59">
         <f>AVERAGE('Detail Data'!E40,'Detail Data'!D40,'Detail Data'!C40)/AVERAGE('Detail Data'!E5,'Detail Data'!D5,'Detail Data'!C5)</f>
-        <v>#DIV/0!</v>
+        <v>4.2660991037583057E-2</v>
       </c>
       <c r="K30" s="58" t="s">
         <v>91</v>
       </c>
       <c r="L30" s="37"/>
-      <c r="M30" s="87" t="e">
+      <c r="M30" s="87">
         <f>'Detail Data'!E11/(1+FrontPage!I13)</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -7617,23 +7619,23 @@
       <c r="B2" s="95"/>
       <c r="C2" s="96" t="str">
         <f>(YEAR(FrontPage!$C$4)-2)&amp;"A"</f>
-        <v>1898A</v>
+        <v>2024A</v>
       </c>
       <c r="D2" s="96" t="str">
         <f>YEAR(FrontPage!$C$4)-1&amp;"A"</f>
-        <v>1899A</v>
+        <v>2025A</v>
       </c>
       <c r="E2" s="97" t="str">
         <f>(YEAR(FrontPage!$C$4))&amp;"F"</f>
-        <v>1900F</v>
+        <v>2026F</v>
       </c>
       <c r="F2" s="97" t="str">
         <f>(YEAR(FrontPage!$C$4)+1)&amp;"F"</f>
-        <v>1901F</v>
+        <v>2027F</v>
       </c>
       <c r="G2" s="97" t="str">
         <f>(YEAR(FrontPage!$C$4)+2)&amp;"F"</f>
-        <v>1902F</v>
+        <v>2028F</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -7669,23 +7671,23 @@
       <c r="B4" s="104"/>
       <c r="C4" s="105">
         <f>C3+C34-C28</f>
-        <v>0</v>
+        <v>2459.5</v>
       </c>
       <c r="D4" s="105">
         <f>D3+D34-D28</f>
-        <v>0</v>
+        <v>3755.2999999999997</v>
       </c>
       <c r="E4" s="105">
         <f>E3+E34-E28</f>
-        <v>0</v>
+        <v>3242.2</v>
       </c>
       <c r="F4" s="105">
         <f>F3+F34-F28</f>
-        <v>0</v>
+        <v>2991.5</v>
       </c>
       <c r="G4" s="106">
         <f>G3+G34-G28</f>
-        <v>0</v>
+        <v>2650.8</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -7694,30 +7696,44 @@
         <v>Revenue (t) - Current FY</v>
       </c>
       <c r="B5" s="108"/>
-      <c r="C5" s="109"/>
-      <c r="D5" s="109"/>
-      <c r="E5" s="109"/>
-      <c r="F5" s="109"/>
-      <c r="G5" s="111"/>
+      <c r="C5" s="109">
+        <v>11202.3</v>
+      </c>
+      <c r="D5" s="109">
+        <v>11692.6</v>
+      </c>
+      <c r="E5" s="109">
+        <v>12296.5</v>
+      </c>
+      <c r="F5" s="109">
+        <v>12603.5</v>
+      </c>
+      <c r="G5" s="111">
+        <v>12931.9</v>
+      </c>
     </row>
     <row r="6" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="107" t="str">
         <f>CONCATENATE("Revenue (t-1) - Previous FY")</f>
         <v>Revenue (t-1) - Previous FY</v>
       </c>
-      <c r="C6" s="109"/>
-      <c r="D6" s="109"/>
+      <c r="C6" s="109">
+        <v>11165</v>
+      </c>
+      <c r="D6" s="109">
+        <v>11202.3</v>
+      </c>
       <c r="E6" s="110">
         <f>D5</f>
-        <v>0</v>
+        <v>11692.6</v>
       </c>
       <c r="F6" s="110">
         <f>E5</f>
-        <v>0</v>
+        <v>12296.5</v>
       </c>
       <c r="G6" s="112">
         <f>F5</f>
-        <v>0</v>
+        <v>12603.5</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -7733,11 +7749,11 @@
         <v>#DIV/0!</v>
       </c>
       <c r="F7" s="114" t="e">
-        <f t="shared" ref="F7:G7" si="0">F5/F9</f>
+        <f>F5/F9</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G7" s="114" t="e">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="G7" si="0">G5/G9</f>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -7788,23 +7804,23 @@
       <c r="B10" s="122"/>
       <c r="C10" s="123" t="str">
         <f t="shared" ref="C10:G10" si="3">C2</f>
-        <v>1898A</v>
+        <v>2024A</v>
       </c>
       <c r="D10" s="123" t="str">
         <f t="shared" si="3"/>
-        <v>1899A</v>
+        <v>2025A</v>
       </c>
       <c r="E10" s="123" t="str">
         <f t="shared" si="3"/>
-        <v>1900F</v>
+        <v>2026F</v>
       </c>
       <c r="F10" s="123" t="str">
         <f t="shared" si="3"/>
-        <v>1901F</v>
+        <v>2027F</v>
       </c>
       <c r="G10" s="29" t="str">
         <f t="shared" si="3"/>
-        <v>1902F</v>
+        <v>2028F</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -7812,25 +7828,25 @@
         <v>98</v>
       </c>
       <c r="B11" s="125"/>
-      <c r="C11" s="126" t="e">
+      <c r="C11" s="126">
         <f>(FrontPage!$C3*C9)/C5</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D11" s="126" t="e">
+        <v>0</v>
+      </c>
+      <c r="D11" s="126">
         <f>(FrontPage!C3*D9)/D5</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E11" s="126" t="e">
+        <v>0</v>
+      </c>
+      <c r="E11" s="126">
         <f>E3/E5</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F11" s="126" t="e">
+        <v>0</v>
+      </c>
+      <c r="F11" s="126">
         <f t="shared" ref="F11:G11" si="4">F3/F5</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G11" s="126" t="e">
+        <v>0</v>
+      </c>
+      <c r="G11" s="126">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -7872,17 +7888,17 @@
         <f t="shared" ref="D13:G13" si="5">$C4/D21</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E13" s="129" t="e">
+      <c r="E13" s="129">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F13" s="129" t="e">
+        <v>0.81035221244769529</v>
+      </c>
+      <c r="F13" s="129">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G13" s="129" t="e">
+        <v>0.7247038717661618</v>
+      </c>
+      <c r="G13" s="129">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+        <v>0.69199819931348827</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
@@ -7892,23 +7908,23 @@
       <c r="B14" s="134"/>
       <c r="C14" s="122" t="str">
         <f>C2</f>
-        <v>1898A</v>
+        <v>2024A</v>
       </c>
       <c r="D14" s="122" t="str">
         <f>D2</f>
-        <v>1899A</v>
+        <v>2025A</v>
       </c>
       <c r="E14" s="122" t="str">
         <f>E2</f>
-        <v>1900F</v>
+        <v>2026F</v>
       </c>
       <c r="F14" s="122" t="str">
         <f>F2</f>
-        <v>1901F</v>
+        <v>2027F</v>
       </c>
       <c r="G14" s="135" t="str">
         <f>G2</f>
-        <v>1902F</v>
+        <v>2028F</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -7916,30 +7932,44 @@
         <v>102</v>
       </c>
       <c r="B15" s="125"/>
-      <c r="C15" s="136"/>
-      <c r="D15" s="136"/>
-      <c r="E15" s="136"/>
-      <c r="F15" s="136"/>
-      <c r="G15" s="136"/>
+      <c r="C15" s="136">
+        <v>5901.4</v>
+      </c>
+      <c r="D15" s="136">
+        <v>7769.9</v>
+      </c>
+      <c r="E15" s="136">
+        <v>7240.4</v>
+      </c>
+      <c r="F15" s="136">
+        <v>7074.5</v>
+      </c>
+      <c r="G15" s="136">
+        <v>7220.6</v>
+      </c>
     </row>
     <row r="16" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="107" t="s">
         <v>103</v>
       </c>
       <c r="B16" s="137"/>
-      <c r="C16" s="138"/>
-      <c r="D16" s="138"/>
-      <c r="E16" s="139" t="e">
+      <c r="C16" s="138">
+        <v>2898.2</v>
+      </c>
+      <c r="D16" s="138">
+        <v>1441.5</v>
+      </c>
+      <c r="E16" s="139">
         <f>E21-E38</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F16" s="139" t="e">
+        <v>2546.6904971403433</v>
+      </c>
+      <c r="F16" s="139">
         <f t="shared" ref="F16:G16" si="6">F21-F38</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G16" s="139" t="e">
+        <v>2835.4752529696439</v>
+      </c>
+      <c r="G16" s="139">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
+        <v>2985.2383853937527</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -7947,38 +7977,56 @@
         <v>104</v>
       </c>
       <c r="B17" s="137"/>
-      <c r="C17" s="138"/>
-      <c r="D17" s="138"/>
-      <c r="E17" s="138"/>
-      <c r="F17" s="138"/>
-      <c r="G17" s="138"/>
+      <c r="C17" s="138">
+        <v>2221.1999999999998</v>
+      </c>
+      <c r="D17" s="138">
+        <v>883.3</v>
+      </c>
+      <c r="E17" s="138">
+        <v>1710.5</v>
+      </c>
+      <c r="F17" s="138">
+        <v>1988.8</v>
+      </c>
+      <c r="G17" s="138">
+        <v>2108.4</v>
+      </c>
     </row>
     <row r="18" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="107" t="str">
         <f>CONCATENATE("Net Income (t-1) - Previous FY")</f>
         <v>Net Income (t-1) - Previous FY</v>
       </c>
-      <c r="C18" s="138"/>
-      <c r="D18" s="138"/>
+      <c r="C18" s="138">
+        <v>1861.8</v>
+      </c>
+      <c r="D18" s="138">
+        <v>2221.1999999999998</v>
+      </c>
       <c r="E18" s="139">
         <f>D17</f>
-        <v>0</v>
+        <v>883.3</v>
       </c>
       <c r="F18" s="139">
         <f>E17</f>
-        <v>0</v>
+        <v>1710.5</v>
       </c>
       <c r="G18" s="139">
         <f>F17</f>
-        <v>0</v>
+        <v>1988.8</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="107" t="s">
         <v>237</v>
       </c>
-      <c r="C19" s="138"/>
-      <c r="D19" s="138"/>
+      <c r="C19" s="138">
+        <v>165.7</v>
+      </c>
+      <c r="D19" s="138">
+        <v>190.2</v>
+      </c>
       <c r="E19" s="139">
         <f>'WACC calculation'!$D$13*'Detail Data'!E34</f>
         <v>0</v>
@@ -7996,11 +8044,21 @@
       <c r="A20" s="107" t="s">
         <v>105</v>
       </c>
-      <c r="C20" s="138"/>
-      <c r="D20" s="138"/>
-      <c r="E20" s="138"/>
-      <c r="F20" s="138"/>
-      <c r="G20" s="138"/>
+      <c r="C20" s="138">
+        <v>252.7</v>
+      </c>
+      <c r="D20" s="138">
+        <v>330.9</v>
+      </c>
+      <c r="E20" s="138">
+        <v>597.70000000000005</v>
+      </c>
+      <c r="F20" s="138">
+        <v>689.8</v>
+      </c>
+      <c r="G20" s="138">
+        <v>707.8</v>
+      </c>
     </row>
     <row r="21" spans="1:7" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A21" s="141" t="s">
@@ -8009,9 +8067,15 @@
       <c r="B21" s="142"/>
       <c r="C21" s="353"/>
       <c r="D21" s="353"/>
-      <c r="E21" s="353"/>
-      <c r="F21" s="353"/>
-      <c r="G21" s="354"/>
+      <c r="E21" s="353">
+        <v>3035.1</v>
+      </c>
+      <c r="F21" s="353">
+        <v>3393.8</v>
+      </c>
+      <c r="G21" s="354">
+        <v>3554.2</v>
+      </c>
     </row>
     <row r="22" spans="1:7" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A22" s="133" t="s">
@@ -8020,23 +8084,23 @@
       <c r="B22" s="134"/>
       <c r="C22" s="123" t="str">
         <f>C2</f>
-        <v>1898A</v>
+        <v>2024A</v>
       </c>
       <c r="D22" s="123" t="str">
         <f>D2</f>
-        <v>1899A</v>
+        <v>2025A</v>
       </c>
       <c r="E22" s="123" t="str">
         <f>E2</f>
-        <v>1900F</v>
+        <v>2026F</v>
       </c>
       <c r="F22" s="123" t="str">
         <f>F2</f>
-        <v>1901F</v>
+        <v>2027F</v>
       </c>
       <c r="G22" s="29" t="str">
         <f>G2</f>
-        <v>1902F</v>
+        <v>2028F</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -8044,25 +8108,25 @@
         <v>108</v>
       </c>
       <c r="B23" s="125"/>
-      <c r="C23" s="143" t="e">
+      <c r="C23" s="143">
         <f>(C5-C15)/C5</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D23" s="143" t="e">
+        <v>0.4731974683770297</v>
+      </c>
+      <c r="D23" s="143">
         <f>(D5-D15)/D5</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E23" s="143" t="e">
+        <v>0.33548569180507337</v>
+      </c>
+      <c r="E23" s="143">
         <f>(E5-E15)/E5</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F23" s="143" t="e">
+        <v>0.41118204367096334</v>
+      </c>
+      <c r="F23" s="143">
         <f>(F5-F15)/F5</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G23" s="144" t="e">
+        <v>0.43868766612448923</v>
+      </c>
+      <c r="G23" s="144">
         <f>(G5-G15)/G5</f>
-        <v>#DIV/0!</v>
+        <v>0.44164430594112231</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -8070,50 +8134,50 @@
         <v>109</v>
       </c>
       <c r="B24" s="132"/>
-      <c r="C24" s="145" t="e">
+      <c r="C24" s="145">
         <f>C16/C5</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D24" s="145" t="e">
+        <v>0.25871472822545372</v>
+      </c>
+      <c r="D24" s="145">
         <f>D16/D5</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E24" s="145" t="e">
+        <v>0.12328310213297299</v>
+      </c>
+      <c r="E24" s="145">
         <f>E16/E5</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F24" s="145" t="e">
+        <v>0.2071069407669128</v>
+      </c>
+      <c r="F24" s="145">
         <f>F16/F5</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G24" s="146" t="e">
+        <v>0.22497522537149553</v>
+      </c>
+      <c r="G24" s="146">
         <f>G16/G5</f>
-        <v>#DIV/0!</v>
+        <v>0.23084298404671802</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="131" t="s">
         <v>110</v>
       </c>
-      <c r="C25" s="145" t="e">
+      <c r="C25" s="145">
         <f>C17/C5</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D25" s="145" t="e">
+        <v>0.1982807102112959</v>
+      </c>
+      <c r="D25" s="145">
         <f>D17/D5</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E25" s="145" t="e">
+        <v>7.5543506149188366E-2</v>
+      </c>
+      <c r="E25" s="145">
         <f>E17/E5</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F25" s="145" t="e">
+        <v>0.13910462326678322</v>
+      </c>
+      <c r="F25" s="145">
         <f>F17/F5</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G25" s="146" t="e">
+        <v>0.1577974372198199</v>
+      </c>
+      <c r="G25" s="146">
         <f>G17/G5</f>
-        <v>#DIV/0!</v>
+        <v>0.16303868727719825</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
@@ -8121,25 +8185,25 @@
         <v>111</v>
       </c>
       <c r="B26" s="148"/>
-      <c r="C26" s="149" t="e">
+      <c r="C26" s="149">
         <f>C21/C5</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D26" s="149" t="e">
+        <v>0</v>
+      </c>
+      <c r="D26" s="149">
         <f>D21/D5</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E26" s="149" t="e">
+        <v>0</v>
+      </c>
+      <c r="E26" s="149">
         <f>E21/E5</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F26" s="149" t="e">
+        <v>0.2468263326962957</v>
+      </c>
+      <c r="F26" s="149">
         <f>F21/F5</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G26" s="150" t="e">
+        <v>0.26927440790256674</v>
+      </c>
+      <c r="G26" s="150">
         <f>G21/G5</f>
-        <v>#DIV/0!</v>
+        <v>0.27483973739357714</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
@@ -8149,23 +8213,23 @@
       <c r="B27" s="152"/>
       <c r="C27" s="123" t="str">
         <f>C2</f>
-        <v>1898A</v>
+        <v>2024A</v>
       </c>
       <c r="D27" s="123" t="str">
         <f>D2</f>
-        <v>1899A</v>
+        <v>2025A</v>
       </c>
       <c r="E27" s="123" t="str">
         <f>E2</f>
-        <v>1900F</v>
+        <v>2026F</v>
       </c>
       <c r="F27" s="123" t="str">
         <f>F2</f>
-        <v>1901F</v>
+        <v>2027F</v>
       </c>
       <c r="G27" s="29" t="str">
         <f>G2</f>
-        <v>1902F</v>
+        <v>2028F</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -8173,11 +8237,21 @@
         <v>113</v>
       </c>
       <c r="B28" s="125"/>
-      <c r="C28" s="136"/>
-      <c r="D28" s="136"/>
-      <c r="E28" s="136"/>
-      <c r="F28" s="136"/>
-      <c r="G28" s="136"/>
+      <c r="C28" s="136">
+        <v>730.7</v>
+      </c>
+      <c r="D28" s="136">
+        <v>925.9</v>
+      </c>
+      <c r="E28" s="136">
+        <v>1451.5</v>
+      </c>
+      <c r="F28" s="136">
+        <v>1635.5</v>
+      </c>
+      <c r="G28" s="136">
+        <v>1909.5</v>
+      </c>
     </row>
     <row r="29" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="127" t="s">
@@ -8210,33 +8284,63 @@
         <v>115</v>
       </c>
       <c r="B30" s="128"/>
-      <c r="C30" s="355"/>
-      <c r="D30" s="355"/>
-      <c r="E30" s="355"/>
-      <c r="F30" s="355"/>
-      <c r="G30" s="356"/>
+      <c r="C30" s="355">
+        <v>12946.9</v>
+      </c>
+      <c r="D30" s="355">
+        <v>13741.3</v>
+      </c>
+      <c r="E30" s="355">
+        <v>13983.3</v>
+      </c>
+      <c r="F30" s="355">
+        <v>14093.3</v>
+      </c>
+      <c r="G30" s="356">
+        <v>14406</v>
+      </c>
     </row>
     <row r="31" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="131" t="s">
         <v>116</v>
       </c>
       <c r="B31" s="132"/>
-      <c r="C31" s="138"/>
-      <c r="D31" s="138"/>
-      <c r="E31" s="138"/>
-      <c r="F31" s="138"/>
-      <c r="G31" s="138"/>
+      <c r="C31" s="138">
+        <v>3759.5</v>
+      </c>
+      <c r="D31" s="138">
+        <v>3588.9</v>
+      </c>
+      <c r="E31" s="138">
+        <v>4123</v>
+      </c>
+      <c r="F31" s="138">
+        <v>4242</v>
+      </c>
+      <c r="G31" s="138">
+        <v>4541</v>
+      </c>
     </row>
     <row r="32" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="131" t="s">
         <v>117</v>
       </c>
       <c r="B32" s="132"/>
-      <c r="C32" s="138"/>
-      <c r="D32" s="138"/>
-      <c r="E32" s="138"/>
-      <c r="F32" s="138"/>
-      <c r="G32" s="138"/>
+      <c r="C32" s="138">
+        <v>3929.5</v>
+      </c>
+      <c r="D32" s="138">
+        <v>3011.9</v>
+      </c>
+      <c r="E32" s="138">
+        <v>3261.5</v>
+      </c>
+      <c r="F32" s="138">
+        <v>3192.5</v>
+      </c>
+      <c r="G32" s="138">
+        <v>3195.5</v>
+      </c>
     </row>
     <row r="33" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="131" t="s">
@@ -8245,45 +8349,65 @@
       <c r="B33" s="132"/>
       <c r="C33" s="139">
         <f t="shared" ref="C33:G33" si="7">C31-C32</f>
-        <v>0</v>
+        <v>-170</v>
       </c>
       <c r="D33" s="139">
         <f>D31-D32</f>
-        <v>0</v>
+        <v>577</v>
       </c>
       <c r="E33" s="139">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>861.5</v>
       </c>
       <c r="F33" s="139">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1049.5</v>
       </c>
       <c r="G33" s="140">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1345.5</v>
       </c>
     </row>
     <row r="34" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="131" t="s">
         <v>119</v>
       </c>
-      <c r="C34" s="138"/>
-      <c r="D34" s="138"/>
-      <c r="E34" s="355"/>
-      <c r="F34" s="355"/>
-      <c r="G34" s="356"/>
+      <c r="C34" s="138">
+        <v>3190.2</v>
+      </c>
+      <c r="D34" s="138">
+        <v>4681.2</v>
+      </c>
+      <c r="E34" s="355">
+        <v>4693.7</v>
+      </c>
+      <c r="F34" s="355">
+        <v>4627</v>
+      </c>
+      <c r="G34" s="356">
+        <v>4560.3</v>
+      </c>
     </row>
     <row r="35" spans="1:10" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A35" s="147" t="s">
         <v>120</v>
       </c>
       <c r="B35" s="92"/>
-      <c r="C35" s="156"/>
-      <c r="D35" s="156"/>
-      <c r="E35" s="353"/>
-      <c r="F35" s="353"/>
-      <c r="G35" s="354"/>
+      <c r="C35" s="156">
+        <v>4714.7</v>
+      </c>
+      <c r="D35" s="156">
+        <v>4636.8</v>
+      </c>
+      <c r="E35" s="353">
+        <v>4780.2</v>
+      </c>
+      <c r="F35" s="353">
+        <v>5081.8</v>
+      </c>
+      <c r="G35" s="354">
+        <v>5441.8</v>
+      </c>
     </row>
     <row r="36" spans="1:10" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A36" s="151" t="s">
@@ -8292,23 +8416,23 @@
       <c r="B36" s="152"/>
       <c r="C36" s="123" t="str">
         <f>C2</f>
-        <v>1898A</v>
+        <v>2024A</v>
       </c>
       <c r="D36" s="123" t="str">
         <f>D2</f>
-        <v>1899A</v>
+        <v>2025A</v>
       </c>
       <c r="E36" s="123" t="str">
         <f>E2</f>
-        <v>1900F</v>
+        <v>2026F</v>
       </c>
       <c r="F36" s="123" t="str">
         <f>F2</f>
-        <v>1901F</v>
+        <v>2027F</v>
       </c>
       <c r="G36" s="29" t="str">
         <f>G2</f>
-        <v>1902F</v>
+        <v>2028F</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.15">
@@ -8317,17 +8441,17 @@
       </c>
       <c r="C37" s="138"/>
       <c r="D37" s="138"/>
-      <c r="E37" s="139" t="e">
+      <c r="E37" s="139">
         <f>E16*(1-E20/E16)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F37" s="139" t="e">
+        <v>1948.9904971403432</v>
+      </c>
+      <c r="F37" s="139">
         <f t="shared" ref="F37:G37" si="8">F16*(1-F20/F16)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G37" s="139" t="e">
+        <v>2145.6752529696437</v>
+      </c>
+      <c r="G37" s="139">
         <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
+        <v>2277.4383853937525</v>
       </c>
     </row>
     <row r="38" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -8335,19 +8459,23 @@
         <v>123</v>
       </c>
       <c r="B38" s="132"/>
-      <c r="C38" s="138"/>
-      <c r="D38" s="138"/>
-      <c r="E38" s="139" t="e">
+      <c r="C38" s="138">
+        <v>455.3</v>
+      </c>
+      <c r="D38" s="138">
+        <v>503.7</v>
+      </c>
+      <c r="E38" s="139">
         <f>D38/D40*E40</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F38" s="139" t="e">
+        <v>488.40950285965675</v>
+      </c>
+      <c r="F38" s="139">
         <f t="shared" ref="F38:G38" si="9">E38/E40*F40</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G38" s="139" t="e">
+        <v>558.32474703035621</v>
+      </c>
+      <c r="G38" s="139">
         <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
+        <v>568.96161460624717</v>
       </c>
     </row>
     <row r="39" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -8358,15 +8486,15 @@
       <c r="D39" s="138"/>
       <c r="E39" s="139">
         <f>E33-D33</f>
-        <v>0</v>
+        <v>284.5</v>
       </c>
       <c r="F39" s="139">
         <f t="shared" ref="F39:G39" si="10">F33-E33</f>
-        <v>0</v>
+        <v>188</v>
       </c>
       <c r="G39" s="139">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>296</v>
       </c>
     </row>
     <row r="40" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -8374,11 +8502,21 @@
         <v>125</v>
       </c>
       <c r="B40" s="132"/>
-      <c r="C40" s="138"/>
-      <c r="D40" s="138"/>
-      <c r="E40" s="355"/>
-      <c r="F40" s="355"/>
-      <c r="G40" s="355"/>
+      <c r="C40" s="138">
+        <v>605.9</v>
+      </c>
+      <c r="D40" s="138">
+        <v>454.6</v>
+      </c>
+      <c r="E40" s="355">
+        <v>440.8</v>
+      </c>
+      <c r="F40" s="355">
+        <v>503.9</v>
+      </c>
+      <c r="G40" s="355">
+        <v>513.5</v>
+      </c>
     </row>
     <row r="41" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A41" s="131" t="s">
@@ -8388,17 +8526,17 @@
         <v>235</v>
       </c>
       <c r="D41" s="138"/>
-      <c r="E41" s="139" t="e">
+      <c r="E41" s="139">
         <f>E37+E38-E39-E40</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F41" s="139" t="e">
+        <v>1712.1000000000001</v>
+      </c>
+      <c r="F41" s="139">
         <f t="shared" ref="F41:G41" si="11">F37+F38-F39-F40</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G41" s="139" t="e">
+        <v>2012.1</v>
+      </c>
+      <c r="G41" s="139">
         <f t="shared" si="11"/>
-        <v>#DIV/0!</v>
+        <v>2036.8999999999996</v>
       </c>
     </row>
     <row r="42" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -8409,17 +8547,17 @@
         <v>236</v>
       </c>
       <c r="D42" s="138"/>
-      <c r="E42" s="139" t="e">
+      <c r="E42" s="139">
         <f>E41+E19*(1-'DCF 1-Pager'!E25)+'Detail Data'!E34-'Detail Data'!D34</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F42" s="139" t="e">
+        <v>1724.6000000000004</v>
+      </c>
+      <c r="F42" s="139">
         <f>F41+F19*(1-'DCF 1-Pager'!F25)+'Detail Data'!F34-'Detail Data'!E34</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G42" s="139" t="e">
+        <v>1945.4000000000005</v>
+      </c>
+      <c r="G42" s="139">
         <f>G41+G19*(1-'DCF 1-Pager'!G25)+'Detail Data'!G34-'Detail Data'!F34</f>
-        <v>#DIV/0!</v>
+        <v>1970.1999999999998</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
@@ -8427,21 +8565,21 @@
       <c r="A44" s="88" t="s">
         <v>257</v>
       </c>
-      <c r="D44" s="349" t="e">
+      <c r="D44" s="349">
         <f>(D33+D40)/D17</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E44" s="349" t="e">
+        <v>1.1678931280425675</v>
+      </c>
+      <c r="E44" s="349">
         <f t="shared" ref="E44:G44" si="12">(E33+E40)/E17</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F44" s="349" t="e">
+        <v>0.7613563285589009</v>
+      </c>
+      <c r="F44" s="349">
         <f t="shared" si="12"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G44" s="349" t="e">
+        <v>0.78107401448109415</v>
+      </c>
+      <c r="G44" s="349">
         <f t="shared" si="12"/>
-        <v>#DIV/0!</v>
+        <v>0.88171125023714658</v>
       </c>
     </row>
     <row r="45" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -8473,21 +8611,21 @@
       <c r="A46" s="88" t="s">
         <v>64</v>
       </c>
-      <c r="D46" s="349" t="e">
+      <c r="D46" s="349">
         <f>D17/D35</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E46" s="349" t="e">
+        <v>0.190497757073844</v>
+      </c>
+      <c r="E46" s="349">
         <f t="shared" ref="E46:G46" si="14">E17/E35</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F46" s="349" t="e">
+        <v>0.35783021630894107</v>
+      </c>
+      <c r="F46" s="349">
         <f t="shared" si="14"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G46" s="349" t="e">
+        <v>0.39135739304970679</v>
+      </c>
+      <c r="G46" s="349">
         <f t="shared" si="14"/>
-        <v>#DIV/0!</v>
+        <v>0.38744533058914332</v>
       </c>
       <c r="J46" s="88" t="s">
         <v>274</v>
@@ -8497,21 +8635,21 @@
       <c r="A47" s="88" t="s">
         <v>256</v>
       </c>
-      <c r="D47" s="349" t="e">
+      <c r="D47" s="349">
         <f>D16*(1-'DCF 1-Pager'!D25)/(C34+C35-C28)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E47" s="349" t="e">
+        <v>0.12565697674677329</v>
+      </c>
+      <c r="E47" s="349">
         <f>E16*(1-'DCF 1-Pager'!E25)/(D34+D35-D28)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F47" s="349" t="e">
+        <v>0.23224109545171567</v>
+      </c>
+      <c r="F47" s="349">
         <f>F16*(1-'DCF 1-Pager'!F25)/(E34+E35-E28)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G47" s="349" t="e">
+        <v>0.26746051717312075</v>
+      </c>
+      <c r="G47" s="349">
         <f>G16*(1-'DCF 1-Pager'!G25)/(F34+F35-F28)</f>
-        <v>#DIV/0!</v>
+        <v>0.28209510180394048</v>
       </c>
       <c r="J47" s="88" t="s">
         <v>275</v>
@@ -8522,42 +8660,42 @@
       <c r="A49" s="88" t="s">
         <v>259</v>
       </c>
-      <c r="D49" s="406" t="e">
+      <c r="D49" s="378">
         <f>D46*D44</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E49" s="349" t="e">
+        <v>0.22248102139406481</v>
+      </c>
+      <c r="E49" s="349">
         <f t="shared" ref="E49:G49" si="15">E46*E44</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F49" s="349" t="e">
+        <v>0.2724362997364127</v>
+      </c>
+      <c r="F49" s="349">
         <f t="shared" si="15"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G49" s="349" t="e">
+        <v>0.30567909008618993</v>
+      </c>
+      <c r="G49" s="349">
         <f t="shared" si="15"/>
-        <v>#DIV/0!</v>
+        <v>0.34161490683229812</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A50" s="88" t="s">
         <v>258</v>
       </c>
-      <c r="D50" s="349" t="e">
+      <c r="D50" s="349">
         <f>D47*D44</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E50" s="349" t="e">
+        <v>0.14675391963316123</v>
+      </c>
+      <c r="E50" s="349">
         <f t="shared" ref="E50:G50" si="16">E47*E44</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F50" s="349" t="e">
+        <v>0.1768182277736155</v>
+      </c>
+      <c r="F50" s="349">
         <f t="shared" si="16"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G50" s="349" t="e">
+        <v>0.20890645986359904</v>
+      </c>
+      <c r="G50" s="349">
         <f t="shared" si="16"/>
-        <v>#DIV/0!</v>
+        <v>0.24872642489732752</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
@@ -8573,42 +8711,42 @@
       <c r="A53" s="88" t="s">
         <v>262</v>
       </c>
-      <c r="D53" s="349" t="e">
+      <c r="D53" s="349">
         <f>$B$52/D46</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E53" s="349" t="e">
+        <v>0.15748216913845808</v>
+      </c>
+      <c r="E53" s="349">
         <f t="shared" ref="E53:G54" si="17">$B$52/E46</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F53" s="349" t="e">
+        <v>8.3838643671441088E-2</v>
+      </c>
+      <c r="F53" s="349">
         <f t="shared" si="17"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G53" s="349" t="e">
+        <v>7.6656275140788419E-2</v>
+      </c>
+      <c r="G53" s="349">
         <f t="shared" si="17"/>
-        <v>#DIV/0!</v>
+        <v>7.7430278884462148E-2</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A54" s="88" t="s">
         <v>261</v>
       </c>
-      <c r="D54" s="349" t="e">
+      <c r="D54" s="349">
         <f>$B$52/D47</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E54" s="349" t="e">
+        <v>0.23874519964344409</v>
+      </c>
+      <c r="E54" s="349">
         <f t="shared" si="17"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F54" s="349" t="e">
+        <v>0.12917610443426961</v>
+      </c>
+      <c r="F54" s="349">
         <f t="shared" si="17"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G54" s="349" t="e">
+        <v>0.11216608835232948</v>
+      </c>
+      <c r="G54" s="349">
         <f t="shared" si="17"/>
-        <v>#DIV/0!</v>
+        <v>0.10634711417587946</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
@@ -8616,9 +8754,9 @@
       <c r="A56" s="88" t="s">
         <v>264</v>
       </c>
-      <c r="D56" s="155" t="e">
+      <c r="D56" s="155">
         <f>D16/D19</f>
-        <v>#DIV/0!</v>
+        <v>7.5788643533123032</v>
       </c>
       <c r="E56" s="155" t="e">
         <f t="shared" ref="E56:G56" si="18">E16/E19</f>
@@ -8733,20 +8871,20 @@
       <c r="B3" s="165" t="s">
         <v>128</v>
       </c>
-      <c r="L3" s="400" t="s">
+      <c r="L3" s="401" t="s">
         <v>246</v>
       </c>
-      <c r="M3" s="401"/>
-      <c r="N3" s="402"/>
-      <c r="P3" s="403" t="s">
+      <c r="M3" s="402"/>
+      <c r="N3" s="403"/>
+      <c r="P3" s="404" t="s">
         <v>289</v>
       </c>
-      <c r="Q3" s="404"/>
-      <c r="R3" s="404"/>
-      <c r="S3" s="404"/>
-      <c r="T3" s="404"/>
-      <c r="U3" s="404"/>
-      <c r="V3" s="405"/>
+      <c r="Q3" s="405"/>
+      <c r="R3" s="405"/>
+      <c r="S3" s="405"/>
+      <c r="T3" s="405"/>
+      <c r="U3" s="405"/>
+      <c r="V3" s="406"/>
     </row>
     <row r="4" spans="2:22" ht="21" x14ac:dyDescent="0.25">
       <c r="B4" s="162" t="s">
@@ -8757,10 +8895,10 @@
         <v>0</v>
       </c>
       <c r="L4" s="339"/>
-      <c r="M4" s="398" t="s">
+      <c r="M4" s="399" t="s">
         <v>249</v>
       </c>
-      <c r="N4" s="399"/>
+      <c r="N4" s="400"/>
       <c r="P4" s="371"/>
       <c r="Q4" s="372"/>
       <c r="R4" s="372" t="s">
@@ -8801,9 +8939,9 @@
         <f>AVERAGE('Relative Valuation'!D4:D6)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="R5" s="372" t="e">
+      <c r="R5" s="372">
         <f>D21-D24</f>
-        <v>#DIV/0!</v>
+        <v>901.48828257670107</v>
       </c>
       <c r="S5" s="372" t="e">
         <f>R5*Q5</f>
@@ -8832,9 +8970,9 @@
       <c r="F6" s="162" t="s">
         <v>132</v>
       </c>
-      <c r="H6" s="167" t="e">
+      <c r="H6" s="167">
         <f>'WACC calculation'!D16</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="L6" s="340"/>
       <c r="M6" s="337"/>
@@ -8887,11 +9025,11 @@
       </c>
       <c r="M7" s="338">
         <f>C77</f>
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="N7" s="342">
         <f>D77</f>
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="P7" s="375" t="s">
         <v>281</v>
@@ -8902,7 +9040,7 @@
       </c>
       <c r="R7" s="376">
         <f>D17</f>
-        <v>0</v>
+        <v>11692.6</v>
       </c>
       <c r="S7" s="376" t="e">
         <f>R7*Q7</f>
@@ -8933,7 +9071,7 @@
       </c>
       <c r="H8" s="170">
         <f>D9</f>
-        <v>0</v>
+        <v>46299</v>
       </c>
       <c r="J8" s="171"/>
       <c r="L8" s="343" t="s">
@@ -8954,7 +9092,7 @@
       </c>
       <c r="D9" s="166">
         <f>FrontPage!C4</f>
-        <v>0</v>
+        <v>46299</v>
       </c>
       <c r="F9" s="162" t="s">
         <v>138</v>
@@ -8971,7 +9109,7 @@
       </c>
       <c r="D10" s="173">
         <f>YEARFRAC(D9,D7)</f>
-        <v>127.00277777777778</v>
+        <v>0.24166666666666667</v>
       </c>
     </row>
     <row r="11" spans="2:22" ht="16" thickBot="1" x14ac:dyDescent="0.25">
@@ -9002,11 +9140,11 @@
       <c r="D14" s="177" t="s">
         <v>141</v>
       </c>
-      <c r="E14" s="397" t="s">
+      <c r="E14" s="398" t="s">
         <v>142</v>
       </c>
-      <c r="F14" s="397"/>
-      <c r="G14" s="397"/>
+      <c r="F14" s="398"/>
+      <c r="G14" s="398"/>
       <c r="H14" s="177"/>
       <c r="I14" s="177"/>
       <c r="J14" s="255"/>
@@ -9018,19 +9156,19 @@
       <c r="C15" s="297"/>
       <c r="D15" s="329" t="str">
         <f>'Detail Data'!D2</f>
-        <v>1899A</v>
+        <v>2025A</v>
       </c>
       <c r="E15" s="329" t="str">
         <f>'Detail Data'!E2</f>
-        <v>1900F</v>
+        <v>2026F</v>
       </c>
       <c r="F15" s="329" t="str">
         <f>'Detail Data'!F2</f>
-        <v>1901F</v>
+        <v>2027F</v>
       </c>
       <c r="G15" s="329" t="str">
         <f>'Detail Data'!G2</f>
-        <v>1902F</v>
+        <v>2028F</v>
       </c>
       <c r="H15" s="329"/>
       <c r="I15" s="329"/>
@@ -9053,19 +9191,19 @@
       <c r="C17" s="262"/>
       <c r="D17" s="302">
         <f>'Detail Data'!D5</f>
-        <v>0</v>
+        <v>11692.6</v>
       </c>
       <c r="E17" s="262">
         <f>'Detail Data'!E5</f>
-        <v>0</v>
+        <v>12296.5</v>
       </c>
       <c r="F17" s="262">
         <f>'Detail Data'!F5</f>
-        <v>0</v>
+        <v>12603.5</v>
       </c>
       <c r="G17" s="262">
         <f>'Detail Data'!G5</f>
-        <v>0</v>
+        <v>12931.9</v>
       </c>
       <c r="H17" s="262"/>
       <c r="I17" s="262"/>
@@ -9075,17 +9213,17 @@
       <c r="B18" s="282" t="s">
         <v>145</v>
       </c>
-      <c r="E18" s="299" t="e">
+      <c r="E18" s="299">
         <f>E17/D17-1</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F18" s="299" t="e">
+        <v>5.1648050903990494E-2</v>
+      </c>
+      <c r="F18" s="299">
         <f t="shared" ref="F18:G18" si="1">F17/E17-1</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G18" s="299" t="e">
+        <v>2.4966453868987104E-2</v>
+      </c>
+      <c r="G18" s="299">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
+        <v>2.6056254215099051E-2</v>
       </c>
       <c r="H18" s="257"/>
       <c r="I18" s="257"/>
@@ -9103,15 +9241,15 @@
       </c>
       <c r="E19" s="262">
         <f>'Detail Data'!E21</f>
-        <v>0</v>
+        <v>3035.1</v>
       </c>
       <c r="F19" s="262">
         <f>'Detail Data'!F21</f>
-        <v>0</v>
+        <v>3393.8</v>
       </c>
       <c r="G19" s="262">
         <f>'Detail Data'!G21</f>
-        <v>0</v>
+        <v>3554.2</v>
       </c>
       <c r="H19" s="262"/>
       <c r="I19" s="262"/>
@@ -9121,21 +9259,21 @@
       <c r="B20" s="282" t="s">
         <v>146</v>
       </c>
-      <c r="D20" s="173" t="e">
+      <c r="D20" s="173">
         <f>D19/D17</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E20" s="173" t="e">
+        <v>0</v>
+      </c>
+      <c r="E20" s="173">
         <f t="shared" ref="E20:G20" si="2">E19/E17</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F20" s="173" t="e">
+        <v>0.2468263326962957</v>
+      </c>
+      <c r="F20" s="173">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G20" s="173" t="e">
+        <v>0.26927440790256674</v>
+      </c>
+      <c r="G20" s="173">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
+        <v>0.27483973739357714</v>
       </c>
       <c r="H20" s="257"/>
       <c r="I20" s="257"/>
@@ -9147,19 +9285,19 @@
       </c>
       <c r="D21" s="302">
         <f>'Detail Data'!D16</f>
-        <v>0</v>
-      </c>
-      <c r="E21" s="262" t="e">
+        <v>1441.5</v>
+      </c>
+      <c r="E21" s="262">
         <f>'Detail Data'!E16</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F21" s="262" t="e">
+        <v>2546.6904971403433</v>
+      </c>
+      <c r="F21" s="262">
         <f>'Detail Data'!F16</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G21" s="262" t="e">
+        <v>2835.4752529696439</v>
+      </c>
+      <c r="G21" s="262">
         <f>'Detail Data'!G16</f>
-        <v>#DIV/0!</v>
+        <v>2985.2383853937527</v>
       </c>
       <c r="H21" s="262"/>
       <c r="I21" s="262"/>
@@ -9169,21 +9307,21 @@
       <c r="B22" s="282" t="s">
         <v>146</v>
       </c>
-      <c r="D22" s="173" t="e">
+      <c r="D22" s="173">
         <f>D21/D17</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E22" s="173" t="e">
+        <v>0.12328310213297299</v>
+      </c>
+      <c r="E22" s="173">
         <f t="shared" ref="E22:G22" si="3">E21/E17</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F22" s="173" t="e">
+        <v>0.2071069407669128</v>
+      </c>
+      <c r="F22" s="173">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G22" s="173" t="e">
+        <v>0.22497522537149553</v>
+      </c>
+      <c r="G22" s="173">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
+        <v>0.23084298404671802</v>
       </c>
       <c r="H22" s="257"/>
       <c r="I22" s="257"/>
@@ -9204,21 +9342,21 @@
         <v>148</v>
       </c>
       <c r="C24" s="262"/>
-      <c r="D24" s="262" t="e">
+      <c r="D24" s="262">
         <f>D25*D21</f>
-        <v>#DIV/0!</v>
+        <v>540.01171742329893</v>
       </c>
       <c r="E24" s="262">
         <f>'Detail Data'!E20</f>
-        <v>0</v>
+        <v>597.70000000000005</v>
       </c>
       <c r="F24" s="262">
         <f>'Detail Data'!F20</f>
-        <v>0</v>
+        <v>689.8</v>
       </c>
       <c r="G24" s="262">
         <f>'Detail Data'!G20</f>
-        <v>0</v>
+        <v>707.8</v>
       </c>
       <c r="H24" s="262"/>
       <c r="I24" s="262"/>
@@ -9228,21 +9366,21 @@
       <c r="B25" s="282" t="s">
         <v>149</v>
       </c>
-      <c r="D25" s="331" t="e">
+      <c r="D25" s="331">
         <f>'Detail Data'!D20/'Detail Data'!D17</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E25" s="331" t="e">
+        <v>0.37461791010981543</v>
+      </c>
+      <c r="E25" s="331">
         <f>E24/E21</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F25" s="331" t="e">
+        <v>0.23469675670096238</v>
+      </c>
+      <c r="F25" s="331">
         <f t="shared" ref="F25:G25" si="4">F24/F21</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G25" s="331" t="e">
+        <v>0.24327491459414435</v>
+      </c>
+      <c r="G25" s="331">
         <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
+        <v>0.23709999290614148</v>
       </c>
       <c r="H25" s="331"/>
       <c r="I25" s="331"/>
@@ -9253,21 +9391,21 @@
         <v>150</v>
       </c>
       <c r="C26" s="178"/>
-      <c r="D26" s="253" t="e">
+      <c r="D26" s="253">
         <f t="shared" ref="D26:G26" si="5">D21-D24</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E26" s="253" t="e">
+        <v>901.48828257670107</v>
+      </c>
+      <c r="E26" s="253">
         <f>E21-E24</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F26" s="253" t="e">
+        <v>1948.9904971403432</v>
+      </c>
+      <c r="F26" s="253">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G26" s="253" t="e">
+        <v>2145.6752529696441</v>
+      </c>
+      <c r="G26" s="253">
         <f t="shared" si="5"/>
-        <v>#DIV/0!</v>
+        <v>2277.4383853937525</v>
       </c>
       <c r="H26" s="253"/>
       <c r="I26" s="253"/>
@@ -9289,19 +9427,19 @@
       </c>
       <c r="D28" s="262">
         <f>'Detail Data'!D38</f>
-        <v>0</v>
-      </c>
-      <c r="E28" s="262" t="e">
+        <v>503.7</v>
+      </c>
+      <c r="E28" s="262">
         <f>'Detail Data'!E38</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F28" s="262" t="e">
+        <v>488.40950285965675</v>
+      </c>
+      <c r="F28" s="262">
         <f>'Detail Data'!F38</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G28" s="262" t="e">
+        <v>558.32474703035621</v>
+      </c>
+      <c r="G28" s="262">
         <f>'Detail Data'!G38</f>
-        <v>#DIV/0!</v>
+        <v>568.96161460624717</v>
       </c>
       <c r="H28" s="262"/>
       <c r="I28" s="262"/>
@@ -9314,19 +9452,19 @@
       </c>
       <c r="D29" s="262">
         <f>C36-D36</f>
-        <v>0</v>
+        <v>-747</v>
       </c>
       <c r="E29" s="262">
         <f t="shared" ref="E29:G29" si="6">D36-E36</f>
-        <v>0</v>
+        <v>-284.5</v>
       </c>
       <c r="F29" s="262">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>-188</v>
       </c>
       <c r="G29" s="262">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>-296</v>
       </c>
       <c r="H29" s="262"/>
       <c r="I29" s="262"/>
@@ -9339,19 +9477,19 @@
       </c>
       <c r="D30" s="302">
         <f>-'Detail Data'!D40</f>
-        <v>0</v>
+        <v>-454.6</v>
       </c>
       <c r="E30" s="302">
         <f>-'Detail Data'!E40</f>
-        <v>0</v>
+        <v>-440.8</v>
       </c>
       <c r="F30" s="302">
         <f>-'Detail Data'!F40</f>
-        <v>0</v>
+        <v>-503.9</v>
       </c>
       <c r="G30" s="302">
         <f>-'Detail Data'!G40</f>
-        <v>0</v>
+        <v>-513.5</v>
       </c>
       <c r="H30" s="301"/>
       <c r="I30" s="301"/>
@@ -9362,21 +9500,21 @@
       <c r="B31" s="282" t="s">
         <v>154</v>
       </c>
-      <c r="D31" s="173" t="e">
+      <c r="D31" s="173">
         <f>FrontPage!I30</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E31" s="257" t="e">
+        <v>4.2660991037583057E-2</v>
+      </c>
+      <c r="E31" s="257">
         <f>D31</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F31" s="257" t="e">
+        <v>4.2660991037583057E-2</v>
+      </c>
+      <c r="F31" s="257">
         <f t="shared" ref="F31:G31" si="7">E31</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G31" s="257" t="e">
+        <v>4.2660991037583057E-2</v>
+      </c>
+      <c r="G31" s="257">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
+        <v>4.2660991037583057E-2</v>
       </c>
       <c r="H31" s="257"/>
       <c r="I31" s="257"/>
@@ -9433,23 +9571,23 @@
       </c>
       <c r="C36" s="302">
         <f>'Detail Data'!C33</f>
-        <v>0</v>
+        <v>-170</v>
       </c>
       <c r="D36" s="302">
         <f>'Detail Data'!D33</f>
-        <v>0</v>
+        <v>577</v>
       </c>
       <c r="E36" s="262">
         <f>'Detail Data'!E33</f>
-        <v>0</v>
+        <v>861.5</v>
       </c>
       <c r="F36" s="262">
         <f>'Detail Data'!F33</f>
-        <v>0</v>
+        <v>1049.5</v>
       </c>
       <c r="G36" s="262">
         <f>'Detail Data'!G33</f>
-        <v>0</v>
+        <v>1345.5</v>
       </c>
       <c r="H36" s="262"/>
       <c r="I36" s="262"/>
@@ -9459,21 +9597,21 @@
       <c r="B37" s="282" t="s">
         <v>154</v>
       </c>
-      <c r="D37" s="173" t="e">
+      <c r="D37" s="173">
         <f>D36/D17</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E37" s="173" t="e">
+        <v>4.934745052426321E-2</v>
+      </c>
+      <c r="E37" s="173">
         <f t="shared" ref="E37:G37" si="8">E36/E17</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F37" s="173" t="e">
+        <v>7.0060586345708123E-2</v>
+      </c>
+      <c r="F37" s="173">
         <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G37" s="173" t="e">
+        <v>8.3270520093624789E-2</v>
+      </c>
+      <c r="G37" s="173">
         <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
+        <v>0.10404503591892916</v>
       </c>
       <c r="H37" s="173"/>
       <c r="I37" s="173"/>
@@ -9494,7 +9632,7 @@
     <row r="39" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B39" s="242" t="str">
         <f>"Present value of UFCF on "&amp;TEXT(D9,"mmm dd, yyyy")&amp;" valuation date"</f>
-        <v>Present value of UFCF on Jan 00, 1900 valuation date</v>
+        <v>Present value of UFCF on Oct 04, 2026 valuation date</v>
       </c>
       <c r="D39" s="300"/>
       <c r="F39" s="300"/>
@@ -9528,7 +9666,7 @@
       <c r="C41" s="246"/>
       <c r="D41" s="247">
         <f>D9</f>
-        <v>0</v>
+        <v>46299</v>
       </c>
       <c r="E41" s="248">
         <f>DATE(YEAR($D$6)+1,12,31)</f>
@@ -9552,20 +9690,20 @@
       </c>
       <c r="C42" s="250">
         <f>D10</f>
-        <v>127.00277777777778</v>
+        <v>0.24166666666666667</v>
       </c>
       <c r="D42" s="179"/>
-      <c r="E42" s="262" t="e">
+      <c r="E42" s="262">
         <f>(E26+E28+E29+E30)*C42</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F42" s="262" t="e">
+        <v>413.75750000000005</v>
+      </c>
+      <c r="F42" s="262">
         <f>F26+F28+F29+F30</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G42" s="262" t="e">
+        <v>2012.1000000000004</v>
+      </c>
+      <c r="G42" s="262">
         <f t="shared" ref="G42" si="9">G26+G28+G29+G30</f>
-        <v>#DIV/0!</v>
+        <v>2036.8999999999996</v>
       </c>
       <c r="H42" s="262"/>
       <c r="I42" s="262"/>
@@ -9579,17 +9717,17 @@
         <v>164</v>
       </c>
       <c r="C43" s="252"/>
-      <c r="E43" s="253" t="e">
+      <c r="E43" s="253">
         <f>E42/(1+$H$6)^((E41-$D$41)/365)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F43" s="253" t="e">
+        <v>413.75750000000005</v>
+      </c>
+      <c r="F43" s="253">
         <f t="shared" ref="F43:G43" si="10">F42/(1+$H$6)^((F41-$D$41)/365)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G43" s="253" t="e">
+        <v>2012.1000000000004</v>
+      </c>
+      <c r="G43" s="253">
         <f t="shared" si="10"/>
-        <v>#DIV/0!</v>
+        <v>2036.8999999999996</v>
       </c>
       <c r="H43" s="253"/>
       <c r="I43" s="253"/>
@@ -9732,9 +9870,9 @@
       <c r="B55" s="267" t="s">
         <v>176</v>
       </c>
-      <c r="C55" s="272" t="e">
+      <c r="C55" s="272">
         <f>C48/G19</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="E55" s="162" t="s">
         <v>177</v>
@@ -9816,7 +9954,7 @@
       </c>
       <c r="C61" s="301">
         <f>'Detail Data'!D34</f>
-        <v>0</v>
+        <v>4681.2</v>
       </c>
       <c r="D61" s="364" t="s">
         <v>278</v>
@@ -9908,7 +10046,7 @@
       </c>
       <c r="C66" s="303">
         <f>'Detail Data'!D28</f>
-        <v>0</v>
+        <v>925.9</v>
       </c>
       <c r="G66" s="178"/>
       <c r="I66" s="300"/>
@@ -9947,7 +10085,7 @@
       </c>
       <c r="C69" s="321">
         <f>SUM(C61:C64)-SUM(C66:C67)</f>
-        <v>0</v>
+        <v>3755.2999999999997</v>
       </c>
       <c r="H69" s="250"/>
       <c r="I69" s="179"/>
@@ -10007,11 +10145,11 @@
       </c>
       <c r="C74" s="334">
         <f>C69</f>
-        <v>0</v>
+        <v>3755.2999999999997</v>
       </c>
       <c r="D74" s="334">
         <f>C74</f>
-        <v>0</v>
+        <v>3755.2999999999997</v>
       </c>
       <c r="G74" s="323"/>
       <c r="H74" s="179"/>
@@ -10024,11 +10162,11 @@
       </c>
       <c r="C75" s="275">
         <f>C73-C74</f>
-        <v>0</v>
+        <v>-3755.2999999999997</v>
       </c>
       <c r="D75" s="275">
         <f>D73-D74</f>
-        <v>0</v>
+        <v>-3755.2999999999997</v>
       </c>
       <c r="H75" s="179"/>
       <c r="J75" s="255"/>
@@ -10056,11 +10194,11 @@
       </c>
       <c r="C77" s="324">
         <f>C75/C76</f>
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="D77" s="324">
         <f>D75/D76</f>
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="H77" s="262"/>
       <c r="J77" s="255"/>
@@ -10095,13 +10233,13 @@
       <c r="B80" s="245" t="s">
         <v>208</v>
       </c>
-      <c r="C80" s="327" t="e">
+      <c r="C80" s="327">
         <f>C73/$E$17</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D80" s="327" t="e">
+        <v>0</v>
+      </c>
+      <c r="D80" s="327">
         <f>D73/$E$17</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="E80" s="326"/>
       <c r="F80" s="326"/>
@@ -10114,13 +10252,13 @@
       <c r="B81" s="245" t="s">
         <v>209</v>
       </c>
-      <c r="C81" s="326" t="e">
+      <c r="C81" s="326">
         <f>C73/$E$19</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D81" s="326" t="e">
+        <v>0</v>
+      </c>
+      <c r="D81" s="326">
         <f>D73/$E$19</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="E81" s="326"/>
       <c r="F81" s="326"/>
@@ -10134,13 +10272,13 @@
       <c r="B82" s="290" t="s">
         <v>210</v>
       </c>
-      <c r="C82" s="291" t="e">
+      <c r="C82" s="291">
         <f>C73/$E$21</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D82" s="291" t="e">
+        <v>0</v>
+      </c>
+      <c r="D82" s="291">
         <f>D73/$E$21</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="E82" s="291"/>
       <c r="F82" s="292"/>
@@ -10171,7 +10309,7 @@
     <row r="86" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B86" s="240" t="str">
         <f>"Present value of UFCF on "&amp;TEXT(D9,"mmm dd, yyyy")&amp;" valuation date"</f>
-        <v>Present value of UFCF on Jan 00, 1900 valuation date</v>
+        <v>Present value of UFCF on Oct 04, 2026 valuation date</v>
       </c>
       <c r="C86" s="176"/>
       <c r="D86" s="180"/>
@@ -10205,7 +10343,7 @@
       <c r="C88" s="246"/>
       <c r="D88" s="247">
         <f>D9</f>
-        <v>0</v>
+        <v>46299</v>
       </c>
       <c r="E88" s="248">
         <f>DATE(YEAR($D$6)+1,12,31)</f>
@@ -10228,20 +10366,20 @@
       </c>
       <c r="C89" s="250">
         <f>C42</f>
-        <v>127.00277777777778</v>
+        <v>0.24166666666666667</v>
       </c>
       <c r="D89" s="179"/>
       <c r="E89" s="182">
         <f>C89*'Detail Data'!D42</f>
         <v>0</v>
       </c>
-      <c r="F89" s="182" t="e">
+      <c r="F89" s="182">
         <f>'Detail Data'!E42</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G89" s="182" t="e">
+        <v>1724.6000000000004</v>
+      </c>
+      <c r="G89" s="182">
         <f>'Detail Data'!F42</f>
-        <v>#DIV/0!</v>
+        <v>1945.4000000000005</v>
       </c>
       <c r="H89" s="182"/>
       <c r="I89" s="251"/>
@@ -10255,13 +10393,13 @@
         <f>E89/(1+'WACC calculation'!$D$11)^((E88-$D$41)/365)</f>
         <v>0</v>
       </c>
-      <c r="F90" s="253" t="e">
+      <c r="F90" s="253">
         <f>F89/(1+'WACC calculation'!$D$11)^((F88-$D$41)/365)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G90" s="253" t="e">
+        <v>1724.6000000000004</v>
+      </c>
+      <c r="G90" s="253">
         <f>G89/(1+'WACC calculation'!$D$11)^((G88-$D$41)/365)</f>
-        <v>#DIV/0!</v>
+        <v>1945.4000000000005</v>
       </c>
       <c r="H90" s="253"/>
       <c r="I90" s="254"/>
@@ -10388,9 +10526,9 @@
       <c r="B102" s="267" t="s">
         <v>279</v>
       </c>
-      <c r="C102" s="272" t="e">
+      <c r="C102" s="272">
         <f>C95/(G21-G24)</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="E102" s="162" t="s">
         <v>177</v>
@@ -10552,7 +10690,7 @@
       <c r="C114" s="190"/>
       <c r="D114" s="191">
         <f>C77</f>
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="E114" s="192">
         <f t="shared" ref="E114" si="15">F114-0.005</f>
@@ -10574,9 +10712,9 @@
         <v>3.9999999999999994E-2</v>
       </c>
       <c r="J114" s="195"/>
-      <c r="L114" s="196" t="e">
+      <c r="L114" s="196">
         <f>C81</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="M114" s="192">
         <f t="shared" ref="M114" si="17">N114-0.005</f>
@@ -10606,40 +10744,40 @@
       </c>
       <c r="E115" s="198">
         <f t="dataTable" ref="E115:I119" dt2D="1" dtr="1" r1="C46" r2="H6"/>
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="F115" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="G115" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="H115" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="I115" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="J115" s="199"/>
       <c r="L115" s="197">
         <f t="shared" ref="L115" si="20">L116+0.005</f>
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="M115" s="200" t="e">
+      <c r="M115" s="200">
         <f t="dataTable" ref="M115:Q119" dt2D="1" dtr="1" r1="C46" r2="H6"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N115" s="200" t="e">
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O115" s="200" t="e">
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P115" s="200" t="e">
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q115" s="200" t="e">
-        <v>#DIV/0!</v>
+        <v>0</v>
+      </c>
+      <c r="N115" s="200">
+        <v>0</v>
+      </c>
+      <c r="O115" s="200">
+        <v>0</v>
+      </c>
+      <c r="P115" s="200">
+        <v>0</v>
+      </c>
+      <c r="Q115" s="200">
+        <v>0</v>
       </c>
     </row>
     <row r="116" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -10649,39 +10787,39 @@
         <v>6.5000000000000002E-2</v>
       </c>
       <c r="E116" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="F116" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="G116" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="H116" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="I116" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="J116" s="199"/>
       <c r="L116" s="197">
         <f>L117+0.005</f>
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="M116" s="200" t="e">
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N116" s="200" t="e">
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O116" s="200" t="e">
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P116" s="200" t="e">
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q116" s="200" t="e">
-        <v>#DIV/0!</v>
+      <c r="M116" s="200">
+        <v>0</v>
+      </c>
+      <c r="N116" s="200">
+        <v>0</v>
+      </c>
+      <c r="O116" s="200">
+        <v>0</v>
+      </c>
+      <c r="P116" s="200">
+        <v>0</v>
+      </c>
+      <c r="Q116" s="200">
+        <v>0</v>
       </c>
     </row>
     <row r="117" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -10693,19 +10831,19 @@
         <v>0.06</v>
       </c>
       <c r="E117" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="F117" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="G117" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="H117" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="I117" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="J117" s="199"/>
       <c r="K117" s="190" t="s">
@@ -10714,20 +10852,20 @@
       <c r="L117" s="201">
         <v>0.06</v>
       </c>
-      <c r="M117" s="200" t="e">
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N117" s="200" t="e">
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O117" s="200" t="e">
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P117" s="200" t="e">
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q117" s="200" t="e">
-        <v>#DIV/0!</v>
+      <c r="M117" s="200">
+        <v>0</v>
+      </c>
+      <c r="N117" s="200">
+        <v>0</v>
+      </c>
+      <c r="O117" s="200">
+        <v>0</v>
+      </c>
+      <c r="P117" s="200">
+        <v>0</v>
+      </c>
+      <c r="Q117" s="200">
+        <v>0</v>
       </c>
     </row>
     <row r="118" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -10737,39 +10875,39 @@
         <v>5.5E-2</v>
       </c>
       <c r="E118" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="F118" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="G118" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="H118" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="I118" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="J118" s="199"/>
       <c r="L118" s="197">
         <f>L117-0.005</f>
         <v>5.5E-2</v>
       </c>
-      <c r="M118" s="200" t="e">
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N118" s="200" t="e">
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O118" s="200" t="e">
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P118" s="200" t="e">
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q118" s="200" t="e">
-        <v>#DIV/0!</v>
+      <c r="M118" s="200">
+        <v>0</v>
+      </c>
+      <c r="N118" s="200">
+        <v>0</v>
+      </c>
+      <c r="O118" s="200">
+        <v>0</v>
+      </c>
+      <c r="P118" s="200">
+        <v>0</v>
+      </c>
+      <c r="Q118" s="200">
+        <v>0</v>
       </c>
     </row>
     <row r="119" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -10781,39 +10919,39 @@
         <v>0.05</v>
       </c>
       <c r="E119" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="F119" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="G119" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="H119" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="I119" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="J119" s="199"/>
       <c r="L119" s="203">
         <f>L118-0.005</f>
         <v>0.05</v>
       </c>
-      <c r="M119" s="200" t="e">
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N119" s="200" t="e">
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O119" s="200" t="e">
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P119" s="200" t="e">
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q119" s="200" t="e">
-        <v>#DIV/0!</v>
+      <c r="M119" s="200">
+        <v>0</v>
+      </c>
+      <c r="N119" s="200">
+        <v>0</v>
+      </c>
+      <c r="O119" s="200">
+        <v>0</v>
+      </c>
+      <c r="P119" s="200">
+        <v>0</v>
+      </c>
+      <c r="Q119" s="200">
+        <v>0</v>
       </c>
     </row>
     <row r="120" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -10869,7 +11007,7 @@
       <c r="B123" s="185"/>
       <c r="D123" s="206">
         <f>D77</f>
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="E123" s="207">
         <f t="shared" ref="E123" si="21">F123-0.5</f>
@@ -10923,19 +11061,19 @@
       </c>
       <c r="E124" s="198">
         <f t="dataTable" ref="E124:I128" dt2D="1" dtr="1" r1="I47" r2="H6"/>
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="F124" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="G124" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="H124" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="I124" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="J124" s="199"/>
       <c r="L124" s="197">
@@ -10966,19 +11104,19 @@
         <v>6.5000000000000002E-2</v>
       </c>
       <c r="E125" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="F125" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="G125" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="H125" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="I125" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="J125" s="199"/>
       <c r="L125" s="197">
@@ -11010,19 +11148,19 @@
         <v>0.06</v>
       </c>
       <c r="E126" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="F126" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="G126" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="H126" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="I126" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="J126" s="199"/>
       <c r="K126" s="190" t="s">
@@ -11054,19 +11192,19 @@
         <v>5.5E-2</v>
       </c>
       <c r="E127" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="F127" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="G127" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="H127" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="I127" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="J127" s="199"/>
       <c r="L127" s="197">
@@ -11096,19 +11234,19 @@
         <v>0.05</v>
       </c>
       <c r="E128" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="F128" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="G128" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="H128" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="I128" s="198">
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="J128" s="199"/>
       <c r="L128" s="203">
@@ -11251,7 +11389,7 @@
       </c>
       <c r="C152" s="220">
         <f>E126</f>
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="D152" s="220">
         <f>E152-C152</f>
@@ -11259,24 +11397,24 @@
       </c>
       <c r="E152" s="221">
         <f>I126</f>
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="G152" s="219" t="str">
         <f>"LTM EBITDA Purchase Multiple at "&amp;TEXT(M114,"0.0%")&amp;"-"&amp;TEXT(Q114,"0.0%")&amp;" Perpetuity Growth at "&amp;TEXT(L117,"0.0%")&amp;" WACC"</f>
         <v>LTM EBITDA Purchase Multiple at 2.0%-4.0% Perpetuity Growth at 6.0% WACC</v>
       </c>
       <c r="J152" s="210"/>
-      <c r="O152" s="222" t="e">
+      <c r="O152" s="222">
         <f>M117</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P152" s="222" t="e">
+        <v>0</v>
+      </c>
+      <c r="P152" s="222">
         <f>Q152-O152</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q152" s="223" t="e">
+        <v>0</v>
+      </c>
+      <c r="Q152" s="223">
         <f>Q117</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="153" spans="2:17" x14ac:dyDescent="0.2">
@@ -11286,7 +11424,7 @@
       </c>
       <c r="C153" s="220">
         <f>E117</f>
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="D153" s="220">
         <f>E153-C153</f>
@@ -11294,7 +11432,7 @@
       </c>
       <c r="E153" s="221">
         <f>I117</f>
-        <v>0</v>
+        <v>-1.8128026589484418E-2</v>
       </c>
       <c r="G153" s="224" t="e">
         <f>"LTM EBITDA Purchase Multiple at "&amp;TEXT(M126,"0.0x")&amp;"-"&amp;TEXT(Q126,"0.0x")&amp;" Exit EBITDA Multiple at "&amp;TEXT(L126,"0.0%")&amp;" WACC"</f>
@@ -11468,9 +11606,9 @@
         <f>'Detail Data'!D3</f>
         <v>0</v>
       </c>
-      <c r="D3" s="233" t="e">
+      <c r="D3" s="233">
         <f>C3/C5</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="E3" s="351"/>
     </row>
@@ -11480,11 +11618,11 @@
       </c>
       <c r="C4" s="347">
         <f>'Detail Data'!D34</f>
-        <v>0</v>
-      </c>
-      <c r="D4" s="233" t="e">
+        <v>4681.2</v>
+      </c>
+      <c r="D4" s="233">
         <f>C4/C5</f>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
       <c r="E4" s="351"/>
       <c r="G4" s="234"/>
@@ -11495,7 +11633,7 @@
       </c>
       <c r="C5" s="347">
         <f>C3+C4</f>
-        <v>0</v>
+        <v>4681.2</v>
       </c>
       <c r="F5" s="235"/>
       <c r="G5" s="234"/>
@@ -11556,9 +11694,9 @@
       <c r="C16" s="232" t="s">
         <v>233</v>
       </c>
-      <c r="D16" s="236" t="e">
+      <c r="D16" s="236">
         <f>D3*D11+D4*D13*(1-D14)</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Workbook: diluted shares and EPS from the 10-K EPS note, actual EBITDA, FrontPage inputs and text boxes; verification form regenerated with the added rows
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/workbook/QD-HSY.xlsx
+++ b/workbook/QD-HSY.xlsx
@@ -256,7 +256,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="300">
   <si>
     <t>Share Symbol:</t>
   </si>
@@ -357,9 +357,6 @@
     <t>Net Debt - M $$</t>
   </si>
   <si>
-    <t>1)                                                                                                                  2)                                                                                                                  3)</t>
-  </si>
-  <si>
     <t>Avg EBITDA Margin (%)</t>
   </si>
   <si>
@@ -399,9 +396,6 @@
     <t>P/E (Fwd 24 Months)</t>
   </si>
   <si>
-    <t xml:space="preserve">1)                                                                                                                  2) </t>
-  </si>
-  <si>
     <t>EPS Growth (LTM)</t>
   </si>
   <si>
@@ -444,18 +438,6 @@
     <t>Mult = (MC + Debt - Cash) / EBITDA</t>
   </si>
   <si>
-    <t>Key Components of Company Unit Economics:
-Unit: Cost/Revenue per customer, per VM, per API call, or AI workload.
-Leverage: Economies of scale from massive data centers, efficient resource utilization, and hybrid cloud consistency.
-Focus: Driving high growth through AI services and infrastructure.
-Productivity &amp; Business Processes:
-Unit: Revenue/Cost per seat, per subscriber, per user.
-Leverage: High-margin subscription models (SaaS) with recurring revenue, increasing revenue per user.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) </t>
-  </si>
-  <si>
     <t>ROE</t>
   </si>
   <si>
@@ -465,9 +447,6 @@
     <t>Mult = ((Pr * SH)+ Debt - Cash) / EBITDA</t>
   </si>
   <si>
-    <t xml:space="preserve">2) </t>
-  </si>
-  <si>
     <t>Avg ROE (3 Yrs)</t>
   </si>
   <si>
@@ -477,9 +456,6 @@
     <t>((Mult*EBITDA)+Cash-Debt)/Sh</t>
   </si>
   <si>
-    <t xml:space="preserve">3) </t>
-  </si>
-  <si>
     <t>Asset Turnover</t>
   </si>
   <si>
@@ -504,21 +480,9 @@
     <t>Pr = ((Mult * FCF)+Cash-Debt) / Sh</t>
   </si>
   <si>
-    <t>1)</t>
-  </si>
-  <si>
-    <t>3)</t>
-  </si>
-  <si>
     <t>Avg Fincl Lev (3 Yrs)</t>
   </si>
   <si>
-    <t>2)</t>
-  </si>
-  <si>
-    <t>4)</t>
-  </si>
-  <si>
     <t>Share Price (USD) - 5 yrs</t>
   </si>
   <si>
@@ -1053,9 +1017,6 @@
     <t>b using FCFE</t>
   </si>
   <si>
-    <t>3QFY26</t>
-  </si>
-  <si>
     <t>Interest Coverage</t>
   </si>
   <si>
@@ -1132,6 +1093,71 @@
   </si>
   <si>
     <t>Relative Valuation</t>
+  </si>
+  <si>
+    <t>The Hershey Company (HSY)</t>
+  </si>
+  <si>
+    <t>HSY</t>
+  </si>
+  <si>
+    <t>NYSE</t>
+  </si>
+  <si>
+    <t>Chris Lester</t>
+  </si>
+  <si>
+    <t>2QFY26</t>
+  </si>
+  <si>
+    <t>wjs65@txstate.edu</t>
+  </si>
+  <si>
+    <t>Founded in 1894, Hershey is the largest producer of quality chocolate in North America and a leading U.S. snack maker. Brands include Hershey's, Reese's, Kisses, Jolly Rancher and Kit Kat (U.S.) and salty snacks (SkinnyPop, Dot's Homestyle Pretzels). FY2025 net sales were $11.69 billion; about 19,600 employees. Source: FY2025 Form 10-K (S1).</t>
+  </si>
+  <si>
+    <t>1) Q3 2026 results, expected Oct 22, 2026: management expects the year's strongest earnings growth as peak cocoa costs are lapped (S3).  2) Cocoa is down more than 70% from late-2024 highs; the relief reaches margins with a lag through hedges and inventory (S6).  3) FY2026 guidance raised in July: net sales growth of 4.5 to 5.0% and adjusted EPS of $8.36 to $8.52 (S2).</t>
+  </si>
+  <si>
+    <t>FY2025 net sales (S1): North America Confectionery $9,479.7M (81%); North America Salty Snacks $1,271.3M (11%); International $941.6M (8%).</t>
+  </si>
+  <si>
+    <t>1) Brands with pricing power: Hershey's, Reese's and Kisses carried roughly 14% price increases in 2026 and net sales still grew (S3, S4).  2) Scale: the largest producer of quality chocolate in North America, with the manufacturing and retail distribution that come with it (S1).</t>
+  </si>
+  <si>
+    <t>Hershey sells branded chocolate, sweets and snacks to retailers and distributors. Revenue is volume times net price, and price is the lever: Q2 2026 net sales rose 6.6% on roughly 14% pricing while confectionery volume fell about 10% (S3, S4).
+The swing cost is cocoa, then sugar, dairy and packaging: gross margin fell from 47.3% in FY2024 to 33.5% in FY2025 as cocoa peaked (S1).
+Reinvestment is light: capex was 3.9% of sales in FY2025, below D&amp;A, so operating profit converts to cash ($2.28B operating cash flow) and is returned as dividends ($1.09B) (S1).</t>
+  </si>
+  <si>
+    <t>1) Cash generation: $2.28B of operating cash flow in FY2025, a trough-margin year (S1).</t>
+  </si>
+  <si>
+    <t>2) Low capital intensity: capex 3.9% of sales, below D&amp;A (S1).</t>
+  </si>
+  <si>
+    <t>3) Pricing power: Q2 2026 net sales up 6.6% on about 14% pricing (S3, S4).</t>
+  </si>
+  <si>
+    <t>1) Volume: confectionery volume fell about 10% in Q2 2026 as prices rose (S4).</t>
+  </si>
+  <si>
+    <t>1) Mondelez (MDLZ)</t>
+  </si>
+  <si>
+    <t>3) Lindt &amp; Spruengli (LISN)</t>
+  </si>
+  <si>
+    <t>2) Cocoa: one input took operating margin from 25.9% to 12.3% in a year (S1, S6).</t>
+  </si>
+  <si>
+    <t>2) Nestle (NESN)</t>
+  </si>
+  <si>
+    <t>4) General Mills (GIS)</t>
+  </si>
+  <si>
+    <t>3) Concentration: North America Confectionery is 81% of net sales (S1).</t>
   </si>
 </sst>
 </file>
@@ -2868,6 +2894,48 @@
     <xf numFmtId="194" fontId="46" fillId="13" borderId="12" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="185" fontId="46" fillId="13" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="18" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2882,48 +2950,6 @@
     </xf>
     <xf numFmtId="165" fontId="13" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -6509,65 +6535,75 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="379"/>
-      <c r="B1" s="379"/>
-      <c r="C1" s="379"/>
-      <c r="D1" s="379"/>
-      <c r="E1" s="379"/>
-      <c r="F1" s="379"/>
-      <c r="G1" s="379"/>
-      <c r="H1" s="380"/>
-      <c r="I1" s="380"/>
-      <c r="J1" s="380"/>
-      <c r="K1" s="380"/>
-      <c r="L1" s="380"/>
-      <c r="M1" s="380"/>
+      <c r="A1" s="393" t="s">
+        <v>279</v>
+      </c>
+      <c r="B1" s="393"/>
+      <c r="C1" s="393"/>
+      <c r="D1" s="393"/>
+      <c r="E1" s="393"/>
+      <c r="F1" s="393"/>
+      <c r="G1" s="393"/>
+      <c r="H1" s="394"/>
+      <c r="I1" s="394"/>
+      <c r="J1" s="394"/>
+      <c r="K1" s="394"/>
+      <c r="L1" s="394"/>
+      <c r="M1" s="394"/>
     </row>
     <row r="2" spans="1:18" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="3"/>
-      <c r="C2" s="4"/>
+      <c r="C2" s="4" t="s">
+        <v>280</v>
+      </c>
       <c r="D2" s="5"/>
       <c r="E2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="381"/>
-      <c r="G2" s="381"/>
-      <c r="H2" s="382" t="s">
+      <c r="F2" s="395" t="s">
+        <v>281</v>
+      </c>
+      <c r="G2" s="395"/>
+      <c r="H2" s="396" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="382"/>
-      <c r="J2" s="382"/>
-      <c r="K2" s="382"/>
-      <c r="L2" s="382"/>
-      <c r="M2" s="382"/>
+      <c r="I2" s="396"/>
+      <c r="J2" s="396"/>
+      <c r="K2" s="396"/>
+      <c r="L2" s="396"/>
+      <c r="M2" s="396"/>
     </row>
     <row r="3" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="8"/>
-      <c r="C3" s="9"/>
+      <c r="C3" s="9">
+        <v>159.46</v>
+      </c>
       <c r="D3" s="10"/>
       <c r="E3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="383"/>
-      <c r="G3" s="383"/>
+      <c r="F3" s="397" t="s">
+        <v>282</v>
+      </c>
+      <c r="G3" s="397"/>
       <c r="H3" s="11" t="s">
         <v>5</v>
       </c>
       <c r="I3" s="12" t="s">
-        <v>263</v>
+        <v>283</v>
       </c>
       <c r="K3" s="11" t="s">
         <v>6</v>
       </c>
       <c r="M3" s="13">
         <f>C3*'Detail Data'!E9</f>
-        <v>0</v>
+        <v>32434.164000000004</v>
       </c>
     </row>
     <row r="4" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -6582,8 +6618,10 @@
       <c r="E4" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="384"/>
-      <c r="G4" s="384"/>
+      <c r="F4" s="392" t="s">
+        <v>284</v>
+      </c>
+      <c r="G4" s="392"/>
       <c r="H4" s="19" t="s">
         <v>9</v>
       </c>
@@ -6596,7 +6634,7 @@
       <c r="L4" s="22"/>
       <c r="M4" s="23">
         <f>M3+'Detail Data'!E34-'Detail Data'!E28</f>
-        <v>3242.2</v>
+        <v>35676.364000000001</v>
       </c>
     </row>
     <row r="5" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -6615,15 +6653,15 @@
       <c r="G5" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="H5" s="385" t="s">
+      <c r="H5" s="380" t="s">
         <v>15</v>
       </c>
-      <c r="I5" s="385"/>
-      <c r="K5" s="386" t="s">
+      <c r="I5" s="380"/>
+      <c r="K5" s="390" t="s">
         <v>16</v>
       </c>
-      <c r="L5" s="386"/>
-      <c r="M5" s="386"/>
+      <c r="L5" s="390"/>
+      <c r="M5" s="390"/>
     </row>
     <row r="6" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="30" t="s">
@@ -6631,7 +6669,7 @@
       </c>
       <c r="B6" s="31"/>
       <c r="C6" s="32">
-        <v>6040.53</v>
+        <v>6715.35</v>
       </c>
       <c r="D6" s="17"/>
       <c r="E6" s="33"/>
@@ -6659,19 +6697,19 @@
       </c>
       <c r="B7" s="31"/>
       <c r="C7" s="39">
-        <v>7656.98</v>
+        <v>7722.72</v>
       </c>
       <c r="D7" s="17"/>
       <c r="E7" s="40">
         <f>C7/C6-1</f>
-        <v>0.26760069066787184</v>
+        <v>0.15001005159820413</v>
       </c>
       <c r="F7" s="41">
         <v>358.17</v>
       </c>
       <c r="G7" s="42">
         <f>C7/F7</f>
-        <v>21.378060697434176</v>
+        <v>21.561604824524668</v>
       </c>
       <c r="H7" s="35" t="s">
         <v>21</v>
@@ -6684,9 +6722,9 @@
         <v>22</v>
       </c>
       <c r="L7" s="37"/>
-      <c r="M7" s="43" t="e">
+      <c r="M7" s="43">
         <f>M6/'Detail Data'!E9</f>
-        <v>#DIV/0!</v>
+        <v>7.1361848574237952</v>
       </c>
     </row>
     <row r="8" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -6754,23 +6792,23 @@
         <v>28</v>
       </c>
       <c r="L9" s="37"/>
-      <c r="M9" s="43" t="e">
+      <c r="M9" s="43">
         <f>M8/'Detail Data'!E9</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="387" t="s">
+      <c r="A10" s="389" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="387"/>
-      <c r="C10" s="387"/>
+      <c r="B10" s="389"/>
+      <c r="C10" s="389"/>
       <c r="D10" s="17"/>
-      <c r="E10" s="385" t="s">
+      <c r="E10" s="380" t="s">
         <v>30</v>
       </c>
-      <c r="F10" s="385"/>
-      <c r="G10" s="385"/>
+      <c r="F10" s="380"/>
+      <c r="G10" s="380"/>
       <c r="H10" s="35" t="s">
         <v>31</v>
       </c>
@@ -6788,24 +6826,26 @@
       </c>
     </row>
     <row r="11" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="388"/>
-      <c r="B11" s="388"/>
-      <c r="C11" s="388"/>
+      <c r="A11" s="385" t="s">
+        <v>285</v>
+      </c>
+      <c r="B11" s="385"/>
+      <c r="C11" s="385"/>
       <c r="D11" s="17"/>
-      <c r="E11" s="389" t="s">
+      <c r="E11" s="391" t="s">
+        <v>286</v>
+      </c>
+      <c r="F11" s="391"/>
+      <c r="G11" s="391"/>
+      <c r="H11" s="51" t="s">
         <v>33</v>
-      </c>
-      <c r="F11" s="389"/>
-      <c r="G11" s="389"/>
-      <c r="H11" s="51" t="s">
-        <v>34</v>
       </c>
       <c r="I11" s="52">
         <f>AVERAGE('Detail Data'!C26,'Detail Data'!D26,'Detail Data'!E26)</f>
-        <v>8.2275444232098566E-2</v>
+        <v>0.23751537688279645</v>
       </c>
       <c r="K11" s="51" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="L11" s="53"/>
       <c r="M11" s="54" t="e">
@@ -6814,142 +6854,144 @@
       </c>
     </row>
     <row r="12" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="388"/>
-      <c r="B12" s="388"/>
-      <c r="C12" s="388"/>
+      <c r="A12" s="385"/>
+      <c r="B12" s="385"/>
+      <c r="C12" s="385"/>
       <c r="D12" s="17"/>
-      <c r="E12" s="389"/>
-      <c r="F12" s="389"/>
-      <c r="G12" s="389"/>
-      <c r="H12" s="385" t="s">
+      <c r="E12" s="391"/>
+      <c r="F12" s="391"/>
+      <c r="G12" s="391"/>
+      <c r="H12" s="380" t="s">
+        <v>35</v>
+      </c>
+      <c r="I12" s="380"/>
+      <c r="K12" s="55" t="s">
         <v>36</v>
-      </c>
-      <c r="I12" s="385"/>
-      <c r="K12" s="55" t="s">
-        <v>37</v>
       </c>
       <c r="L12" s="56" t="s">
         <v>14</v>
       </c>
       <c r="M12" s="57" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="385"/>
+      <c r="B13" s="385"/>
+      <c r="C13" s="385"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="391"/>
+      <c r="F13" s="391"/>
+      <c r="G13" s="391"/>
+      <c r="H13" s="58" t="s">
         <v>38</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="388"/>
-      <c r="B13" s="388"/>
-      <c r="C13" s="388"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="389"/>
-      <c r="F13" s="389"/>
-      <c r="G13" s="389"/>
-      <c r="H13" s="58" t="s">
-        <v>39</v>
       </c>
       <c r="I13" s="59">
         <f>('Detail Data'!E5/'Detail Data'!D5)-1</f>
         <v>5.1648050903990494E-2</v>
       </c>
       <c r="K13" s="60" t="s">
+        <v>39</v>
+      </c>
+      <c r="L13" s="61">
+        <f>'Detail Data'!E12</f>
+        <v>2.6376744602122559</v>
+      </c>
+      <c r="M13" s="62">
+        <f>L13*'Detail Data'!E7</f>
+        <v>159.46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="385"/>
+      <c r="B14" s="385"/>
+      <c r="C14" s="385"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="391"/>
+      <c r="F14" s="391"/>
+      <c r="G14" s="391"/>
+      <c r="H14" s="58" t="s">
         <v>40</v>
-      </c>
-      <c r="L13" s="61" t="e">
-        <f>'Detail Data'!E12</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M13" s="62" t="e">
-        <f>L13*'Detail Data'!E7</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="14" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="388"/>
-      <c r="B14" s="388"/>
-      <c r="C14" s="388"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="389"/>
-      <c r="F14" s="389"/>
-      <c r="G14" s="389"/>
-      <c r="H14" s="58" t="s">
-        <v>41</v>
       </c>
       <c r="I14" s="59">
         <f>'Detail Data'!F5/'Detail Data'!E5-1</f>
         <v>2.4966453868987104E-2</v>
       </c>
       <c r="K14" s="58" t="s">
+        <v>41</v>
+      </c>
+      <c r="L14" s="63">
+        <f>'Detail Data'!F12</f>
+        <v>2.5734251596778672</v>
+      </c>
+      <c r="M14" s="64">
+        <f>L13*'Detail Data'!F7</f>
+        <v>163.44115073394872</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="380" t="s">
         <v>42</v>
       </c>
-      <c r="L14" s="63" t="e">
-        <f>'Detail Data'!F12</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M14" s="64" t="e">
-        <f>L13*'Detail Data'!F7</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="385" t="s">
+      <c r="B15" s="380"/>
+      <c r="C15" s="380"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="380" t="s">
         <v>43</v>
       </c>
-      <c r="B15" s="385"/>
-      <c r="C15" s="385"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="385" t="s">
+      <c r="F15" s="380"/>
+      <c r="G15" s="380"/>
+      <c r="H15" s="58" t="s">
         <v>44</v>
-      </c>
-      <c r="F15" s="385"/>
-      <c r="G15" s="385"/>
-      <c r="H15" s="58" t="s">
-        <v>45</v>
       </c>
       <c r="I15" s="59">
         <f>(('Detail Data'!G5/'Detail Data'!E5)^(1/2))-1</f>
         <v>2.551120927708328E-2</v>
       </c>
       <c r="K15" s="65" t="s">
+        <v>45</v>
+      </c>
+      <c r="L15" s="66">
+        <f>'Detail Data'!G12</f>
+        <v>2.5080741422374131</v>
+      </c>
+      <c r="M15" s="67">
+        <f>L13*'Detail Data'!G7</f>
+        <v>167.69981490668079</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="388" t="s">
+        <v>287</v>
+      </c>
+      <c r="B16" s="388"/>
+      <c r="C16" s="388"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="386" t="s">
+        <v>288</v>
+      </c>
+      <c r="F16" s="386"/>
+      <c r="G16" s="386"/>
+      <c r="H16" s="58" t="s">
         <v>46</v>
       </c>
-      <c r="L15" s="66" t="e">
-        <f>'Detail Data'!G12</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M15" s="67" t="e">
-        <f>L13*'Detail Data'!G7</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="390"/>
-      <c r="B16" s="390"/>
-      <c r="C16" s="390"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="391" t="s">
+      <c r="I16" s="59">
+        <f>'Detail Data'!E7/'Detail Data'!D7-1</f>
+        <v>12.929670259958584</v>
+      </c>
+      <c r="K16" s="60" t="s">
         <v>47</v>
-      </c>
-      <c r="F16" s="391"/>
-      <c r="G16" s="391"/>
-      <c r="H16" s="58" t="s">
-        <v>48</v>
-      </c>
-      <c r="I16" s="59" t="e">
-        <f>'Detail Data'!E7/'Detail Data'!D7-1</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K16" s="60" t="s">
-        <v>49</v>
       </c>
       <c r="L16" s="68">
         <f>'Detail Data'!E11</f>
-        <v>0</v>
-      </c>
-      <c r="M16" s="62" t="e">
+        <v>2.6376744602122559</v>
+      </c>
+      <c r="M16" s="62">
         <f>('Detail Data'!E11*'Detail Data'!E5)/'Detail Data'!E9</f>
-        <v>#DIV/0!</v>
+        <v>159.46</v>
       </c>
       <c r="N16" s="69" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="O16" s="70"/>
       <c r="P16" s="70"/>
@@ -6957,33 +6999,33 @@
       <c r="R16" s="72"/>
     </row>
     <row r="17" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="390"/>
-      <c r="B17" s="390"/>
-      <c r="C17" s="390"/>
+      <c r="A17" s="388"/>
+      <c r="B17" s="388"/>
+      <c r="C17" s="388"/>
       <c r="D17" s="17"/>
-      <c r="E17" s="391"/>
-      <c r="F17" s="391"/>
-      <c r="G17" s="391"/>
+      <c r="E17" s="386"/>
+      <c r="F17" s="386"/>
+      <c r="G17" s="386"/>
       <c r="H17" s="58" t="s">
-        <v>51</v>
-      </c>
-      <c r="I17" s="59" t="e">
+        <v>49</v>
+      </c>
+      <c r="I17" s="59">
         <f>'Detail Data'!F7/'Detail Data'!E7-1</f>
-        <v>#DIV/0!</v>
+        <v>2.4966453868987104E-2</v>
       </c>
       <c r="K17" s="58" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="L17" s="63">
         <f>'Detail Data'!F11</f>
-        <v>0</v>
-      </c>
-      <c r="M17" s="64" t="e">
+        <v>2.5734251596778677</v>
+      </c>
+      <c r="M17" s="64">
         <f>('Detail Data'!E11*'Detail Data'!F5)/'Detail Data'!F9</f>
-        <v>#DIV/0!</v>
+        <v>163.44115073394869</v>
       </c>
       <c r="N17" s="73" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="O17" s="72"/>
       <c r="P17" s="72"/>
@@ -6991,33 +7033,33 @@
       <c r="R17" s="72"/>
     </row>
     <row r="18" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="390"/>
-      <c r="B18" s="390"/>
-      <c r="C18" s="390"/>
+      <c r="A18" s="388"/>
+      <c r="B18" s="388"/>
+      <c r="C18" s="388"/>
       <c r="D18" s="17"/>
-      <c r="E18" s="391"/>
-      <c r="F18" s="391"/>
-      <c r="G18" s="391"/>
+      <c r="E18" s="386"/>
+      <c r="F18" s="386"/>
+      <c r="G18" s="386"/>
       <c r="H18" s="65" t="s">
-        <v>54</v>
-      </c>
-      <c r="I18" s="54" t="e">
+        <v>52</v>
+      </c>
+      <c r="I18" s="54">
         <f>(('Detail Data'!G7/'Detail Data'!E7)^(1/2))-1</f>
-        <v>#DIV/0!</v>
+        <v>2.551120927708328E-2</v>
       </c>
       <c r="K18" s="65" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L18" s="66">
         <f>'Detail Data'!G11</f>
-        <v>0</v>
-      </c>
-      <c r="M18" s="67" t="e">
+        <v>2.5080741422374131</v>
+      </c>
+      <c r="M18" s="67">
         <f>('Detail Data'!E11*'Detail Data'!G5)/'Detail Data'!G9</f>
-        <v>#DIV/0!</v>
+        <v>167.69981490668076</v>
       </c>
       <c r="N18" s="69" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="O18" s="70"/>
       <c r="P18" s="70"/>
@@ -7025,34 +7067,34 @@
       <c r="R18" s="71"/>
     </row>
     <row r="19" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="387" t="s">
+      <c r="A19" s="389" t="s">
+        <v>55</v>
+      </c>
+      <c r="B19" s="389"/>
+      <c r="C19" s="389"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="390" t="s">
+        <v>56</v>
+      </c>
+      <c r="F19" s="390"/>
+      <c r="G19" s="390"/>
+      <c r="H19" s="380" t="s">
         <v>57</v>
       </c>
-      <c r="B19" s="387"/>
-      <c r="C19" s="387"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="386" t="s">
+      <c r="I19" s="380"/>
+      <c r="K19" s="60" t="s">
         <v>58</v>
-      </c>
-      <c r="F19" s="386"/>
-      <c r="G19" s="386"/>
-      <c r="H19" s="385" t="s">
-        <v>59</v>
-      </c>
-      <c r="I19" s="385"/>
-      <c r="K19" s="60" t="s">
-        <v>60</v>
       </c>
       <c r="L19" s="68">
         <f>'Detail Data'!E13</f>
-        <v>0.81035221244769529</v>
-      </c>
-      <c r="M19" s="62" t="e">
+        <v>11.501963691476393</v>
+      </c>
+      <c r="M19" s="62">
         <f>(('Detail Data'!E13*'Detail Data'!E21)-'Detail Data'!E34+'Detail Data'!E28)/'Detail Data'!E9</f>
-        <v>#DIV/0!</v>
+        <v>155.69031465093411</v>
       </c>
       <c r="N19" s="73" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="O19" s="72"/>
       <c r="P19" s="72"/>
@@ -7060,37 +7102,37 @@
       <c r="R19" s="74"/>
     </row>
     <row r="20" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="388" t="s">
-        <v>62</v>
-      </c>
-      <c r="B20" s="388"/>
-      <c r="C20" s="388"/>
+      <c r="A20" s="385" t="s">
+        <v>289</v>
+      </c>
+      <c r="B20" s="385"/>
+      <c r="C20" s="385"/>
       <c r="D20" s="17"/>
-      <c r="E20" s="392" t="s">
-        <v>63</v>
-      </c>
-      <c r="F20" s="392"/>
-      <c r="G20" s="392"/>
+      <c r="E20" s="381" t="s">
+        <v>290</v>
+      </c>
+      <c r="F20" s="381"/>
+      <c r="G20" s="381"/>
       <c r="H20" s="60" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I20" s="75">
         <f>'Detail Data'!E35/AVERAGE('Detail Data'!E30,'Detail Data'!D30)</f>
         <v>0.34483455126494161</v>
       </c>
       <c r="K20" s="58" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="L20" s="63">
         <f>'Detail Data'!F13</f>
-        <v>0.7247038717661618</v>
-      </c>
-      <c r="M20" s="64" t="e">
+        <v>10.286289704755731</v>
+      </c>
+      <c r="M20" s="64">
         <f>(('Detail Data'!E13*'Detail Data'!F21)+'Detail Data'!F28-'Detail Data'!F34)/'Detail Data'!F9</f>
-        <v>#DIV/0!</v>
+        <v>177.20680617567641</v>
       </c>
       <c r="N20" s="73" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="O20" s="72"/>
       <c r="P20" s="72"/>
@@ -7098,35 +7140,35 @@
       <c r="R20" s="74"/>
     </row>
     <row r="21" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="388"/>
-      <c r="B21" s="388"/>
-      <c r="C21" s="388"/>
+      <c r="A21" s="385"/>
+      <c r="B21" s="385"/>
+      <c r="C21" s="385"/>
       <c r="D21" s="17"/>
-      <c r="E21" s="393" t="s">
-        <v>67</v>
-      </c>
-      <c r="F21" s="393"/>
-      <c r="G21" s="393"/>
+      <c r="E21" s="383" t="s">
+        <v>291</v>
+      </c>
+      <c r="F21" s="383"/>
+      <c r="G21" s="383"/>
       <c r="H21" s="58" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="I21" s="59">
         <f>'Detail Data'!E17/AVERAGE('Detail Data'!C35,'Detail Data'!D35,'Detail Data'!E35)</f>
         <v>0.36311979450455362</v>
       </c>
       <c r="K21" s="65" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="L21" s="66">
         <f>'Detail Data'!G13</f>
-        <v>0.69199819931348827</v>
-      </c>
-      <c r="M21" s="67" t="e">
+        <v>9.8220724776320978</v>
+      </c>
+      <c r="M21" s="67">
         <f>(('Detail Data'!E13*'Detail Data'!G21)+'Detail Data'!G28-'Detail Data'!G34)/'Detail Data'!G9</f>
-        <v>#DIV/0!</v>
+        <v>187.95220920474625</v>
       </c>
       <c r="N21" s="76" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="O21" s="77"/>
       <c r="P21" s="77"/>
@@ -7134,17 +7176,17 @@
       <c r="R21" s="78"/>
     </row>
     <row r="22" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="388"/>
-      <c r="B22" s="388"/>
-      <c r="C22" s="388"/>
+      <c r="A22" s="385"/>
+      <c r="B22" s="385"/>
+      <c r="C22" s="385"/>
       <c r="D22" s="17"/>
-      <c r="E22" s="391" t="s">
-        <v>71</v>
-      </c>
-      <c r="F22" s="391"/>
-      <c r="G22" s="391"/>
+      <c r="E22" s="386" t="s">
+        <v>292</v>
+      </c>
+      <c r="F22" s="386"/>
+      <c r="G22" s="386"/>
       <c r="H22" s="58" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="I22" s="59">
         <f>'Detail Data'!E40/AVERAGE('Detail Data'!E30,'Detail Data'!D30,'Detail Data'!C30)</f>
@@ -7154,7 +7196,7 @@
       <c r="L22" s="68"/>
       <c r="M22" s="62"/>
       <c r="N22" s="69" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="O22" s="70"/>
       <c r="P22" s="70"/>
@@ -7162,17 +7204,17 @@
       <c r="R22" s="71"/>
     </row>
     <row r="23" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="388"/>
-      <c r="B23" s="388"/>
-      <c r="C23" s="388"/>
+      <c r="A23" s="385"/>
+      <c r="B23" s="385"/>
+      <c r="C23" s="385"/>
       <c r="D23" s="17"/>
-      <c r="E23" s="394" t="s">
-        <v>74</v>
-      </c>
-      <c r="F23" s="394"/>
-      <c r="G23" s="394"/>
+      <c r="E23" s="387" t="s">
+        <v>68</v>
+      </c>
+      <c r="F23" s="387"/>
+      <c r="G23" s="387"/>
       <c r="H23" s="58" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="I23" s="59">
         <f>'Detail Data'!E17/'Detail Data'!E35</f>
@@ -7182,7 +7224,7 @@
       <c r="L23" s="63"/>
       <c r="M23" s="64"/>
       <c r="N23" s="73" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="O23" s="72"/>
       <c r="P23" s="72"/>
@@ -7190,19 +7232,19 @@
       <c r="R23" s="74"/>
     </row>
     <row r="24" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="385" t="s">
-        <v>77</v>
-      </c>
-      <c r="B24" s="385"/>
-      <c r="C24" s="385"/>
+      <c r="A24" s="380" t="s">
+        <v>71</v>
+      </c>
+      <c r="B24" s="380"/>
+      <c r="C24" s="380"/>
       <c r="D24" s="17"/>
-      <c r="E24" s="392" t="s">
-        <v>63</v>
-      </c>
-      <c r="F24" s="392"/>
-      <c r="G24" s="392"/>
+      <c r="E24" s="381" t="s">
+        <v>293</v>
+      </c>
+      <c r="F24" s="381"/>
+      <c r="G24" s="381"/>
       <c r="H24" s="58" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="I24" s="59">
         <f>AVERAGE('Detail Data'!D30,'Detail Data'!E30)/AVERAGE('Detail Data'!D35,'Detail Data'!E35)</f>
@@ -7212,7 +7254,7 @@
       <c r="L24" s="66"/>
       <c r="M24" s="67"/>
       <c r="N24" s="76" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="O24" s="77"/>
       <c r="P24" s="77"/>
@@ -7221,20 +7263,20 @@
     </row>
     <row r="25" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="79" t="s">
-        <v>80</v>
-      </c>
-      <c r="B25" s="396" t="s">
-        <v>81</v>
-      </c>
-      <c r="C25" s="396"/>
+        <v>294</v>
+      </c>
+      <c r="B25" s="382" t="s">
+        <v>295</v>
+      </c>
+      <c r="C25" s="382"/>
       <c r="D25" s="17"/>
-      <c r="E25" s="393" t="s">
-        <v>67</v>
-      </c>
-      <c r="F25" s="393"/>
-      <c r="G25" s="393"/>
+      <c r="E25" s="383" t="s">
+        <v>296</v>
+      </c>
+      <c r="F25" s="383"/>
+      <c r="G25" s="383"/>
       <c r="H25" s="58" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="I25" s="59">
         <f>AVERAGE('Detail Data'!C30,'Detail Data'!D30,'Detail Data'!E30)/AVERAGE('Detail Data'!C35,'Detail Data'!D35,'Detail Data'!E35)</f>
@@ -7243,31 +7285,31 @@
     </row>
     <row r="26" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="79" t="s">
-        <v>83</v>
-      </c>
-      <c r="B26" s="397" t="s">
-        <v>84</v>
-      </c>
-      <c r="C26" s="397"/>
+        <v>297</v>
+      </c>
+      <c r="B26" s="384" t="s">
+        <v>298</v>
+      </c>
+      <c r="C26" s="384"/>
       <c r="D26" s="17"/>
-      <c r="E26" s="393" t="s">
-        <v>71</v>
-      </c>
-      <c r="F26" s="393"/>
-      <c r="G26" s="393"/>
+      <c r="E26" s="383" t="s">
+        <v>299</v>
+      </c>
+      <c r="F26" s="383"/>
+      <c r="G26" s="383"/>
       <c r="H26" s="58"/>
       <c r="I26" s="59"/>
     </row>
     <row r="27" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="395" t="s">
-        <v>85</v>
-      </c>
-      <c r="B27" s="395"/>
-      <c r="C27" s="395"/>
-      <c r="D27" s="395"/>
-      <c r="E27" s="395"/>
-      <c r="F27" s="395"/>
-      <c r="G27" s="395"/>
+      <c r="A27" s="379" t="s">
+        <v>75</v>
+      </c>
+      <c r="B27" s="379"/>
+      <c r="C27" s="379"/>
+      <c r="D27" s="379"/>
+      <c r="E27" s="379"/>
+      <c r="F27" s="379"/>
+      <c r="G27" s="379"/>
       <c r="H27" s="65"/>
       <c r="I27" s="54"/>
     </row>
@@ -7279,15 +7321,15 @@
       <c r="E28" s="81"/>
       <c r="F28" s="81"/>
       <c r="G28" s="83"/>
-      <c r="H28" s="385" t="s">
-        <v>86</v>
-      </c>
-      <c r="I28" s="385"/>
-      <c r="K28" s="385" t="s">
-        <v>87</v>
-      </c>
-      <c r="L28" s="385"/>
-      <c r="M28" s="385"/>
+      <c r="H28" s="380" t="s">
+        <v>76</v>
+      </c>
+      <c r="I28" s="380"/>
+      <c r="K28" s="380" t="s">
+        <v>77</v>
+      </c>
+      <c r="L28" s="380"/>
+      <c r="M28" s="380"/>
     </row>
     <row r="29" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="80"/>
@@ -7298,19 +7340,19 @@
       <c r="F29" s="81"/>
       <c r="G29" s="83"/>
       <c r="H29" s="58" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="I29" s="59">
         <f>'Detail Data'!E40/'Detail Data'!E5</f>
         <v>3.5847598910259015E-2</v>
       </c>
       <c r="K29" s="60" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="L29" s="84"/>
-      <c r="M29" s="85" t="e">
+      <c r="M29" s="85">
         <f>'Detail Data'!E12/(1+FrontPage!I16)</f>
-        <v>#DIV/0!</v>
+        <v>0.18935656128159478</v>
       </c>
       <c r="N29" s="86"/>
     </row>
@@ -7323,19 +7365,19 @@
       <c r="F30" s="81"/>
       <c r="G30" s="83"/>
       <c r="H30" s="58" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="I30" s="59">
         <f>AVERAGE('Detail Data'!E40,'Detail Data'!D40,'Detail Data'!C40)/AVERAGE('Detail Data'!E5,'Detail Data'!D5,'Detail Data'!C5)</f>
         <v>4.2660991037583057E-2</v>
       </c>
       <c r="K30" s="58" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="L30" s="37"/>
       <c r="M30" s="87">
         <f>'Detail Data'!E11/(1+FrontPage!I13)</f>
-        <v>0</v>
+        <v>2.5081342165232243</v>
       </c>
     </row>
     <row r="31" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -7349,11 +7391,11 @@
       <c r="H31" s="58"/>
       <c r="I31" s="59"/>
       <c r="K31" s="58" t="s">
-        <v>92</v>
-      </c>
-      <c r="M31" s="87" t="e">
+        <v>82</v>
+      </c>
+      <c r="M31" s="87">
         <f>'Detail Data'!E13/(('Detail Data'!E21/'Detail Data'!D21))</f>
-        <v>#DIV/0!</v>
+        <v>7.3716252422193271</v>
       </c>
     </row>
     <row r="32" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -7544,6 +7586,31 @@
     <row r="69" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="34">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="H1:M1"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="H2:M2"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="K5:M5"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="A11:C14"/>
+    <mergeCell ref="E11:G14"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="A16:C18"/>
+    <mergeCell ref="E16:G18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="A20:C23"/>
+    <mergeCell ref="E20:G20"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="E23:G23"/>
     <mergeCell ref="A27:G27"/>
     <mergeCell ref="H28:I28"/>
     <mergeCell ref="K28:M28"/>
@@ -7553,31 +7620,6 @@
     <mergeCell ref="E25:G25"/>
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="E26:G26"/>
-    <mergeCell ref="A20:C23"/>
-    <mergeCell ref="E20:G20"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="E22:G22"/>
-    <mergeCell ref="E23:G23"/>
-    <mergeCell ref="A16:C18"/>
-    <mergeCell ref="E16:G18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="A11:C14"/>
-    <mergeCell ref="E11:G14"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="E15:G15"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="K5:M5"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="H1:M1"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="H2:M2"/>
-    <mergeCell ref="F3:G3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.45" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
@@ -7614,7 +7656,7 @@
     </row>
     <row r="2" spans="1:7" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="45" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="B2" s="95"/>
       <c r="C2" s="96" t="str">
@@ -7640,54 +7682,54 @@
     </row>
     <row r="3" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="98" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="B3" s="99"/>
       <c r="C3" s="100">
         <f>C9*FrontPage!$C3</f>
-        <v>0</v>
+        <v>32450.11</v>
       </c>
       <c r="D3" s="100">
         <f>D9*FrontPage!C3</f>
-        <v>0</v>
+        <v>32434.164000000004</v>
       </c>
       <c r="E3" s="101">
         <f>E9*FrontPage!C3</f>
-        <v>0</v>
+        <v>32434.164000000004</v>
       </c>
       <c r="F3" s="101">
         <f>F9*FrontPage!C3</f>
-        <v>0</v>
+        <v>32434.164000000004</v>
       </c>
       <c r="G3" s="102">
         <f>G9*FrontPage!C3</f>
-        <v>0</v>
+        <v>32434.164000000004</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="103" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="B4" s="104"/>
       <c r="C4" s="105">
         <f>C3+C34-C28</f>
-        <v>2459.5</v>
+        <v>34909.61</v>
       </c>
       <c r="D4" s="105">
         <f>D3+D34-D28</f>
-        <v>3755.2999999999997</v>
+        <v>36189.464</v>
       </c>
       <c r="E4" s="105">
         <f>E3+E34-E28</f>
-        <v>3242.2</v>
+        <v>35676.364000000001</v>
       </c>
       <c r="F4" s="105">
         <f>F3+F34-F28</f>
-        <v>2991.5</v>
+        <v>35425.664000000004</v>
       </c>
       <c r="G4" s="106">
         <f>G3+G34-G28</f>
-        <v>2650.8</v>
+        <v>35084.964000000007</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -7742,19 +7784,23 @@
         <v>FD EPS (t) - Current FY</v>
       </c>
       <c r="B7" s="108"/>
-      <c r="C7" s="113"/>
-      <c r="D7" s="113"/>
-      <c r="E7" s="114" t="e">
+      <c r="C7" s="113">
+        <v>10.92</v>
+      </c>
+      <c r="D7" s="113">
+        <v>4.34</v>
+      </c>
+      <c r="E7" s="114">
         <f>E5/E9</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F7" s="114" t="e">
+        <v>60.454768928220254</v>
+      </c>
+      <c r="F7" s="114">
         <f>F5/F9</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G7" s="114" t="e">
+        <v>61.964110127826942</v>
+      </c>
+      <c r="G7" s="114">
         <f t="shared" ref="G7" si="0">G5/G9</f>
-        <v>#DIV/0!</v>
+        <v>63.578662733529988</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -7762,44 +7808,52 @@
         <f>CONCATENATE("FD EPS (t-1) - Previous FY")</f>
         <v>FD EPS (t-1) - Previous FY</v>
       </c>
-      <c r="C8" s="113"/>
-      <c r="D8" s="113"/>
+      <c r="C8" s="113">
+        <v>9.06</v>
+      </c>
+      <c r="D8" s="113">
+        <v>10.92</v>
+      </c>
       <c r="E8" s="114">
         <f>D7</f>
-        <v>0</v>
-      </c>
-      <c r="F8" s="114" t="e">
+        <v>4.34</v>
+      </c>
+      <c r="F8" s="114">
         <f t="shared" ref="F8:G8" si="1">E7</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G8" s="114" t="e">
+        <v>60.454768928220254</v>
+      </c>
+      <c r="G8" s="114">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
+        <v>61.964110127826942</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A9" s="115" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="B9" s="116"/>
-      <c r="C9" s="117"/>
-      <c r="D9" s="117"/>
+      <c r="C9" s="117">
+        <v>203.5</v>
+      </c>
+      <c r="D9" s="117">
+        <v>203.4</v>
+      </c>
       <c r="E9" s="119">
         <f>D9</f>
-        <v>0</v>
+        <v>203.4</v>
       </c>
       <c r="F9" s="118">
         <f t="shared" ref="F9:G9" si="2">E9</f>
-        <v>0</v>
+        <v>203.4</v>
       </c>
       <c r="G9" s="120">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>203.4</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A10" s="121" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B10" s="122"/>
       <c r="C10" s="123" t="str">
@@ -7825,85 +7879,85 @@
     </row>
     <row r="11" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="124" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B11" s="125"/>
       <c r="C11" s="126">
         <f>(FrontPage!$C3*C9)/C5</f>
-        <v>0</v>
+        <v>2.8967363844924705</v>
       </c>
       <c r="D11" s="126">
         <f>(FrontPage!C3*D9)/D5</f>
-        <v>0</v>
+        <v>2.7739052050014541</v>
       </c>
       <c r="E11" s="126">
         <f>E3/E5</f>
-        <v>0</v>
+        <v>2.6376744602122559</v>
       </c>
       <c r="F11" s="126">
         <f t="shared" ref="F11:G11" si="4">F3/F5</f>
-        <v>0</v>
+        <v>2.5734251596778677</v>
       </c>
       <c r="G11" s="126">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>2.5080741422374131</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="127" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="B12" s="128"/>
-      <c r="C12" s="129" t="e">
+      <c r="C12" s="129">
         <f>FrontPage!$C3/C7</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D12" s="129" t="e">
+        <v>14.602564102564104</v>
+      </c>
+      <c r="D12" s="129">
         <f>FrontPage!C3/D7</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E12" s="129" t="e">
+        <v>36.741935483870968</v>
+      </c>
+      <c r="E12" s="129">
         <f>FrontPage!C3/E7</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F12" s="129" t="e">
+        <v>2.6376744602122559</v>
+      </c>
+      <c r="F12" s="129">
         <f>FrontPage!$C3/F7</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G12" s="130" t="e">
+        <v>2.5734251596778672</v>
+      </c>
+      <c r="G12" s="130">
         <f>FrontPage!$C3/G7</f>
-        <v>#DIV/0!</v>
+        <v>2.5080741422374131</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A13" s="131" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="B13" s="132"/>
-      <c r="C13" s="129" t="e">
+      <c r="C13" s="129">
         <f>$C4/C21</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D13" s="129" t="e">
+        <v>10.409903086327718</v>
+      </c>
+      <c r="D13" s="129">
         <f t="shared" ref="D13:G13" si="5">$C4/D21</f>
-        <v>#DIV/0!</v>
+        <v>17.946540201521696</v>
       </c>
       <c r="E13" s="129">
         <f t="shared" si="5"/>
-        <v>0.81035221244769529</v>
+        <v>11.501963691476393</v>
       </c>
       <c r="F13" s="129">
         <f t="shared" si="5"/>
-        <v>0.7247038717661618</v>
+        <v>10.286289704755731</v>
       </c>
       <c r="G13" s="129">
         <f t="shared" si="5"/>
-        <v>0.69199819931348827</v>
+        <v>9.8220724776320978</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A14" s="133" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="B14" s="134"/>
       <c r="C14" s="122" t="str">
@@ -7929,7 +7983,7 @@
     </row>
     <row r="15" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="124" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="B15" s="125"/>
       <c r="C15" s="136">
@@ -7950,7 +8004,7 @@
     </row>
     <row r="16" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="107" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="B16" s="137"/>
       <c r="C16" s="138">
@@ -7974,7 +8028,7 @@
     </row>
     <row r="17" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="107" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="B17" s="137"/>
       <c r="C17" s="138">
@@ -8019,7 +8073,7 @@
     </row>
     <row r="19" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="107" t="s">
-        <v>237</v>
+        <v>227</v>
       </c>
       <c r="C19" s="138">
         <v>165.7</v>
@@ -8042,7 +8096,7 @@
     </row>
     <row r="20" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="107" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="C20" s="138">
         <v>252.7</v>
@@ -8062,11 +8116,15 @@
     </row>
     <row r="21" spans="1:7" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A21" s="141" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="B21" s="142"/>
-      <c r="C21" s="353"/>
-      <c r="D21" s="353"/>
+      <c r="C21" s="353">
+        <v>3353.5</v>
+      </c>
+      <c r="D21" s="353">
+        <v>1945.2</v>
+      </c>
       <c r="E21" s="353">
         <v>3035.1</v>
       </c>
@@ -8079,7 +8137,7 @@
     </row>
     <row r="22" spans="1:7" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A22" s="133" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="B22" s="134"/>
       <c r="C22" s="123" t="str">
@@ -8105,7 +8163,7 @@
     </row>
     <row r="23" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="124" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="B23" s="125"/>
       <c r="C23" s="143">
@@ -8131,7 +8189,7 @@
     </row>
     <row r="24" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="131" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="B24" s="132"/>
       <c r="C24" s="145">
@@ -8157,7 +8215,7 @@
     </row>
     <row r="25" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="131" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="C25" s="145">
         <f>C17/C5</f>
@@ -8182,16 +8240,16 @@
     </row>
     <row r="26" spans="1:7" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A26" s="147" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="B26" s="148"/>
       <c r="C26" s="149">
         <f>C21/C5</f>
-        <v>0</v>
+        <v>0.29935816751917022</v>
       </c>
       <c r="D26" s="149">
         <f>D21/D5</f>
-        <v>0</v>
+        <v>0.16636163043292337</v>
       </c>
       <c r="E26" s="149">
         <f>E21/E5</f>
@@ -8208,7 +8266,7 @@
     </row>
     <row r="27" spans="1:7" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A27" s="151" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="B27" s="152"/>
       <c r="C27" s="123" t="str">
@@ -8234,7 +8292,7 @@
     </row>
     <row r="28" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="124" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="B28" s="125"/>
       <c r="C28" s="136">
@@ -8255,33 +8313,33 @@
     </row>
     <row r="29" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="127" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="B29" s="128"/>
-      <c r="C29" s="153" t="e">
+      <c r="C29" s="153">
         <f>C28/C9</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D29" s="153" t="e">
+        <v>3.5906633906633907</v>
+      </c>
+      <c r="D29" s="153">
         <f>D28/D9</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E29" s="153" t="e">
+        <v>4.5521140609636186</v>
+      </c>
+      <c r="E29" s="153">
         <f>E28/E9</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F29" s="153" t="e">
+        <v>7.1361848574237952</v>
+      </c>
+      <c r="F29" s="153">
         <f>F28/F9</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G29" s="154" t="e">
+        <v>8.040806293018683</v>
+      </c>
+      <c r="G29" s="154">
         <f>G28/G9</f>
-        <v>#DIV/0!</v>
+        <v>9.387905604719764</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="127" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="B30" s="128"/>
       <c r="C30" s="355">
@@ -8302,7 +8360,7 @@
     </row>
     <row r="31" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="131" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="B31" s="132"/>
       <c r="C31" s="138">
@@ -8323,7 +8381,7 @@
     </row>
     <row r="32" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="131" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="B32" s="132"/>
       <c r="C32" s="138">
@@ -8344,7 +8402,7 @@
     </row>
     <row r="33" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="131" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="B33" s="132"/>
       <c r="C33" s="139">
@@ -8370,7 +8428,7 @@
     </row>
     <row r="34" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="131" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="C34" s="138">
         <v>3190.2</v>
@@ -8390,7 +8448,7 @@
     </row>
     <row r="35" spans="1:10" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A35" s="147" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="B35" s="92"/>
       <c r="C35" s="156">
@@ -8411,7 +8469,7 @@
     </row>
     <row r="36" spans="1:10" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A36" s="151" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="B36" s="152"/>
       <c r="C36" s="123" t="str">
@@ -8437,7 +8495,7 @@
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A37" s="88" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="C37" s="138"/>
       <c r="D37" s="138"/>
@@ -8456,7 +8514,7 @@
     </row>
     <row r="38" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A38" s="131" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="B38" s="132"/>
       <c r="C38" s="138">
@@ -8480,7 +8538,7 @@
     </row>
     <row r="39" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A39" s="131" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="C39" s="138"/>
       <c r="D39" s="138"/>
@@ -8499,7 +8557,7 @@
     </row>
     <row r="40" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A40" s="131" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="B40" s="132"/>
       <c r="C40" s="138">
@@ -8520,10 +8578,10 @@
     </row>
     <row r="41" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A41" s="131" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="B41" s="131" t="s">
-        <v>235</v>
+        <v>225</v>
       </c>
       <c r="D41" s="138"/>
       <c r="E41" s="139">
@@ -8541,10 +8599,10 @@
     </row>
     <row r="42" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A42" s="131" t="s">
-        <v>234</v>
+        <v>224</v>
       </c>
       <c r="B42" s="131" t="s">
-        <v>236</v>
+        <v>226</v>
       </c>
       <c r="D42" s="138"/>
       <c r="E42" s="139">
@@ -8563,7 +8621,7 @@
     <row r="43" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="44" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A44" s="88" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="D44" s="349">
         <f>(D33+D40)/D17</f>
@@ -8584,32 +8642,32 @@
     </row>
     <row r="45" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A45" s="88" t="s">
-        <v>253</v>
-      </c>
-      <c r="C45" s="349" t="e">
+        <v>243</v>
+      </c>
+      <c r="C45" s="349">
         <f>C34/C3</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D45" s="349" t="e">
+        <v>9.8310914816621575E-2</v>
+      </c>
+      <c r="D45" s="349">
         <f>D34/D3</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E45" s="349" t="e">
+        <v>0.1443292942589795</v>
+      </c>
+      <c r="E45" s="349">
         <f t="shared" ref="E45:G45" si="13">E34/E3</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F45" s="349" t="e">
+        <v>0.14471469034934889</v>
+      </c>
+      <c r="F45" s="349">
         <f t="shared" si="13"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G45" s="349" t="e">
+        <v>0.14265821681113777</v>
+      </c>
+      <c r="G45" s="349">
         <f t="shared" si="13"/>
-        <v>#DIV/0!</v>
+        <v>0.14060174327292665</v>
       </c>
     </row>
     <row r="46" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A46" s="88" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D46" s="349">
         <f>D17/D35</f>
@@ -8628,12 +8686,12 @@
         <v>0.38744533058914332</v>
       </c>
       <c r="J46" s="88" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
     </row>
     <row r="47" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A47" s="88" t="s">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="D47" s="349">
         <f>D16*(1-'DCF 1-Pager'!D25)/(C34+C35-C28)</f>
@@ -8652,13 +8710,13 @@
         <v>0.28209510180394048</v>
       </c>
       <c r="J47" s="88" t="s">
-        <v>275</v>
+        <v>264</v>
       </c>
     </row>
     <row r="48" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="49" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A49" s="88" t="s">
-        <v>259</v>
+        <v>249</v>
       </c>
       <c r="D49" s="378">
         <f>D46*D44</f>
@@ -8679,7 +8737,7 @@
     </row>
     <row r="50" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A50" s="88" t="s">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="D50" s="349">
         <f>D47*D44</f>
@@ -8701,7 +8759,7 @@
     <row r="51" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="52" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A52" s="88" t="s">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="B52" s="88">
         <v>0.03</v>
@@ -8709,7 +8767,7 @@
     </row>
     <row r="53" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A53" s="88" t="s">
-        <v>262</v>
+        <v>252</v>
       </c>
       <c r="D53" s="349">
         <f>$B$52/D46</f>
@@ -8730,7 +8788,7 @@
     </row>
     <row r="54" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A54" s="88" t="s">
-        <v>261</v>
+        <v>251</v>
       </c>
       <c r="D54" s="349">
         <f>$B$52/D47</f>
@@ -8752,7 +8810,7 @@
     <row r="55" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="56" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A56" s="88" t="s">
-        <v>264</v>
+        <v>253</v>
       </c>
       <c r="D56" s="155">
         <f>D16/D19</f>
@@ -8857,7 +8915,7 @@
     <row r="1" spans="2:22" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:22" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B2" s="163" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="C2" s="164"/>
       <c r="D2" s="164"/>
@@ -8869,15 +8927,15 @@
     </row>
     <row r="3" spans="2:22" ht="21" x14ac:dyDescent="0.25">
       <c r="B3" s="165" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="L3" s="401" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="M3" s="402"/>
       <c r="N3" s="403"/>
       <c r="P3" s="404" t="s">
-        <v>289</v>
+        <v>278</v>
       </c>
       <c r="Q3" s="405"/>
       <c r="R3" s="405"/>
@@ -8888,52 +8946,52 @@
     </row>
     <row r="4" spans="2:22" ht="21" x14ac:dyDescent="0.25">
       <c r="B4" s="162" t="s">
-        <v>129</v>
-      </c>
-      <c r="D4" s="162">
+        <v>119</v>
+      </c>
+      <c r="D4" s="162" t="str">
         <f>FrontPage!A1</f>
-        <v>0</v>
+        <v>The Hershey Company (HSY)</v>
       </c>
       <c r="L4" s="339"/>
       <c r="M4" s="399" t="s">
-        <v>249</v>
+        <v>239</v>
       </c>
       <c r="N4" s="400"/>
       <c r="P4" s="371"/>
       <c r="Q4" s="372"/>
       <c r="R4" s="372" t="s">
-        <v>284</v>
+        <v>273</v>
       </c>
       <c r="S4" s="372" t="s">
-        <v>285</v>
+        <v>274</v>
       </c>
       <c r="T4" s="372" t="s">
-        <v>286</v>
+        <v>275</v>
       </c>
       <c r="U4" s="372" t="s">
-        <v>287</v>
+        <v>276</v>
       </c>
       <c r="V4" s="373" t="s">
-        <v>288</v>
+        <v>277</v>
       </c>
     </row>
     <row r="5" spans="2:22" ht="22" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="162" t="s">
-        <v>130</v>
-      </c>
-      <c r="D5" s="162">
+        <v>120</v>
+      </c>
+      <c r="D5" s="162" t="str">
         <f>FrontPage!C2</f>
-        <v>0</v>
+        <v>HSY</v>
       </c>
       <c r="L5" s="343"/>
       <c r="M5" s="369" t="s">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="N5" s="370" t="s">
-        <v>282</v>
+        <v>271</v>
       </c>
       <c r="P5" s="371" t="s">
-        <v>283</v>
+        <v>272</v>
       </c>
       <c r="Q5" s="372" t="e">
         <f>AVERAGE('Relative Valuation'!D4:D6)</f>
@@ -8962,13 +9020,13 @@
     </row>
     <row r="6" spans="2:22" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="162" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="D6" s="166">
         <v>46022</v>
       </c>
       <c r="F6" s="162" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="H6" s="167">
         <f>'WACC calculation'!D16</f>
@@ -8978,7 +9036,7 @@
       <c r="M6" s="337"/>
       <c r="N6" s="341"/>
       <c r="P6" s="371" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="Q6" s="372" t="e">
         <f>AVERAGE('Relative Valuation'!C4:C6)</f>
@@ -8986,7 +9044,7 @@
       </c>
       <c r="R6" s="372">
         <f>D19</f>
-        <v>0</v>
+        <v>1945.2</v>
       </c>
       <c r="S6" s="372" t="e">
         <f>R6*Q6</f>
@@ -9007,21 +9065,21 @@
     </row>
     <row r="7" spans="2:22" ht="22" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="162" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="D7" s="168">
         <f>EOMONTH(D6,12)</f>
         <v>46387</v>
       </c>
       <c r="F7" s="162" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="H7" s="169">
         <f>FrontPage!C3</f>
-        <v>0</v>
+        <v>159.46</v>
       </c>
       <c r="L7" s="339" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="M7" s="338">
         <f>C77</f>
@@ -9032,7 +9090,7 @@
         <v>-1.8128026589484418E-2</v>
       </c>
       <c r="P7" s="375" t="s">
-        <v>281</v>
+        <v>270</v>
       </c>
       <c r="Q7" s="376" t="e">
         <f>AVERAGE('Relative Valuation'!E4:E6)</f>
@@ -9061,13 +9119,13 @@
     </row>
     <row r="8" spans="2:22" ht="22" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="162" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="D8" s="166">
         <v>46203</v>
       </c>
       <c r="F8" s="162" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="H8" s="170">
         <f>D9</f>
@@ -9075,7 +9133,7 @@
       </c>
       <c r="J8" s="171"/>
       <c r="L8" s="343" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="M8" s="344">
         <f>C108</f>
@@ -9088,14 +9146,14 @@
     </row>
     <row r="9" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B9" s="162" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="D9" s="166">
         <f>FrontPage!C4</f>
         <v>46299</v>
       </c>
       <c r="F9" s="162" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="H9" s="172">
         <v>0</v>
@@ -9105,7 +9163,7 @@
     </row>
     <row r="10" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B10" s="162" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="D10" s="173">
         <f>YEARFRAC(D9,D7)</f>
@@ -9117,7 +9175,7 @@
     </row>
     <row r="12" spans="2:22" ht="24" x14ac:dyDescent="0.3">
       <c r="B12" s="295" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
       <c r="C12" s="237"/>
       <c r="D12" s="335"/>
@@ -9130,7 +9188,7 @@
     </row>
     <row r="13" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B13" s="242" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="J13" s="255"/>
     </row>
@@ -9138,10 +9196,10 @@
       <c r="B14" s="245"/>
       <c r="C14" s="177"/>
       <c r="D14" s="177" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="E14" s="398" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="F14" s="398"/>
       <c r="G14" s="398"/>
@@ -9151,7 +9209,7 @@
     </row>
     <row r="15" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B15" s="281" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C15" s="297"/>
       <c r="D15" s="329" t="str">
@@ -9186,7 +9244,7 @@
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B17" s="245" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C17" s="262"/>
       <c r="D17" s="302">
@@ -9211,7 +9269,7 @@
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B18" s="282" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="E18" s="299">
         <f>E17/D17-1</f>
@@ -9232,12 +9290,12 @@
     </row>
     <row r="19" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B19" s="245" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="C19" s="262"/>
       <c r="D19" s="302">
         <f>'Detail Data'!D21</f>
-        <v>0</v>
+        <v>1945.2</v>
       </c>
       <c r="E19" s="262">
         <f>'Detail Data'!E21</f>
@@ -9257,11 +9315,11 @@
     </row>
     <row r="20" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B20" s="282" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="D20" s="173">
         <f>D19/D17</f>
-        <v>0</v>
+        <v>0.16636163043292337</v>
       </c>
       <c r="E20" s="173">
         <f t="shared" ref="E20:G20" si="2">E19/E17</f>
@@ -9281,7 +9339,7 @@
     </row>
     <row r="21" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B21" s="245" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="D21" s="302">
         <f>'Detail Data'!D16</f>
@@ -9305,7 +9363,7 @@
     </row>
     <row r="22" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B22" s="282" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="D22" s="173">
         <f>D21/D17</f>
@@ -9339,7 +9397,7 @@
     </row>
     <row r="24" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="245" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="C24" s="262"/>
       <c r="D24" s="262">
@@ -9364,7 +9422,7 @@
     </row>
     <row r="25" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="282" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="D25" s="331">
         <f>'Detail Data'!D20/'Detail Data'!D17</f>
@@ -9388,7 +9446,7 @@
     </row>
     <row r="26" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="242" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="C26" s="178"/>
       <c r="D26" s="253">
@@ -9423,7 +9481,7 @@
     </row>
     <row r="28" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="245" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="D28" s="262">
         <f>'Detail Data'!D38</f>
@@ -9448,7 +9506,7 @@
     </row>
     <row r="29" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="245" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
       <c r="D29" s="262">
         <f>C36-D36</f>
@@ -9473,7 +9531,7 @@
     </row>
     <row r="30" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="245" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="D30" s="302">
         <f>-'Detail Data'!D40</f>
@@ -9498,7 +9556,7 @@
     </row>
     <row r="31" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="282" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="D31" s="173">
         <f>FrontPage!I30</f>
@@ -9534,7 +9592,7 @@
     </row>
     <row r="33" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B33" s="283" t="s">
-        <v>238</v>
+        <v>228</v>
       </c>
       <c r="D33" s="302"/>
       <c r="E33" s="303"/>
@@ -9547,7 +9605,7 @@
     </row>
     <row r="34" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B34" s="242" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="C34" s="178"/>
       <c r="D34" s="253"/>
@@ -9567,7 +9625,7 @@
     </row>
     <row r="36" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B36" s="245" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="C36" s="302">
         <f>'Detail Data'!C33</f>
@@ -9595,7 +9653,7 @@
     </row>
     <row r="37" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B37" s="282" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="D37" s="173">
         <f>D36/D17</f>
@@ -9644,16 +9702,16 @@
     <row r="40" spans="2:13" ht="18" x14ac:dyDescent="0.35">
       <c r="B40" s="242"/>
       <c r="D40" s="332" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="E40" s="332" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="F40" s="243" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="G40" s="243" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="H40" s="243"/>
       <c r="I40" s="243"/>
@@ -9661,7 +9719,7 @@
     </row>
     <row r="41" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B41" s="245" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="C41" s="246"/>
       <c r="D41" s="247">
@@ -9686,7 +9744,7 @@
     </row>
     <row r="42" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B42" s="245" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
       <c r="C42" s="250">
         <f>D10</f>
@@ -9709,12 +9767,12 @@
       <c r="I42" s="262"/>
       <c r="J42" s="305"/>
       <c r="K42" s="162" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
     </row>
     <row r="43" spans="2:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B43" s="242" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="C43" s="252"/>
       <c r="E43" s="253">
@@ -9742,21 +9800,21 @@
     </row>
     <row r="45" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B45" s="242" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="C45" s="178"/>
       <c r="E45" s="178" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="J45" s="255"/>
     </row>
     <row r="46" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B46" s="245" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="C46" s="257"/>
       <c r="E46" s="162" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="I46" s="179"/>
       <c r="J46" s="259"/>
@@ -9768,10 +9826,10 @@
       </c>
       <c r="C47" s="179"/>
       <c r="D47" s="364" t="s">
-        <v>276</v>
+        <v>265</v>
       </c>
       <c r="E47" s="162" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="I47" s="306"/>
       <c r="J47" s="261"/>
@@ -9789,39 +9847,39 @@
       <c r="I48" s="179"/>
       <c r="J48" s="259"/>
       <c r="L48" s="364" t="s">
-        <v>277</v>
+        <v>266</v>
       </c>
     </row>
     <row r="49" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B49" s="245" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="C49" s="253"/>
       <c r="E49" s="162" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="I49" s="253"/>
       <c r="J49" s="259"/>
     </row>
     <row r="50" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B50" s="245" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="C50" s="253"/>
       <c r="E50" s="162" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="I50" s="179"/>
       <c r="J50" s="259"/>
     </row>
     <row r="51" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B51" s="242" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="C51" s="263"/>
       <c r="D51" s="264"/>
       <c r="E51" s="178" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="I51" s="263"/>
       <c r="J51" s="265"/>
@@ -9833,14 +9891,14 @@
     </row>
     <row r="53" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B53" s="267" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="C53" s="268" t="e">
         <f>C49/$C$51</f>
         <v>#DIV/0!</v>
       </c>
       <c r="E53" s="269" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="I53" s="268" t="e">
         <f>I49/$I$51</f>
@@ -9850,14 +9908,14 @@
     </row>
     <row r="54" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B54" s="267" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="C54" s="268" t="e">
         <f t="shared" ref="C54" si="11">C50/$C$51</f>
         <v>#DIV/0!</v>
       </c>
       <c r="E54" s="269" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="G54" s="271"/>
       <c r="I54" s="268" t="e">
@@ -9868,14 +9926,14 @@
     </row>
     <row r="55" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B55" s="267" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="C55" s="272">
         <f>C48/G19</f>
         <v>0</v>
       </c>
       <c r="E55" s="162" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
       <c r="I55" s="308" t="e">
         <f>(H6-G42/I48)/(1+G42/I48)</f>
@@ -9892,52 +9950,52 @@
     </row>
     <row r="57" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B57" s="242" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="E57" s="178" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="G57" s="178"/>
       <c r="J57" s="255"/>
     </row>
     <row r="58" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B58" s="245" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="C58" s="170" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="J58" s="255"/>
       <c r="L58" s="333"/>
     </row>
     <row r="59" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B59" s="284" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
       <c r="C59" s="166">
         <v>46022</v>
       </c>
       <c r="G59" s="310" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="H59" s="311" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="I59" s="311" t="s">
-        <v>184</v>
+        <v>174</v>
       </c>
       <c r="J59" s="255"/>
     </row>
     <row r="60" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B60" s="285" t="s">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="C60" s="168"/>
       <c r="E60" s="162" t="s">
-        <v>186</v>
+        <v>176</v>
       </c>
       <c r="G60" s="170" t="s">
-        <v>187</v>
+        <v>177</v>
       </c>
       <c r="H60" s="170">
         <v>43847</v>
@@ -9950,20 +10008,20 @@
     </row>
     <row r="61" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B61" s="282" t="s">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="C61" s="301">
         <f>'Detail Data'!D34</f>
         <v>4681.2</v>
       </c>
       <c r="D61" s="364" t="s">
-        <v>278</v>
+        <v>267</v>
       </c>
       <c r="E61" s="183" t="s">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="G61" s="170" t="s">
-        <v>187</v>
+        <v>177</v>
       </c>
       <c r="H61" s="170">
         <v>43827</v>
@@ -9975,11 +10033,11 @@
     </row>
     <row r="62" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B62" s="282" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="C62" s="315"/>
       <c r="E62" s="183" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="G62" s="170"/>
       <c r="H62" s="170"/>
@@ -9988,16 +10046,16 @@
       </c>
       <c r="J62" s="255"/>
       <c r="K62" s="162" t="s">
-        <v>192</v>
+        <v>182</v>
       </c>
     </row>
     <row r="63" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B63" s="282" t="s">
-        <v>193</v>
+        <v>183</v>
       </c>
       <c r="C63" s="315"/>
       <c r="E63" s="162" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="G63" s="170"/>
       <c r="H63" s="170"/>
@@ -10006,16 +10064,16 @@
       </c>
       <c r="J63" s="255"/>
       <c r="K63" s="162" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
     </row>
     <row r="64" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B64" s="286" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="C64" s="303"/>
       <c r="E64" s="162" t="s">
-        <v>196</v>
+        <v>186</v>
       </c>
       <c r="G64" s="170"/>
       <c r="H64" s="170"/>
@@ -10024,15 +10082,15 @@
       </c>
       <c r="J64" s="255"/>
       <c r="K64" s="162" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
     </row>
     <row r="65" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B65" s="285" t="s">
-        <v>198</v>
+        <v>188</v>
       </c>
       <c r="E65" s="317" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
       <c r="I65" s="318">
         <f>SUM(I60:I64)</f>
@@ -10042,7 +10100,7 @@
     </row>
     <row r="66" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B66" s="287" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="C66" s="303">
         <f>'Detail Data'!D28</f>
@@ -10058,7 +10116,7 @@
     </row>
     <row r="67" spans="2:14" ht="18" x14ac:dyDescent="0.35">
       <c r="B67" s="287" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="C67" s="303"/>
       <c r="G67" s="178"/>
@@ -10081,7 +10139,7 @@
     </row>
     <row r="69" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B69" s="288" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="C69" s="321">
         <f>SUM(C61:C64)-SUM(C66:C67)</f>
@@ -10107,17 +10165,17 @@
     </row>
     <row r="71" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B71" s="242" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="J71" s="255"/>
     </row>
     <row r="72" spans="2:14" ht="18" x14ac:dyDescent="0.35">
       <c r="B72" s="245"/>
       <c r="C72" s="274" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
       <c r="D72" s="274" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="G72" s="178"/>
       <c r="H72" s="178"/>
@@ -10125,7 +10183,7 @@
     </row>
     <row r="73" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B73" s="245" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="C73" s="322">
         <f>C51</f>
@@ -10141,7 +10199,7 @@
     </row>
     <row r="74" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B74" s="245" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="C74" s="334">
         <f>C69</f>
@@ -10158,7 +10216,7 @@
     </row>
     <row r="75" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B75" s="245" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="C75" s="275">
         <f>C73-C74</f>
@@ -10174,7 +10232,7 @@
     </row>
     <row r="76" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B76" s="245" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="C76" s="275">
         <f>I65</f>
@@ -10190,7 +10248,7 @@
     </row>
     <row r="77" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B77" s="242" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
       <c r="C77" s="324">
         <f>C75/C76</f>
@@ -10216,13 +10274,13 @@
     </row>
     <row r="79" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B79" s="289" t="s">
-        <v>207</v>
+        <v>197</v>
       </c>
       <c r="C79" s="311" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
       <c r="D79" s="311" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="E79" s="326"/>
       <c r="F79" s="326"/>
@@ -10231,7 +10289,7 @@
     </row>
     <row r="80" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B80" s="245" t="s">
-        <v>208</v>
+        <v>198</v>
       </c>
       <c r="C80" s="327">
         <f>C73/$E$17</f>
@@ -10250,7 +10308,7 @@
     </row>
     <row r="81" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B81" s="245" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="C81" s="326">
         <f>C73/$E$19</f>
@@ -10270,7 +10328,7 @@
     </row>
     <row r="82" spans="2:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B82" s="290" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="C82" s="291">
         <f>C73/$E$21</f>
@@ -10296,7 +10354,7 @@
     </row>
     <row r="85" spans="2:14" ht="24" x14ac:dyDescent="0.3">
       <c r="B85" s="295" t="s">
-        <v>239</v>
+        <v>229</v>
       </c>
       <c r="C85" s="237"/>
       <c r="D85" s="237"/>
@@ -10322,23 +10380,23 @@
     <row r="87" spans="2:14" ht="18" x14ac:dyDescent="0.35">
       <c r="B87" s="242"/>
       <c r="D87" s="181" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="E87" s="181" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="F87" s="243" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="G87" s="243" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="H87" s="243"/>
       <c r="I87" s="244"/>
     </row>
     <row r="88" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B88" s="245" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="C88" s="246"/>
       <c r="D88" s="247">
@@ -10362,7 +10420,7 @@
     </row>
     <row r="89" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B89" s="245" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
       <c r="C89" s="250">
         <f>C42</f>
@@ -10386,7 +10444,7 @@
     </row>
     <row r="90" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B90" s="242" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="C90" s="252"/>
       <c r="E90" s="253">
@@ -10410,11 +10468,11 @@
     </row>
     <row r="92" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B92" s="240" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="C92" s="175"/>
       <c r="E92" s="175" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="F92" s="176"/>
       <c r="G92" s="176"/>
@@ -10423,11 +10481,11 @@
     </row>
     <row r="93" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B93" s="245" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="C93" s="257"/>
       <c r="E93" s="258" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="I93" s="179"/>
     </row>
@@ -10438,7 +10496,7 @@
       </c>
       <c r="C94" s="179"/>
       <c r="E94" s="296" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
     </row>
     <row r="95" spans="2:14" x14ac:dyDescent="0.2">
@@ -10455,32 +10513,32 @@
     </row>
     <row r="96" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B96" s="245" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="C96" s="253"/>
       <c r="E96" s="162" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="I96" s="253"/>
     </row>
     <row r="97" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B97" s="245" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="C97" s="262"/>
       <c r="E97" s="162" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="I97" s="179"/>
     </row>
     <row r="98" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B98" s="242" t="s">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="C98" s="263"/>
       <c r="D98" s="264"/>
       <c r="E98" s="178" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="I98" s="179"/>
     </row>
@@ -10491,14 +10549,14 @@
     </row>
     <row r="100" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B100" s="267" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="C100" s="268" t="e">
         <f>C96/C98</f>
         <v>#DIV/0!</v>
       </c>
       <c r="E100" s="269" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="I100" s="365" t="e">
         <f>I96/I98</f>
@@ -10507,14 +10565,14 @@
     </row>
     <row r="101" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B101" s="267" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="C101" s="268" t="e">
         <f t="shared" ref="C101" si="13">C97/$C$51</f>
         <v>#DIV/0!</v>
       </c>
       <c r="E101" s="269" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="G101" s="271"/>
       <c r="I101" s="365" t="e">
@@ -10524,14 +10582,14 @@
     </row>
     <row r="102" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B102" s="267" t="s">
-        <v>279</v>
+        <v>268</v>
       </c>
       <c r="C102" s="272">
         <f>C95/(G21-G24)</f>
         <v>0</v>
       </c>
       <c r="E102" s="162" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
       <c r="I102" s="273" t="e">
         <f>('WACC calculation'!D11-'DCF 1-Pager'!G89/'DCF 1-Pager'!I95)/(1+('DCF 1-Pager'!G89/'DCF 1-Pager'!I95))</f>
@@ -10545,7 +10603,7 @@
     </row>
     <row r="104" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B104" s="240" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="C104" s="176"/>
       <c r="D104" s="176"/>
@@ -10554,10 +10612,10 @@
     <row r="105" spans="2:17" ht="18" x14ac:dyDescent="0.35">
       <c r="B105" s="245"/>
       <c r="C105" s="274" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
       <c r="D105" s="274" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="G105" s="175"/>
       <c r="H105" s="175"/>
@@ -10570,7 +10628,7 @@
     </row>
     <row r="106" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B106" s="245" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="C106" s="275">
         <f>C98</f>
@@ -10586,7 +10644,7 @@
     </row>
     <row r="107" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B107" s="245" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="C107" s="275">
         <v>205306</v>
@@ -10601,7 +10659,7 @@
     </row>
     <row r="108" spans="2:17" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B108" s="276" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
       <c r="C108" s="277">
         <f>C106/C107</f>
@@ -10623,7 +10681,7 @@
     </row>
     <row r="110" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B110" s="175" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="C110" s="175"/>
       <c r="D110" s="175"/>
@@ -10648,7 +10706,7 @@
       <c r="B112" s="185"/>
       <c r="C112" s="178"/>
       <c r="D112" s="186" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
       <c r="E112" s="177"/>
       <c r="F112" s="177"/>
@@ -10657,7 +10715,7 @@
       <c r="I112" s="177"/>
       <c r="J112" s="187"/>
       <c r="L112" s="186" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="M112" s="177"/>
       <c r="N112" s="177"/>
@@ -10669,7 +10727,7 @@
       <c r="B113" s="185"/>
       <c r="D113" s="183"/>
       <c r="E113" s="188" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="F113" s="188"/>
       <c r="G113" s="188"/>
@@ -10678,7 +10736,7 @@
       <c r="J113" s="189"/>
       <c r="L113" s="183"/>
       <c r="M113" s="188" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="N113" s="188"/>
       <c r="O113" s="188"/>
@@ -10825,7 +10883,7 @@
     <row r="117" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B117" s="185"/>
       <c r="C117" s="190" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="D117" s="201">
         <v>0.06</v>
@@ -10847,7 +10905,7 @@
       </c>
       <c r="J117" s="199"/>
       <c r="K117" s="190" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="L117" s="201">
         <v>0.06</v>
@@ -10912,7 +10970,7 @@
     </row>
     <row r="119" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B119" s="202" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="D119" s="203">
         <f>D118-0.005</f>
@@ -10956,7 +11014,7 @@
     </row>
     <row r="120" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B120" s="202" t="s">
-        <v>216</v>
+        <v>206</v>
       </c>
       <c r="E120" s="204"/>
       <c r="F120" s="204"/>
@@ -10968,7 +11026,7 @@
     <row r="121" spans="2:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B121" s="185"/>
       <c r="D121" s="186" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
       <c r="E121" s="177"/>
       <c r="F121" s="177"/>
@@ -10977,7 +11035,7 @@
       <c r="I121" s="177"/>
       <c r="J121" s="187"/>
       <c r="L121" s="186" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
       <c r="M121" s="177"/>
       <c r="N121" s="177"/>
@@ -10988,7 +11046,7 @@
     <row r="122" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B122" s="185"/>
       <c r="E122" s="188" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
       <c r="F122" s="188"/>
       <c r="G122" s="188"/>
@@ -10996,7 +11054,7 @@
       <c r="I122" s="188"/>
       <c r="J122" s="189"/>
       <c r="M122" s="188" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
       <c r="N122" s="188"/>
       <c r="O122" s="188"/>
@@ -11142,7 +11200,7 @@
     <row r="126" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B126" s="185"/>
       <c r="C126" s="190" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="D126" s="201">
         <v>0.06</v>
@@ -11164,7 +11222,7 @@
       </c>
       <c r="J126" s="199"/>
       <c r="K126" s="190" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="L126" s="201">
         <v>0.06</v>
@@ -11274,13 +11332,13 @@
     </row>
     <row r="130" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B130" s="211" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="C130" s="211"/>
       <c r="D130" s="211"/>
       <c r="E130" s="211"/>
       <c r="G130" s="211" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
       <c r="H130" s="211"/>
       <c r="I130" s="211"/>
@@ -11356,13 +11414,13 @@
     <row r="151" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B151" s="214"/>
       <c r="C151" s="215" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="D151" s="215" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="E151" s="216" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
       <c r="G151" s="214"/>
       <c r="H151" s="217"/>
@@ -11373,13 +11431,13 @@
       <c r="M151" s="217"/>
       <c r="N151" s="217"/>
       <c r="O151" s="215" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="P151" s="215" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="Q151" s="216" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
     </row>
     <row r="152" spans="2:17" x14ac:dyDescent="0.2">
@@ -11454,7 +11512,7 @@
     </row>
     <row r="154" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B154" s="225" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="C154" s="226">
         <v>169.5</v>
@@ -11531,16 +11589,16 @@
   <sheetData>
     <row r="2" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B2" s="368" t="s">
-        <v>280</v>
+        <v>269</v>
       </c>
       <c r="C2" s="368" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="D2" s="368" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="E2" s="368" t="s">
-        <v>281</v>
+        <v>270</v>
       </c>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.2">
@@ -11591,30 +11649,30 @@
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C2" s="346" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="D2" s="346" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="E2" s="346"/>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B3" s="232" t="s">
-        <v>224</v>
+        <v>214</v>
       </c>
       <c r="C3" s="347">
         <f>'Detail Data'!D3</f>
-        <v>0</v>
+        <v>32434.164000000004</v>
       </c>
       <c r="D3" s="233">
         <f>C3/C5</f>
-        <v>0</v>
+        <v>0.87387433408978565</v>
       </c>
       <c r="E3" s="351"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B4" s="232" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="C4" s="347">
         <f>'Detail Data'!D34</f>
@@ -11622,51 +11680,51 @@
       </c>
       <c r="D4" s="233">
         <f>C4/C5</f>
-        <v>1</v>
+        <v>0.12612566591021443</v>
       </c>
       <c r="E4" s="351"/>
       <c r="G4" s="234"/>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B5" s="232" t="s">
-        <v>226</v>
+        <v>216</v>
       </c>
       <c r="C5" s="347">
         <f>C3+C4</f>
-        <v>4681.2</v>
+        <v>37115.364000000001</v>
       </c>
       <c r="F5" s="235"/>
       <c r="G5" s="234"/>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C7" s="232" t="s">
-        <v>227</v>
+        <v>217</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C8" s="232" t="s">
-        <v>228</v>
+        <v>218</v>
       </c>
       <c r="D8" s="236"/>
       <c r="F8" s="357" t="s">
-        <v>265</v>
+        <v>254</v>
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C9" s="232" t="s">
-        <v>229</v>
+        <v>219</v>
       </c>
       <c r="D9" s="236"/>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C10" s="232" t="s">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="D10" s="348"/>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C11" s="232" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="D11" s="236"/>
     </row>
@@ -11675,14 +11733,14 @@
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C13" s="232" t="s">
-        <v>232</v>
+        <v>222</v>
       </c>
       <c r="D13" s="236"/>
       <c r="E13" s="361"/>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C14" s="232" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="D14" s="236"/>
       <c r="E14" s="362"/>
@@ -11692,7 +11750,7 @@
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C16" s="232" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="D16" s="236">
         <f>D3*D11+D4*D13*(1-D14)</f>
@@ -11701,54 +11759,54 @@
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B20" s="352" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="C20" s="233"/>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B21" s="357" t="s">
-        <v>266</v>
+        <v>255</v>
       </c>
       <c r="C21" s="358"/>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B22" s="357" t="s">
-        <v>267</v>
+        <v>256</v>
       </c>
       <c r="C22" s="234"/>
     </row>
     <row r="23" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B23" s="357" t="s">
-        <v>268</v>
+        <v>257</v>
       </c>
       <c r="C23" s="236"/>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B25" s="357" t="s">
-        <v>269</v>
+        <v>258</v>
       </c>
       <c r="C25" s="359"/>
     </row>
     <row r="27" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B27" s="357" t="s">
-        <v>270</v>
+        <v>259</v>
       </c>
     </row>
     <row r="28" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B28" s="357" t="s">
-        <v>271</v>
+        <v>260</v>
       </c>
       <c r="C28" s="360"/>
     </row>
     <row r="29" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B29" s="357" t="s">
-        <v>272</v>
+        <v>261</v>
       </c>
       <c r="C29" s="360"/>
     </row>
     <row r="30" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B30" s="357" t="s">
-        <v>273</v>
+        <v>262</v>
       </c>
       <c r="C30" s="359"/>
     </row>

</xml_diff>

<commit_message>
Workbook formula corrections (FCFE sign, forecast EPS, EV/EBITDA, 2025A cash flow block, FrontPage ratios); 22 vault notes confirmed; FactSet export removed from the repo and ignored
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/workbook/QD-HSY.xlsx
+++ b/workbook/QD-HSY.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chrislester/Documents/GitHub/HSY-valuation/workbook/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBEB0C49-7238-6143-BBD4-31006369D13E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8C3FD3C-5A73-F547-A142-491B6148EE3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="15740" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2894,62 +2894,62 @@
     <xf numFmtId="194" fontId="46" fillId="13" borderId="12" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="185" fontId="46" fillId="13" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="18" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="19" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="19" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -6535,21 +6535,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="393" t="s">
+      <c r="A1" s="379" t="s">
         <v>279</v>
       </c>
-      <c r="B1" s="393"/>
-      <c r="C1" s="393"/>
-      <c r="D1" s="393"/>
-      <c r="E1" s="393"/>
-      <c r="F1" s="393"/>
-      <c r="G1" s="393"/>
-      <c r="H1" s="394"/>
-      <c r="I1" s="394"/>
-      <c r="J1" s="394"/>
-      <c r="K1" s="394"/>
-      <c r="L1" s="394"/>
-      <c r="M1" s="394"/>
+      <c r="B1" s="379"/>
+      <c r="C1" s="379"/>
+      <c r="D1" s="379"/>
+      <c r="E1" s="379"/>
+      <c r="F1" s="379"/>
+      <c r="G1" s="379"/>
+      <c r="H1" s="380"/>
+      <c r="I1" s="380"/>
+      <c r="J1" s="380"/>
+      <c r="K1" s="380"/>
+      <c r="L1" s="380"/>
+      <c r="M1" s="380"/>
     </row>
     <row r="2" spans="1:18" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
@@ -6563,18 +6563,18 @@
       <c r="E2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="395" t="s">
+      <c r="F2" s="381" t="s">
         <v>281</v>
       </c>
-      <c r="G2" s="395"/>
-      <c r="H2" s="396" t="s">
+      <c r="G2" s="381"/>
+      <c r="H2" s="382" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="396"/>
-      <c r="J2" s="396"/>
-      <c r="K2" s="396"/>
-      <c r="L2" s="396"/>
-      <c r="M2" s="396"/>
+      <c r="I2" s="382"/>
+      <c r="J2" s="382"/>
+      <c r="K2" s="382"/>
+      <c r="L2" s="382"/>
+      <c r="M2" s="382"/>
     </row>
     <row r="3" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
@@ -6588,10 +6588,10 @@
       <c r="E3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="397" t="s">
+      <c r="F3" s="383" t="s">
         <v>282</v>
       </c>
-      <c r="G3" s="397"/>
+      <c r="G3" s="383"/>
       <c r="H3" s="11" t="s">
         <v>5</v>
       </c>
@@ -6618,10 +6618,10 @@
       <c r="E4" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="392" t="s">
+      <c r="F4" s="384" t="s">
         <v>284</v>
       </c>
-      <c r="G4" s="392"/>
+      <c r="G4" s="384"/>
       <c r="H4" s="19" t="s">
         <v>9</v>
       </c>
@@ -6653,15 +6653,15 @@
       <c r="G5" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="H5" s="380" t="s">
+      <c r="H5" s="385" t="s">
         <v>15</v>
       </c>
-      <c r="I5" s="380"/>
-      <c r="K5" s="390" t="s">
+      <c r="I5" s="385"/>
+      <c r="K5" s="386" t="s">
         <v>16</v>
       </c>
-      <c r="L5" s="390"/>
-      <c r="M5" s="390"/>
+      <c r="L5" s="386"/>
+      <c r="M5" s="386"/>
     </row>
     <row r="6" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="30" t="s">
@@ -6758,7 +6758,7 @@
       <c r="L8" s="37"/>
       <c r="M8" s="38">
         <f>'Detail Data'!D41</f>
-        <v>0</v>
+        <v>412.69999999999993</v>
       </c>
     </row>
     <row r="9" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -6794,21 +6794,21 @@
       <c r="L9" s="37"/>
       <c r="M9" s="43">
         <f>M8/'Detail Data'!E9</f>
-        <v>0</v>
+        <v>2.0290068829891834</v>
       </c>
     </row>
     <row r="10" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="389" t="s">
+      <c r="A10" s="387" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="389"/>
-      <c r="C10" s="389"/>
+      <c r="B10" s="387"/>
+      <c r="C10" s="387"/>
       <c r="D10" s="17"/>
-      <c r="E10" s="380" t="s">
+      <c r="E10" s="385" t="s">
         <v>30</v>
       </c>
-      <c r="F10" s="380"/>
-      <c r="G10" s="380"/>
+      <c r="F10" s="385"/>
+      <c r="G10" s="385"/>
       <c r="H10" s="35" t="s">
         <v>31</v>
       </c>
@@ -6826,17 +6826,17 @@
       </c>
     </row>
     <row r="11" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="385" t="s">
+      <c r="A11" s="388" t="s">
         <v>285</v>
       </c>
-      <c r="B11" s="385"/>
-      <c r="C11" s="385"/>
+      <c r="B11" s="388"/>
+      <c r="C11" s="388"/>
       <c r="D11" s="17"/>
-      <c r="E11" s="391" t="s">
+      <c r="E11" s="389" t="s">
         <v>286</v>
       </c>
-      <c r="F11" s="391"/>
-      <c r="G11" s="391"/>
+      <c r="F11" s="389"/>
+      <c r="G11" s="389"/>
       <c r="H11" s="51" t="s">
         <v>33</v>
       </c>
@@ -6848,23 +6848,23 @@
         <v>34</v>
       </c>
       <c r="L11" s="53"/>
-      <c r="M11" s="54" t="e">
+      <c r="M11" s="54">
         <f>'DCF 1-Pager'!C69/'Detail Data'!D41</f>
-        <v>#DIV/0!</v>
+        <v>9.0993457717470321</v>
       </c>
     </row>
     <row r="12" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="385"/>
-      <c r="B12" s="385"/>
-      <c r="C12" s="385"/>
+      <c r="A12" s="388"/>
+      <c r="B12" s="388"/>
+      <c r="C12" s="388"/>
       <c r="D12" s="17"/>
-      <c r="E12" s="391"/>
-      <c r="F12" s="391"/>
-      <c r="G12" s="391"/>
-      <c r="H12" s="380" t="s">
+      <c r="E12" s="389"/>
+      <c r="F12" s="389"/>
+      <c r="G12" s="389"/>
+      <c r="H12" s="385" t="s">
         <v>35</v>
       </c>
-      <c r="I12" s="380"/>
+      <c r="I12" s="385"/>
       <c r="K12" s="55" t="s">
         <v>36</v>
       </c>
@@ -6876,13 +6876,13 @@
       </c>
     </row>
     <row r="13" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="385"/>
-      <c r="B13" s="385"/>
-      <c r="C13" s="385"/>
+      <c r="A13" s="388"/>
+      <c r="B13" s="388"/>
+      <c r="C13" s="388"/>
       <c r="D13" s="17"/>
-      <c r="E13" s="391"/>
-      <c r="F13" s="391"/>
-      <c r="G13" s="391"/>
+      <c r="E13" s="389"/>
+      <c r="F13" s="389"/>
+      <c r="G13" s="389"/>
       <c r="H13" s="58" t="s">
         <v>38</v>
       </c>
@@ -6895,7 +6895,7 @@
       </c>
       <c r="L13" s="61">
         <f>'Detail Data'!E12</f>
-        <v>2.6376744602122559</v>
+        <v>18.961802981584331</v>
       </c>
       <c r="M13" s="62">
         <f>L13*'Detail Data'!E7</f>
@@ -6903,13 +6903,13 @@
       </c>
     </row>
     <row r="14" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="385"/>
-      <c r="B14" s="385"/>
-      <c r="C14" s="385"/>
+      <c r="A14" s="388"/>
+      <c r="B14" s="388"/>
+      <c r="C14" s="388"/>
       <c r="D14" s="17"/>
-      <c r="E14" s="391"/>
-      <c r="F14" s="391"/>
-      <c r="G14" s="391"/>
+      <c r="E14" s="389"/>
+      <c r="F14" s="389"/>
+      <c r="G14" s="389"/>
       <c r="H14" s="58" t="s">
         <v>40</v>
       </c>
@@ -6922,25 +6922,25 @@
       </c>
       <c r="L14" s="63">
         <f>'Detail Data'!F12</f>
-        <v>2.5734251596778672</v>
+        <v>16.308409090909095</v>
       </c>
       <c r="M14" s="64">
         <f>L13*'Detail Data'!F7</f>
-        <v>163.44115073394872</v>
+        <v>185.40429581993567</v>
       </c>
     </row>
     <row r="15" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="380" t="s">
+      <c r="A15" s="385" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="380"/>
-      <c r="C15" s="380"/>
+      <c r="B15" s="385"/>
+      <c r="C15" s="385"/>
       <c r="D15" s="17"/>
-      <c r="E15" s="380" t="s">
+      <c r="E15" s="385" t="s">
         <v>43</v>
       </c>
-      <c r="F15" s="380"/>
-      <c r="G15" s="380"/>
+      <c r="F15" s="385"/>
+      <c r="G15" s="385"/>
       <c r="H15" s="58" t="s">
         <v>44</v>
       </c>
@@ -6953,31 +6953,31 @@
       </c>
       <c r="L15" s="66">
         <f>'Detail Data'!G12</f>
-        <v>2.5080741422374131</v>
+        <v>15.383306772908368</v>
       </c>
       <c r="M15" s="67">
         <f>L13*'Detail Data'!G7</f>
-        <v>167.69981490668079</v>
+        <v>196.55391055247003</v>
       </c>
     </row>
     <row r="16" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="388" t="s">
+      <c r="A16" s="390" t="s">
         <v>287</v>
       </c>
-      <c r="B16" s="388"/>
-      <c r="C16" s="388"/>
+      <c r="B16" s="390"/>
+      <c r="C16" s="390"/>
       <c r="D16" s="17"/>
-      <c r="E16" s="386" t="s">
+      <c r="E16" s="391" t="s">
         <v>288</v>
       </c>
-      <c r="F16" s="386"/>
-      <c r="G16" s="386"/>
+      <c r="F16" s="391"/>
+      <c r="G16" s="391"/>
       <c r="H16" s="58" t="s">
         <v>46</v>
       </c>
       <c r="I16" s="59">
         <f>'Detail Data'!E7/'Detail Data'!D7-1</f>
-        <v>12.929670259958584</v>
+        <v>0.93768153374205343</v>
       </c>
       <c r="K16" s="60" t="s">
         <v>47</v>
@@ -6999,19 +6999,19 @@
       <c r="R16" s="72"/>
     </row>
     <row r="17" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="388"/>
-      <c r="B17" s="388"/>
-      <c r="C17" s="388"/>
+      <c r="A17" s="390"/>
+      <c r="B17" s="390"/>
+      <c r="C17" s="390"/>
       <c r="D17" s="17"/>
-      <c r="E17" s="386"/>
-      <c r="F17" s="386"/>
-      <c r="G17" s="386"/>
+      <c r="E17" s="391"/>
+      <c r="F17" s="391"/>
+      <c r="G17" s="391"/>
       <c r="H17" s="58" t="s">
         <v>49</v>
       </c>
       <c r="I17" s="59">
         <f>'Detail Data'!F7/'Detail Data'!E7-1</f>
-        <v>2.4966453868987104E-2</v>
+        <v>0.16270096463022488</v>
       </c>
       <c r="K17" s="58" t="s">
         <v>50</v>
@@ -7033,19 +7033,19 @@
       <c r="R17" s="72"/>
     </row>
     <row r="18" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="388"/>
-      <c r="B18" s="388"/>
-      <c r="C18" s="388"/>
+      <c r="A18" s="390"/>
+      <c r="B18" s="390"/>
+      <c r="C18" s="390"/>
       <c r="D18" s="17"/>
-      <c r="E18" s="386"/>
-      <c r="F18" s="386"/>
-      <c r="G18" s="386"/>
+      <c r="E18" s="391"/>
+      <c r="F18" s="391"/>
+      <c r="G18" s="391"/>
       <c r="H18" s="65" t="s">
         <v>52</v>
       </c>
       <c r="I18" s="54">
         <f>(('Detail Data'!G7/'Detail Data'!E7)^(1/2))-1</f>
-        <v>2.551120927708328E-2</v>
+        <v>0.1102351284025751</v>
       </c>
       <c r="K18" s="65" t="s">
         <v>53</v>
@@ -7067,31 +7067,31 @@
       <c r="R18" s="71"/>
     </row>
     <row r="19" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="389" t="s">
+      <c r="A19" s="387" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="389"/>
-      <c r="C19" s="389"/>
+      <c r="B19" s="387"/>
+      <c r="C19" s="387"/>
       <c r="D19" s="17"/>
-      <c r="E19" s="390" t="s">
+      <c r="E19" s="386" t="s">
         <v>56</v>
       </c>
-      <c r="F19" s="390"/>
-      <c r="G19" s="390"/>
-      <c r="H19" s="380" t="s">
+      <c r="F19" s="386"/>
+      <c r="G19" s="386"/>
+      <c r="H19" s="385" t="s">
         <v>57</v>
       </c>
-      <c r="I19" s="380"/>
+      <c r="I19" s="385"/>
       <c r="K19" s="60" t="s">
         <v>58</v>
       </c>
       <c r="L19" s="68">
         <f>'Detail Data'!E13</f>
-        <v>11.501963691476393</v>
+        <v>11.754592599914336</v>
       </c>
       <c r="M19" s="62">
         <f>(('Detail Data'!E13*'Detail Data'!E21)-'Detail Data'!E34+'Detail Data'!E28)/'Detail Data'!E9</f>
-        <v>155.69031465093411</v>
+        <v>159.46</v>
       </c>
       <c r="N19" s="73" t="s">
         <v>59</v>
@@ -7102,34 +7102,34 @@
       <c r="R19" s="74"/>
     </row>
     <row r="20" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="385" t="s">
+      <c r="A20" s="388" t="s">
         <v>289</v>
       </c>
-      <c r="B20" s="385"/>
-      <c r="C20" s="385"/>
+      <c r="B20" s="388"/>
+      <c r="C20" s="388"/>
       <c r="D20" s="17"/>
-      <c r="E20" s="381" t="s">
+      <c r="E20" s="392" t="s">
         <v>290</v>
       </c>
-      <c r="F20" s="381"/>
-      <c r="G20" s="381"/>
+      <c r="F20" s="392"/>
+      <c r="G20" s="392"/>
       <c r="H20" s="60" t="s">
         <v>60</v>
       </c>
       <c r="I20" s="75">
-        <f>'Detail Data'!E35/AVERAGE('Detail Data'!E30,'Detail Data'!D30)</f>
-        <v>0.34483455126494161</v>
+        <f>'Detail Data'!E17/AVERAGE('Detail Data'!E35,'Detail Data'!D35)</f>
+        <v>0.36327917595837317</v>
       </c>
       <c r="K20" s="58" t="s">
         <v>61</v>
       </c>
       <c r="L20" s="63">
         <f>'Detail Data'!F13</f>
-        <v>10.286289704755731</v>
+        <v>10.438347574989688</v>
       </c>
       <c r="M20" s="64">
         <f>(('Detail Data'!E13*'Detail Data'!F21)+'Detail Data'!F28-'Detail Data'!F34)/'Detail Data'!F9</f>
-        <v>177.20680617567641</v>
+        <v>181.42200769709575</v>
       </c>
       <c r="N20" s="73" t="s">
         <v>62</v>
@@ -7140,15 +7140,15 @@
       <c r="R20" s="74"/>
     </row>
     <row r="21" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="385"/>
-      <c r="B21" s="385"/>
-      <c r="C21" s="385"/>
+      <c r="A21" s="388"/>
+      <c r="B21" s="388"/>
+      <c r="C21" s="388"/>
       <c r="D21" s="17"/>
-      <c r="E21" s="383" t="s">
+      <c r="E21" s="393" t="s">
         <v>291</v>
       </c>
-      <c r="F21" s="383"/>
-      <c r="G21" s="383"/>
+      <c r="F21" s="393"/>
+      <c r="G21" s="393"/>
       <c r="H21" s="58" t="s">
         <v>63</v>
       </c>
@@ -7161,11 +7161,11 @@
       </c>
       <c r="L21" s="66">
         <f>'Detail Data'!G13</f>
-        <v>9.8220724776320978</v>
+        <v>9.8714095999099687</v>
       </c>
       <c r="M21" s="67">
         <f>(('Detail Data'!E13*'Detail Data'!G21)+'Detail Data'!G28-'Detail Data'!G34)/'Detail Data'!G9</f>
-        <v>187.95220920474625</v>
+        <v>192.36663234324251</v>
       </c>
       <c r="N21" s="76" t="s">
         <v>65</v>
@@ -7176,21 +7176,21 @@
       <c r="R21" s="78"/>
     </row>
     <row r="22" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="385"/>
-      <c r="B22" s="385"/>
-      <c r="C22" s="385"/>
+      <c r="A22" s="388"/>
+      <c r="B22" s="388"/>
+      <c r="C22" s="388"/>
       <c r="D22" s="17"/>
-      <c r="E22" s="386" t="s">
+      <c r="E22" s="391" t="s">
         <v>292</v>
       </c>
-      <c r="F22" s="386"/>
-      <c r="G22" s="386"/>
+      <c r="F22" s="391"/>
+      <c r="G22" s="391"/>
       <c r="H22" s="58" t="s">
         <v>66</v>
       </c>
       <c r="I22" s="59">
-        <f>'Detail Data'!E40/AVERAGE('Detail Data'!E30,'Detail Data'!D30,'Detail Data'!C30)</f>
-        <v>3.2514168398018267E-2</v>
+        <f>'Detail Data'!E5/AVERAGE('Detail Data'!E30,'Detail Data'!D30)</f>
+        <v>0.8870461611709457</v>
       </c>
       <c r="K22" s="60"/>
       <c r="L22" s="68"/>
@@ -7204,21 +7204,21 @@
       <c r="R22" s="71"/>
     </row>
     <row r="23" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="385"/>
-      <c r="B23" s="385"/>
-      <c r="C23" s="385"/>
+      <c r="A23" s="388"/>
+      <c r="B23" s="388"/>
+      <c r="C23" s="388"/>
       <c r="D23" s="17"/>
-      <c r="E23" s="387" t="s">
+      <c r="E23" s="394" t="s">
         <v>68</v>
       </c>
-      <c r="F23" s="387"/>
-      <c r="G23" s="387"/>
+      <c r="F23" s="394"/>
+      <c r="G23" s="394"/>
       <c r="H23" s="58" t="s">
         <v>69</v>
       </c>
       <c r="I23" s="59">
-        <f>'Detail Data'!E17/'Detail Data'!E35</f>
-        <v>0.35783021630894107</v>
+        <f>AVERAGE('Detail Data'!C5,'Detail Data'!D5,'Detail Data'!E5)/AVERAGE('Detail Data'!C30,'Detail Data'!D30,'Detail Data'!E30)</f>
+        <v>0.86525945686783134</v>
       </c>
       <c r="K23" s="58"/>
       <c r="L23" s="63"/>
@@ -7232,17 +7232,17 @@
       <c r="R23" s="74"/>
     </row>
     <row r="24" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="380" t="s">
+      <c r="A24" s="385" t="s">
         <v>71</v>
       </c>
-      <c r="B24" s="380"/>
-      <c r="C24" s="380"/>
+      <c r="B24" s="385"/>
+      <c r="C24" s="385"/>
       <c r="D24" s="17"/>
-      <c r="E24" s="381" t="s">
+      <c r="E24" s="392" t="s">
         <v>293</v>
       </c>
-      <c r="F24" s="381"/>
-      <c r="G24" s="381"/>
+      <c r="F24" s="392"/>
+      <c r="G24" s="392"/>
       <c r="H24" s="58" t="s">
         <v>72</v>
       </c>
@@ -7265,16 +7265,16 @@
       <c r="A25" s="79" t="s">
         <v>294</v>
       </c>
-      <c r="B25" s="382" t="s">
+      <c r="B25" s="396" t="s">
         <v>295</v>
       </c>
-      <c r="C25" s="382"/>
+      <c r="C25" s="396"/>
       <c r="D25" s="17"/>
-      <c r="E25" s="383" t="s">
+      <c r="E25" s="393" t="s">
         <v>296</v>
       </c>
-      <c r="F25" s="383"/>
-      <c r="G25" s="383"/>
+      <c r="F25" s="393"/>
+      <c r="G25" s="393"/>
       <c r="H25" s="58" t="s">
         <v>74</v>
       </c>
@@ -7287,29 +7287,29 @@
       <c r="A26" s="79" t="s">
         <v>297</v>
       </c>
-      <c r="B26" s="384" t="s">
+      <c r="B26" s="397" t="s">
         <v>298</v>
       </c>
-      <c r="C26" s="384"/>
+      <c r="C26" s="397"/>
       <c r="D26" s="17"/>
-      <c r="E26" s="383" t="s">
+      <c r="E26" s="393" t="s">
         <v>299</v>
       </c>
-      <c r="F26" s="383"/>
-      <c r="G26" s="383"/>
+      <c r="F26" s="393"/>
+      <c r="G26" s="393"/>
       <c r="H26" s="58"/>
       <c r="I26" s="59"/>
     </row>
     <row r="27" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="379" t="s">
+      <c r="A27" s="395" t="s">
         <v>75</v>
       </c>
-      <c r="B27" s="379"/>
-      <c r="C27" s="379"/>
-      <c r="D27" s="379"/>
-      <c r="E27" s="379"/>
-      <c r="F27" s="379"/>
-      <c r="G27" s="379"/>
+      <c r="B27" s="395"/>
+      <c r="C27" s="395"/>
+      <c r="D27" s="395"/>
+      <c r="E27" s="395"/>
+      <c r="F27" s="395"/>
+      <c r="G27" s="395"/>
       <c r="H27" s="65"/>
       <c r="I27" s="54"/>
     </row>
@@ -7321,15 +7321,15 @@
       <c r="E28" s="81"/>
       <c r="F28" s="81"/>
       <c r="G28" s="83"/>
-      <c r="H28" s="380" t="s">
+      <c r="H28" s="385" t="s">
         <v>76</v>
       </c>
-      <c r="I28" s="380"/>
-      <c r="K28" s="380" t="s">
+      <c r="I28" s="385"/>
+      <c r="K28" s="385" t="s">
         <v>77</v>
       </c>
-      <c r="L28" s="380"/>
-      <c r="M28" s="380"/>
+      <c r="L28" s="385"/>
+      <c r="M28" s="385"/>
     </row>
     <row r="29" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="80"/>
@@ -7352,7 +7352,7 @@
       <c r="L29" s="84"/>
       <c r="M29" s="85">
         <f>'Detail Data'!E12/(1+FrontPage!I16)</f>
-        <v>0.18935656128159478</v>
+        <v>9.7858201419534971</v>
       </c>
       <c r="N29" s="86"/>
     </row>
@@ -7395,7 +7395,7 @@
       </c>
       <c r="M31" s="87">
         <f>'Detail Data'!E13/(('Detail Data'!E21/'Detail Data'!D21))</f>
-        <v>7.3716252422193271</v>
+        <v>7.5335354767069846</v>
       </c>
     </row>
     <row r="32" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -7586,31 +7586,6 @@
     <row r="69" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="H1:M1"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="H2:M2"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="K5:M5"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="A11:C14"/>
-    <mergeCell ref="E11:G14"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="E15:G15"/>
-    <mergeCell ref="A16:C18"/>
-    <mergeCell ref="E16:G18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="A20:C23"/>
-    <mergeCell ref="E20:G20"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="E22:G22"/>
-    <mergeCell ref="E23:G23"/>
     <mergeCell ref="A27:G27"/>
     <mergeCell ref="H28:I28"/>
     <mergeCell ref="K28:M28"/>
@@ -7620,6 +7595,31 @@
     <mergeCell ref="E25:G25"/>
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="E26:G26"/>
+    <mergeCell ref="A20:C23"/>
+    <mergeCell ref="E20:G20"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="E23:G23"/>
+    <mergeCell ref="A16:C18"/>
+    <mergeCell ref="E16:G18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="A11:C14"/>
+    <mergeCell ref="E11:G14"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="K5:M5"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="H1:M1"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="H2:M2"/>
+    <mergeCell ref="F3:G3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.45" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
@@ -7791,16 +7791,16 @@
         <v>4.34</v>
       </c>
       <c r="E7" s="114">
-        <f>E5/E9</f>
-        <v>60.454768928220254</v>
+        <f>E17/E9</f>
+        <v>8.4095378564405117</v>
       </c>
       <c r="F7" s="114">
-        <f>F5/F9</f>
-        <v>61.964110127826942</v>
+        <f>F17/F9</f>
+        <v>9.7777777777777768</v>
       </c>
       <c r="G7" s="114">
-        <f t="shared" ref="G7" si="0">G5/G9</f>
-        <v>63.578662733529988</v>
+        <f>G17/G9</f>
+        <v>10.365781710914455</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -7819,12 +7819,12 @@
         <v>4.34</v>
       </c>
       <c r="F8" s="114">
-        <f t="shared" ref="F8:G8" si="1">E7</f>
-        <v>60.454768928220254</v>
+        <f t="shared" ref="F8:G8" si="0">E7</f>
+        <v>8.4095378564405117</v>
       </c>
       <c r="G8" s="114">
-        <f t="shared" si="1"/>
-        <v>61.964110127826942</v>
+        <f t="shared" si="0"/>
+        <v>9.7777777777777768</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
@@ -7843,11 +7843,11 @@
         <v>203.4</v>
       </c>
       <c r="F9" s="118">
-        <f t="shared" ref="F9:G9" si="2">E9</f>
+        <f t="shared" ref="F9:G9" si="1">E9</f>
         <v>203.4</v>
       </c>
       <c r="G9" s="120">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>203.4</v>
       </c>
     </row>
@@ -7857,23 +7857,23 @@
       </c>
       <c r="B10" s="122"/>
       <c r="C10" s="123" t="str">
-        <f t="shared" ref="C10:G10" si="3">C2</f>
+        <f t="shared" ref="C10:G10" si="2">C2</f>
         <v>2024A</v>
       </c>
       <c r="D10" s="123" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>2025A</v>
       </c>
       <c r="E10" s="123" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>2026F</v>
       </c>
       <c r="F10" s="123" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>2027F</v>
       </c>
       <c r="G10" s="29" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>2028F</v>
       </c>
     </row>
@@ -7895,11 +7895,11 @@
         <v>2.6376744602122559</v>
       </c>
       <c r="F11" s="126">
-        <f t="shared" ref="F11:G11" si="4">F3/F5</f>
+        <f t="shared" ref="F11:G11" si="3">F3/F5</f>
         <v>2.5734251596778677</v>
       </c>
       <c r="G11" s="126">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2.5080741422374131</v>
       </c>
     </row>
@@ -7918,15 +7918,15 @@
       </c>
       <c r="E12" s="129">
         <f>FrontPage!C3/E7</f>
-        <v>2.6376744602122559</v>
+        <v>18.961802981584331</v>
       </c>
       <c r="F12" s="129">
         <f>FrontPage!$C3/F7</f>
-        <v>2.5734251596778672</v>
+        <v>16.308409090909095</v>
       </c>
       <c r="G12" s="130">
         <f>FrontPage!$C3/G7</f>
-        <v>2.5080741422374131</v>
+        <v>15.383306772908368</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
@@ -7939,20 +7939,20 @@
         <v>10.409903086327718</v>
       </c>
       <c r="D13" s="129">
-        <f t="shared" ref="D13:G13" si="5">$C4/D21</f>
-        <v>17.946540201521696</v>
+        <f>D4/D21</f>
+        <v>18.60449516759202</v>
       </c>
       <c r="E13" s="129">
-        <f t="shared" si="5"/>
-        <v>11.501963691476393</v>
+        <f>E4/E21</f>
+        <v>11.754592599914336</v>
       </c>
       <c r="F13" s="129">
-        <f t="shared" si="5"/>
-        <v>10.286289704755731</v>
+        <f>F4/F21</f>
+        <v>10.438347574989688</v>
       </c>
       <c r="G13" s="129">
-        <f t="shared" si="5"/>
-        <v>9.8220724776320978</v>
+        <f>G4/G21</f>
+        <v>9.8714095999099687</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
@@ -8018,11 +8018,11 @@
         <v>2546.6904971403433</v>
       </c>
       <c r="F16" s="139">
-        <f t="shared" ref="F16:G16" si="6">F21-F38</f>
+        <f t="shared" ref="F16:G16" si="4">F21-F38</f>
         <v>2835.4752529696439</v>
       </c>
       <c r="G16" s="139">
-        <f t="shared" si="6"/>
+        <f t="shared" si="4"/>
         <v>2985.2383853937527</v>
       </c>
     </row>
@@ -8120,9 +8120,11 @@
       </c>
       <c r="B21" s="142"/>
       <c r="C21" s="353">
+        <f>C16+C38</f>
         <v>3353.5</v>
       </c>
       <c r="D21" s="353">
+        <f>D16+D38</f>
         <v>1945.2</v>
       </c>
       <c r="E21" s="353">
@@ -8406,7 +8408,7 @@
       </c>
       <c r="B33" s="132"/>
       <c r="C33" s="139">
-        <f t="shared" ref="C33:G33" si="7">C31-C32</f>
+        <f t="shared" ref="C33:G33" si="5">C31-C32</f>
         <v>-170</v>
       </c>
       <c r="D33" s="139">
@@ -8414,15 +8416,15 @@
         <v>577</v>
       </c>
       <c r="E33" s="139">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>861.5</v>
       </c>
       <c r="F33" s="139">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>1049.5</v>
       </c>
       <c r="G33" s="140">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>1345.5</v>
       </c>
     </row>
@@ -8498,17 +8500,20 @@
         <v>112</v>
       </c>
       <c r="C37" s="138"/>
-      <c r="D37" s="138"/>
+      <c r="D37" s="138">
+        <f>D16*(1-D20/D16)</f>
+        <v>1110.5999999999999</v>
+      </c>
       <c r="E37" s="139">
         <f>E16*(1-E20/E16)</f>
         <v>1948.9904971403432</v>
       </c>
       <c r="F37" s="139">
-        <f t="shared" ref="F37:G37" si="8">F16*(1-F20/F16)</f>
+        <f t="shared" ref="F37:G37" si="6">F16*(1-F20/F16)</f>
         <v>2145.6752529696437</v>
       </c>
       <c r="G37" s="139">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>2277.4383853937525</v>
       </c>
     </row>
@@ -8528,11 +8533,11 @@
         <v>488.40950285965675</v>
       </c>
       <c r="F38" s="139">
-        <f t="shared" ref="F38:G38" si="9">E38/E40*F40</f>
+        <f t="shared" ref="F38:G38" si="7">E38/E40*F40</f>
         <v>558.32474703035621</v>
       </c>
       <c r="G38" s="139">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>568.96161460624717</v>
       </c>
     </row>
@@ -8541,17 +8546,20 @@
         <v>114</v>
       </c>
       <c r="C39" s="138"/>
-      <c r="D39" s="138"/>
+      <c r="D39" s="138">
+        <f>D33-C33</f>
+        <v>747</v>
+      </c>
       <c r="E39" s="139">
         <f>E33-D33</f>
         <v>284.5</v>
       </c>
       <c r="F39" s="139">
-        <f t="shared" ref="F39:G39" si="10">F33-E33</f>
+        <f t="shared" ref="F39:G39" si="8">F33-E33</f>
         <v>188</v>
       </c>
       <c r="G39" s="139">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>296</v>
       </c>
     </row>
@@ -8583,17 +8591,20 @@
       <c r="B41" s="131" t="s">
         <v>225</v>
       </c>
-      <c r="D41" s="138"/>
+      <c r="D41" s="138">
+        <f>D37+D38-D39-D40</f>
+        <v>412.69999999999993</v>
+      </c>
       <c r="E41" s="139">
         <f>E37+E38-E39-E40</f>
         <v>1712.1000000000001</v>
       </c>
       <c r="F41" s="139">
-        <f t="shared" ref="F41:G41" si="11">F37+F38-F39-F40</f>
+        <f t="shared" ref="F41:G41" si="9">F37+F38-F39-F40</f>
         <v>2012.1</v>
       </c>
       <c r="G41" s="139">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>2036.8999999999996</v>
       </c>
     </row>
@@ -8604,17 +8615,20 @@
       <c r="B42" s="131" t="s">
         <v>226</v>
       </c>
-      <c r="D42" s="138"/>
+      <c r="D42" s="138">
+        <f>D41-D19*(1-'DCF 1-Pager'!D25)+'Detail Data'!D34-'Detail Data'!C34</f>
+        <v>1784.7523265028867</v>
+      </c>
       <c r="E42" s="139">
-        <f>E41+E19*(1-'DCF 1-Pager'!E25)+'Detail Data'!E34-'Detail Data'!D34</f>
+        <f>E41-E19*(1-'DCF 1-Pager'!E25)+'Detail Data'!E34-'Detail Data'!D34</f>
         <v>1724.6000000000004</v>
       </c>
       <c r="F42" s="139">
-        <f>F41+F19*(1-'DCF 1-Pager'!F25)+'Detail Data'!F34-'Detail Data'!E34</f>
+        <f>F41-F19*(1-'DCF 1-Pager'!F25)+'Detail Data'!F34-'Detail Data'!E34</f>
         <v>1945.4000000000005</v>
       </c>
       <c r="G42" s="139">
-        <f>G41+G19*(1-'DCF 1-Pager'!G25)+'Detail Data'!G34-'Detail Data'!F34</f>
+        <f>G41-G19*(1-'DCF 1-Pager'!G25)+'Detail Data'!G34-'Detail Data'!F34</f>
         <v>1970.1999999999998</v>
       </c>
     </row>
@@ -8628,15 +8642,15 @@
         <v>1.1678931280425675</v>
       </c>
       <c r="E44" s="349">
-        <f t="shared" ref="E44:G44" si="12">(E33+E40)/E17</f>
+        <f t="shared" ref="E44:G44" si="10">(E33+E40)/E17</f>
         <v>0.7613563285589009</v>
       </c>
       <c r="F44" s="349">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>0.78107401448109415</v>
       </c>
       <c r="G44" s="349">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>0.88171125023714658</v>
       </c>
     </row>
@@ -8653,15 +8667,15 @@
         <v>0.1443292942589795</v>
       </c>
       <c r="E45" s="349">
-        <f t="shared" ref="E45:G45" si="13">E34/E3</f>
+        <f t="shared" ref="E45:G45" si="11">E34/E3</f>
         <v>0.14471469034934889</v>
       </c>
       <c r="F45" s="349">
-        <f t="shared" si="13"/>
+        <f t="shared" si="11"/>
         <v>0.14265821681113777</v>
       </c>
       <c r="G45" s="349">
-        <f t="shared" si="13"/>
+        <f t="shared" si="11"/>
         <v>0.14060174327292665</v>
       </c>
     </row>
@@ -8674,15 +8688,15 @@
         <v>0.190497757073844</v>
       </c>
       <c r="E46" s="349">
-        <f t="shared" ref="E46:G46" si="14">E17/E35</f>
+        <f t="shared" ref="E46:G46" si="12">E17/E35</f>
         <v>0.35783021630894107</v>
       </c>
       <c r="F46" s="349">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0.39135739304970679</v>
       </c>
       <c r="G46" s="349">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0.38744533058914332</v>
       </c>
       <c r="J46" s="88" t="s">
@@ -8723,15 +8737,15 @@
         <v>0.22248102139406481</v>
       </c>
       <c r="E49" s="349">
-        <f t="shared" ref="E49:G49" si="15">E46*E44</f>
+        <f t="shared" ref="E49:G49" si="13">E46*E44</f>
         <v>0.2724362997364127</v>
       </c>
       <c r="F49" s="349">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.30567909008618993</v>
       </c>
       <c r="G49" s="349">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.34161490683229812</v>
       </c>
     </row>
@@ -8744,15 +8758,15 @@
         <v>0.14675391963316123</v>
       </c>
       <c r="E50" s="349">
-        <f t="shared" ref="E50:G50" si="16">E47*E44</f>
+        <f t="shared" ref="E50:G50" si="14">E47*E44</f>
         <v>0.1768182277736155</v>
       </c>
       <c r="F50" s="349">
-        <f t="shared" si="16"/>
+        <f t="shared" si="14"/>
         <v>0.20890645986359904</v>
       </c>
       <c r="G50" s="349">
-        <f t="shared" si="16"/>
+        <f t="shared" si="14"/>
         <v>0.24872642489732752</v>
       </c>
     </row>
@@ -8774,15 +8788,15 @@
         <v>0.15748216913845808</v>
       </c>
       <c r="E53" s="349">
-        <f t="shared" ref="E53:G54" si="17">$B$52/E46</f>
+        <f t="shared" ref="E53:G54" si="15">$B$52/E46</f>
         <v>8.3838643671441088E-2</v>
       </c>
       <c r="F53" s="349">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>7.6656275140788419E-2</v>
       </c>
       <c r="G53" s="349">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>7.7430278884462148E-2</v>
       </c>
     </row>
@@ -8795,15 +8809,15 @@
         <v>0.23874519964344409</v>
       </c>
       <c r="E54" s="349">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>0.12917610443426961</v>
       </c>
       <c r="F54" s="349">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>0.11216608835232948</v>
       </c>
       <c r="G54" s="349">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>0.10634711417587946</v>
       </c>
     </row>
@@ -8817,15 +8831,15 @@
         <v>7.5788643533123032</v>
       </c>
       <c r="E56" s="155" t="e">
-        <f t="shared" ref="E56:G56" si="18">E16/E19</f>
+        <f t="shared" ref="E56:G56" si="16">E16/E19</f>
         <v>#DIV/0!</v>
       </c>
       <c r="F56" s="155" t="e">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>#DIV/0!</v>
       </c>
       <c r="G56" s="155" t="e">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -10429,7 +10443,7 @@
       <c r="D89" s="179"/>
       <c r="E89" s="182">
         <f>C89*'Detail Data'!D42</f>
-        <v>0</v>
+        <v>431.31514557153093</v>
       </c>
       <c r="F89" s="182">
         <f>'Detail Data'!E42</f>
@@ -10449,7 +10463,7 @@
       <c r="C90" s="252"/>
       <c r="E90" s="253">
         <f>E89/(1+'WACC calculation'!$D$11)^((E88-$D$41)/365)</f>
-        <v>0</v>
+        <v>431.31514557153093</v>
       </c>
       <c r="F90" s="253">
         <f>F89/(1+'WACC calculation'!$D$11)^((F88-$D$41)/365)</f>

</xml_diff>

<commit_message>
Module 3 prep: Dr. Payne's workbook with the WACC tab filled (WACC 6.78%), converter reads WACC labels in column C, site data regenerated, Milestone 3 Cost of Capital Memo drafted
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/workbook/QD-HSY.xlsx
+++ b/workbook/QD-HSY.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://txst-my.sharepoint.com/personal/jp40_txstate_edu/Documents/Documents/classes/FIN 5370/Module 2 - Cash Flow Forecasting &amp; Fundamentals-Based Modeling/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://txst-my.sharepoint.com/personal/jp40_txstate_edu/Documents/Documents/classes/FIN 5370/Module 3 - Risk, Discount Rates &amp; the Cost of Capital/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="225" documentId="8_{366BB503-0842-44C7-BE75-DE9CE711263C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C31F04C7-90BE-4C71-99C6-5F4423FE3DF1}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="8_{1756F969-F916-4EB6-8583-6A06C6DAFBE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F07B3C0A-3BB8-44FA-AC98-2BAB12CA1E73}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -265,7 +265,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="379">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="388">
   <si>
     <t>Hershey Company</t>
   </si>
@@ -1408,6 +1408,33 @@
   </si>
   <si>
     <t>P/E ratio</t>
+  </si>
+  <si>
+    <t>https://pages.stern.nyu.edu/~adamodar/New_Home_Page/datafile/ctryprem.html</t>
+  </si>
+  <si>
+    <t>https://home.treasury.gov/resource-center/data-chart-center/interest-rates/TextView?type=daily_treasury_long_term_rate&amp;field_tdr_date_value=2026</t>
+  </si>
+  <si>
+    <t>FactSet</t>
+  </si>
+  <si>
+    <t>https://pages.stern.nyu.edu/~adamodar/New_Home_Page/datafile/Betas.html</t>
+  </si>
+  <si>
+    <t>levered beta</t>
+  </si>
+  <si>
+    <t>Adjust regresssion beta according to the (2/3)*calculated beta + (1/3)*(1)</t>
+  </si>
+  <si>
+    <t>Regression</t>
+  </si>
+  <si>
+    <t>Interest coverage ratio</t>
+  </si>
+  <si>
+    <t>https://pages.stern.nyu.edu/~adamodar/New_Home_Page/datafile/ratings.html</t>
   </si>
 </sst>
 </file>
@@ -1456,6 +1483,13 @@
       <sz val="10"/>
       <name val="Courier New"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1806,13 +1840,6 @@
     <font>
       <sz val="16"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2404,328 +2431,410 @@
   </borders>
   <cellStyleXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="32" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="33" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="44" fontId="32" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="32" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="33" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="33" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="432">
+  <cellXfs count="437">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="12" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="14" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="11" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="12" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="166" fontId="14" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="38" fontId="17" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="38" fontId="17" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="40" fontId="19" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="20" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="16" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="16" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="40" fontId="19" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="20" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="40" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="19" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="16" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="19" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="40" fontId="19" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="20" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="40" fontId="19" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="19" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="16" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="16" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="16" fillId="7" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="16" fillId="7" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="38" fontId="16" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="38" fontId="16" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="40" fontId="18" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="19" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="15" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="16" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="15" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="40" fontId="18" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="19" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="40" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="18" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="15" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="18" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="40" fontId="18" fillId="5" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="19" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="40" fontId="18" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="18" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="15" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="15" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="15" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="15" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="15" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="15" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="15" fillId="7" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="15" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="15" fillId="7" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="15" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="15" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="18" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="15" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="16" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="15" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="16" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="15" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="16" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="15" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="16" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="15" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="16" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="171" fontId="15" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="171" fontId="16" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="15" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="172" fontId="16" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="15" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="16" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="38" fontId="15" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="38" fontId="16" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="15" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="16" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="15" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="15" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="16" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="15" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="16" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="25" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="22" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="168" fontId="23" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="23" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="24" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="24" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="168" fontId="23" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="23" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="24" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="24" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="24" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="24" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="24" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="24" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="171" fontId="23" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="23" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="24" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="23" fillId="8" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="169" fontId="23" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="169" fontId="23" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="23" fillId="9" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="23" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="168" fontId="22" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="17" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="17" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="17" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="22" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="23" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="166" fontId="23" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2733,586 +2842,507 @@
     <xf numFmtId="166" fontId="23" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="23" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="166" fontId="23" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="173" fontId="23" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="27" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="27" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="27" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="27" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="27" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="27" fillId="8" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="173" fontId="23" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="171" fontId="22" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="173" fontId="23" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="22" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="23" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="23" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="22" fillId="8" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="173" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="169" fontId="22" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="169" fontId="22" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="22" fillId="9" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="16" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="16" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="16" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="22" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="22" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="22" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="22" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="26" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="26" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="26" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="26" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="26" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="26" fillId="8" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="173" fontId="22" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="173" fontId="22" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="22" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="173" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="168" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="173" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="38" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="173" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="38" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="173" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="173" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="174" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="17" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="35" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="174" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="17" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="36" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="175" fontId="37" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="38" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="7" fontId="36" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="36" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="3" applyBorder="1"/>
+    <xf numFmtId="177" fontId="38" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="7" fontId="37" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="18" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="176" fontId="37" fillId="0" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="41" fillId="0" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="38" fillId="0" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="38" fillId="10" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="39" fontId="7" fillId="0" borderId="20" xfId="2" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="38" fillId="11" borderId="21" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="38" fillId="11" borderId="22" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="36" fillId="11" borderId="22" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="38" fillId="11" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="181" fontId="7" fillId="0" borderId="23" xfId="2" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="38" fillId="11" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="190" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="190" fontId="7" fillId="0" borderId="19" xfId="2" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="181" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="36" fillId="11" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="10" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="38" fillId="11" borderId="25" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="191" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="191" fontId="7" fillId="0" borderId="19" xfId="2" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="187" fontId="7" fillId="0" borderId="23" xfId="2" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="181" fontId="38" fillId="11" borderId="22" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="181" fontId="36" fillId="11" borderId="22" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="181" fontId="38" fillId="11" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="19" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="12" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="34" fillId="12" borderId="19" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="192" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="2" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="39" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="39" fontId="7" fillId="0" borderId="29" xfId="2" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="39" fontId="38" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="39" fontId="38" fillId="0" borderId="29" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="2" applyBorder="1"/>
+    <xf numFmtId="39" fontId="7" fillId="0" borderId="20" xfId="2" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="39" fontId="7" fillId="0" borderId="23" xfId="2" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="2" applyBorder="1"/>
+    <xf numFmtId="39" fontId="38" fillId="0" borderId="20" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="39" fontId="38" fillId="0" borderId="23" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="4"/>
+    <xf numFmtId="193" fontId="6" fillId="0" borderId="0" xfId="4" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="6" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="37" fontId="6" fillId="0" borderId="0" xfId="4" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="6" fillId="0" borderId="0" xfId="4" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="2" applyBorder="1"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="32" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="37" fillId="0" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="41" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="176" fontId="41" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="38" fillId="0" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="176" fontId="43" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="176" fontId="43" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="33" xfId="2" applyBorder="1"/>
+    <xf numFmtId="177" fontId="36" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="176" fontId="7" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="180" fontId="7" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="181" fontId="36" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="38" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="176" fontId="34" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="176" fontId="34" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="177" fontId="42" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="177" fontId="42" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="182" fontId="42" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="181" fontId="42" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="175" fontId="7" fillId="0" borderId="10" xfId="2" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="37" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="187" fontId="34" fillId="0" borderId="12" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="2" applyBorder="1"/>
+    <xf numFmtId="176" fontId="38" fillId="0" borderId="12" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="38" fillId="0" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="188" fontId="7" fillId="0" borderId="12" xfId="2" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="177" fontId="7" fillId="0" borderId="12" xfId="2" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="181" fontId="42" fillId="0" borderId="12" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="34" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="177" fontId="49" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="176" fontId="37" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="37" fontId="38" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="176" fontId="36" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="37" fontId="36" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="176" fontId="37" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="38" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="181" fontId="36" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="177" fontId="7" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="175" fontId="7" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="183" fontId="36" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="183" fontId="36" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="184" fontId="36" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="37" fontId="37" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="184" fontId="37" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="185" fontId="34" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="186" fontId="36" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="37" fontId="34" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="180" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="187" fontId="34" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="10" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="188" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="189" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="10" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="178" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="34" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="175" fontId="36" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="14" fontId="37" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="7" fontId="35" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="14" fontId="35" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="41" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="37" fontId="42" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="3" applyBorder="1"/>
-    <xf numFmtId="177" fontId="37" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="7" fontId="36" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="7" fontId="37" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="18" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="176" fontId="36" fillId="0" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="176" fontId="40" fillId="0" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="41" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="176" fontId="37" fillId="0" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="187" fontId="51" fillId="13" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="51" fillId="13" borderId="37" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="37" xfId="2" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="38" xfId="2" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="187" fontId="51" fillId="13" borderId="38" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="51" fillId="13" borderId="39" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="187" fontId="51" fillId="13" borderId="40" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="187" fontId="51" fillId="13" borderId="41" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="51" fillId="13" borderId="40" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="51" fillId="13" borderId="41" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="4" applyFont="1"/>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" xfId="8" applyFont="1"/>
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="16" fillId="0" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="4" applyFont="1"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="4" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="23" fillId="14" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="23" fillId="14" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="23" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="23" fillId="14" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="195" fontId="51" fillId="13" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="195" fontId="51" fillId="13" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="195" fontId="51" fillId="13" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="187" fontId="51" fillId="13" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="195" fontId="51" fillId="13" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="195" fontId="51" fillId="13" borderId="12" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="187" fontId="51" fillId="13" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="37" fillId="10" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="39" fontId="6" fillId="0" borderId="20" xfId="2" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="167" fontId="37" fillId="11" borderId="21" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="37" fillId="11" borderId="22" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="35" fillId="11" borderId="22" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="37" fillId="11" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="181" fontId="6" fillId="0" borderId="23" xfId="2" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="167" fontId="37" fillId="11" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="190" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="190" fontId="6" fillId="0" borderId="19" xfId="2" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="181" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="167" fontId="35" fillId="11" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="10" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="37" fillId="11" borderId="25" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="191" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="191" fontId="6" fillId="0" borderId="19" xfId="2" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="187" fontId="6" fillId="0" borderId="23" xfId="2" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="181" fontId="37" fillId="11" borderId="22" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="181" fontId="35" fillId="11" borderId="22" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="181" fontId="37" fillId="11" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="33" fillId="12" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="33" fillId="12" borderId="19" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="192" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="2" quotePrefix="1" applyBorder="1"/>
-    <xf numFmtId="39" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="39" fontId="6" fillId="0" borderId="29" xfId="2" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="39" fontId="37" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="39" fontId="37" fillId="0" borderId="29" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="2" applyBorder="1"/>
-    <xf numFmtId="39" fontId="6" fillId="0" borderId="20" xfId="2" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="39" fontId="6" fillId="0" borderId="23" xfId="2" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="2" applyBorder="1"/>
-    <xf numFmtId="39" fontId="37" fillId="0" borderId="20" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="39" fontId="37" fillId="0" borderId="23" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="4"/>
-    <xf numFmtId="193" fontId="5" fillId="0" borderId="0" xfId="4" applyNumberFormat="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="6" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="37" fontId="5" fillId="0" borderId="0" xfId="4" applyNumberFormat="1"/>
-    <xf numFmtId="10" fontId="5" fillId="0" borderId="0" xfId="4" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="2" applyBorder="1"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="32" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="176" fontId="36" fillId="0" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="176" fontId="40" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="176" fontId="40" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="13" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="177" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="18" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="176" fontId="37" fillId="0" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="176" fontId="42" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="176" fontId="42" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="33" xfId="2" applyBorder="1"/>
-    <xf numFmtId="177" fontId="35" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="176" fontId="6" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="180" fontId="6" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="181" fontId="35" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="176" fontId="37" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="176" fontId="33" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="176" fontId="33" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="177" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="177" fontId="41" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="21" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="177" fontId="41" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="182" fontId="41" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="181" fontId="41" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="175" fontId="6" fillId="0" borderId="10" xfId="2" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="37" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="187" fontId="33" fillId="0" borderId="12" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="2" applyBorder="1"/>
-    <xf numFmtId="176" fontId="37" fillId="0" borderId="12" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="176" fontId="37" fillId="0" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="188" fontId="6" fillId="0" borderId="12" xfId="2" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="177" fontId="6" fillId="0" borderId="12" xfId="2" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="181" fontId="41" fillId="0" borderId="12" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="49" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="180" fontId="33" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="177" fontId="48" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="176" fontId="36" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="37" fontId="37" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="176" fontId="35" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="37" fontId="35" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="176" fontId="36" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="176" fontId="37" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="181" fontId="35" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="177" fontId="6" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="175" fontId="6" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="183" fontId="35" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="183" fontId="35" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="184" fontId="35" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="37" fontId="36" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="184" fontId="36" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="185" fontId="33" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="186" fontId="35" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="37" fontId="33" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="180" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="187" fontId="33" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="10" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="188" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="189" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="10" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="178" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="51" fillId="13" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="179" fontId="33" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="175" fontId="35" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="176" fontId="40" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="51" fillId="13" borderId="38" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="37" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="37" fontId="41" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="7" fontId="36" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="176" fontId="40" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="51" fillId="13" borderId="34" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" xfId="2" applyFill="1"/>
-    <xf numFmtId="187" fontId="50" fillId="13" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="50" fillId="13" borderId="37" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="37" xfId="2" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="38" xfId="2" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="187" fontId="50" fillId="13" borderId="38" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="50" fillId="13" borderId="39" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="187" fontId="50" fillId="13" borderId="40" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="187" fontId="50" fillId="13" borderId="41" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="50" fillId="13" borderId="40" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="50" fillId="13" borderId="41" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="4" applyFont="1"/>
-    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" xfId="8" applyFont="1"/>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="10" fontId="15" fillId="0" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="4" applyFont="1"/>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="4" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" xfId="4" applyFont="1"/>
-    <xf numFmtId="10" fontId="51" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="194" fontId="51" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="43" fontId="51" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="22" fillId="14" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="51" fillId="13" borderId="35" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="22" fillId="14" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="51" fillId="13" borderId="36" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="22" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="22" fillId="14" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="195" fontId="50" fillId="13" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="195" fontId="50" fillId="13" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="195" fontId="50" fillId="13" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="187" fontId="50" fillId="13" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="195" fontId="50" fillId="13" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="195" fontId="50" fillId="13" borderId="12" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="187" fontId="50" fillId="13" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="195" fontId="51" fillId="13" borderId="43" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="195" fontId="51" fillId="13" borderId="44" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="195" fontId="51" fillId="13" borderId="45" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="13" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="13" borderId="38" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="13" borderId="34" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="13" borderId="35" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="13" borderId="36" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="195" fontId="50" fillId="13" borderId="43" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="195" fontId="50" fillId="13" borderId="44" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="195" fontId="50" fillId="13" borderId="45" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="193" fontId="49" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="0" xfId="4" applyFont="1"/>
+    <xf numFmtId="10" fontId="49" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="194" fontId="49" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="49" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="4" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" xfId="4" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -6729,6 +6759,7 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="FrontPage"/>
@@ -7023,21 +7054,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="28.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="402" t="s">
+      <c r="A1" s="398" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="402"/>
-      <c r="C1" s="402"/>
-      <c r="D1" s="402"/>
-      <c r="E1" s="402"/>
-      <c r="F1" s="402"/>
-      <c r="G1" s="402"/>
-      <c r="H1" s="403"/>
-      <c r="I1" s="403"/>
-      <c r="J1" s="403"/>
-      <c r="K1" s="403"/>
-      <c r="L1" s="403"/>
-      <c r="M1" s="403"/>
+      <c r="B1" s="398"/>
+      <c r="C1" s="398"/>
+      <c r="D1" s="398"/>
+      <c r="E1" s="398"/>
+      <c r="F1" s="398"/>
+      <c r="G1" s="398"/>
+      <c r="H1" s="399"/>
+      <c r="I1" s="399"/>
+      <c r="J1" s="399"/>
+      <c r="K1" s="399"/>
+      <c r="L1" s="399"/>
+      <c r="M1" s="399"/>
     </row>
     <row r="2" spans="1:18" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -7051,18 +7082,18 @@
       <c r="E2" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="404" t="s">
+      <c r="F2" s="400" t="s">
         <v>343</v>
       </c>
-      <c r="G2" s="404"/>
-      <c r="H2" s="405" t="s">
+      <c r="G2" s="400"/>
+      <c r="H2" s="401" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="405"/>
-      <c r="J2" s="405"/>
-      <c r="K2" s="405"/>
-      <c r="L2" s="405"/>
-      <c r="M2" s="405"/>
+      <c r="I2" s="401"/>
+      <c r="J2" s="401"/>
+      <c r="K2" s="401"/>
+      <c r="L2" s="401"/>
+      <c r="M2" s="401"/>
     </row>
     <row r="3" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
@@ -7076,8 +7107,8 @@
       <c r="E3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="406"/>
-      <c r="G3" s="406"/>
+      <c r="F3" s="402"/>
+      <c r="G3" s="402"/>
       <c r="H3" s="11" t="s">
         <v>7</v>
       </c>
@@ -7104,8 +7135,8 @@
       <c r="E4" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="407"/>
-      <c r="G4" s="407"/>
+      <c r="F4" s="403"/>
+      <c r="G4" s="403"/>
       <c r="H4" s="19" t="s">
         <v>12</v>
       </c>
@@ -7137,15 +7168,15 @@
       <c r="G5" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="408" t="s">
+      <c r="H5" s="404" t="s">
         <v>18</v>
       </c>
-      <c r="I5" s="408"/>
-      <c r="K5" s="409" t="s">
+      <c r="I5" s="404"/>
+      <c r="K5" s="405" t="s">
         <v>19</v>
       </c>
-      <c r="L5" s="409"/>
-      <c r="M5" s="409"/>
+      <c r="L5" s="405"/>
+      <c r="M5" s="405"/>
     </row>
     <row r="6" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="30" t="s">
@@ -7282,17 +7313,17 @@
       </c>
     </row>
     <row r="10" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="410" t="s">
+      <c r="A10" s="406" t="s">
         <v>32</v>
       </c>
-      <c r="B10" s="410"/>
-      <c r="C10" s="410"/>
+      <c r="B10" s="406"/>
+      <c r="C10" s="406"/>
       <c r="D10" s="17"/>
-      <c r="E10" s="408" t="s">
+      <c r="E10" s="404" t="s">
         <v>33</v>
       </c>
-      <c r="F10" s="408"/>
-      <c r="G10" s="408"/>
+      <c r="F10" s="404"/>
+      <c r="G10" s="404"/>
       <c r="H10" s="35" t="s">
         <v>34</v>
       </c>
@@ -7310,15 +7341,15 @@
       </c>
     </row>
     <row r="11" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="411"/>
-      <c r="B11" s="411"/>
-      <c r="C11" s="411"/>
+      <c r="A11" s="407"/>
+      <c r="B11" s="407"/>
+      <c r="C11" s="407"/>
       <c r="D11" s="17"/>
-      <c r="E11" s="412" t="s">
+      <c r="E11" s="408" t="s">
         <v>36</v>
       </c>
-      <c r="F11" s="412"/>
-      <c r="G11" s="412"/>
+      <c r="F11" s="408"/>
+      <c r="G11" s="408"/>
       <c r="H11" s="51" t="s">
         <v>37</v>
       </c>
@@ -7336,17 +7367,17 @@
       </c>
     </row>
     <row r="12" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="411"/>
-      <c r="B12" s="411"/>
-      <c r="C12" s="411"/>
+      <c r="A12" s="407"/>
+      <c r="B12" s="407"/>
+      <c r="C12" s="407"/>
       <c r="D12" s="17"/>
-      <c r="E12" s="412"/>
-      <c r="F12" s="412"/>
-      <c r="G12" s="412"/>
-      <c r="H12" s="408" t="s">
+      <c r="E12" s="408"/>
+      <c r="F12" s="408"/>
+      <c r="G12" s="408"/>
+      <c r="H12" s="404" t="s">
         <v>39</v>
       </c>
-      <c r="I12" s="408"/>
+      <c r="I12" s="404"/>
       <c r="K12" s="55" t="s">
         <v>40</v>
       </c>
@@ -7358,13 +7389,13 @@
       </c>
     </row>
     <row r="13" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="411"/>
-      <c r="B13" s="411"/>
-      <c r="C13" s="411"/>
+      <c r="A13" s="407"/>
+      <c r="B13" s="407"/>
+      <c r="C13" s="407"/>
       <c r="D13" s="17"/>
-      <c r="E13" s="412"/>
-      <c r="F13" s="412"/>
-      <c r="G13" s="412"/>
+      <c r="E13" s="408"/>
+      <c r="F13" s="408"/>
+      <c r="G13" s="408"/>
       <c r="H13" s="58" t="s">
         <v>42</v>
       </c>
@@ -7385,13 +7416,13 @@
       </c>
     </row>
     <row r="14" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="411"/>
-      <c r="B14" s="411"/>
-      <c r="C14" s="411"/>
+      <c r="A14" s="407"/>
+      <c r="B14" s="407"/>
+      <c r="C14" s="407"/>
       <c r="D14" s="17"/>
-      <c r="E14" s="412"/>
-      <c r="F14" s="412"/>
-      <c r="G14" s="412"/>
+      <c r="E14" s="408"/>
+      <c r="F14" s="408"/>
+      <c r="G14" s="408"/>
       <c r="H14" s="58" t="s">
         <v>44</v>
       </c>
@@ -7412,17 +7443,17 @@
       </c>
     </row>
     <row r="15" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="408" t="s">
+      <c r="A15" s="404" t="s">
         <v>46</v>
       </c>
-      <c r="B15" s="408"/>
-      <c r="C15" s="408"/>
+      <c r="B15" s="404"/>
+      <c r="C15" s="404"/>
       <c r="D15" s="17"/>
-      <c r="E15" s="408" t="s">
+      <c r="E15" s="404" t="s">
         <v>47</v>
       </c>
-      <c r="F15" s="408"/>
-      <c r="G15" s="408"/>
+      <c r="F15" s="404"/>
+      <c r="G15" s="404"/>
       <c r="H15" s="58" t="s">
         <v>48</v>
       </c>
@@ -7443,15 +7474,15 @@
       </c>
     </row>
     <row r="16" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="413"/>
-      <c r="B16" s="413"/>
-      <c r="C16" s="413"/>
+      <c r="A16" s="409"/>
+      <c r="B16" s="409"/>
+      <c r="C16" s="409"/>
       <c r="D16" s="17"/>
-      <c r="E16" s="414" t="s">
+      <c r="E16" s="410" t="s">
         <v>50</v>
       </c>
-      <c r="F16" s="414"/>
-      <c r="G16" s="414"/>
+      <c r="F16" s="410"/>
+      <c r="G16" s="410"/>
       <c r="H16" s="58" t="s">
         <v>51</v>
       </c>
@@ -7479,13 +7510,13 @@
       <c r="R16" s="72"/>
     </row>
     <row r="17" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="413"/>
-      <c r="B17" s="413"/>
-      <c r="C17" s="413"/>
+      <c r="A17" s="409"/>
+      <c r="B17" s="409"/>
+      <c r="C17" s="409"/>
       <c r="D17" s="17"/>
-      <c r="E17" s="414"/>
-      <c r="F17" s="414"/>
-      <c r="G17" s="414"/>
+      <c r="E17" s="410"/>
+      <c r="F17" s="410"/>
+      <c r="G17" s="410"/>
       <c r="H17" s="58" t="s">
         <v>54</v>
       </c>
@@ -7513,13 +7544,13 @@
       <c r="R17" s="72"/>
     </row>
     <row r="18" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="413"/>
-      <c r="B18" s="413"/>
-      <c r="C18" s="413"/>
+      <c r="A18" s="409"/>
+      <c r="B18" s="409"/>
+      <c r="C18" s="409"/>
       <c r="D18" s="17"/>
-      <c r="E18" s="414"/>
-      <c r="F18" s="414"/>
-      <c r="G18" s="414"/>
+      <c r="E18" s="410"/>
+      <c r="F18" s="410"/>
+      <c r="G18" s="410"/>
       <c r="H18" s="65" t="s">
         <v>57</v>
       </c>
@@ -7547,21 +7578,21 @@
       <c r="R18" s="71"/>
     </row>
     <row r="19" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="410" t="s">
+      <c r="A19" s="406" t="s">
         <v>60</v>
       </c>
-      <c r="B19" s="410"/>
-      <c r="C19" s="410"/>
+      <c r="B19" s="406"/>
+      <c r="C19" s="406"/>
       <c r="D19" s="17"/>
-      <c r="E19" s="409" t="s">
+      <c r="E19" s="405" t="s">
         <v>61</v>
       </c>
-      <c r="F19" s="409"/>
-      <c r="G19" s="409"/>
-      <c r="H19" s="408" t="s">
+      <c r="F19" s="405"/>
+      <c r="G19" s="405"/>
+      <c r="H19" s="404" t="s">
         <v>62</v>
       </c>
-      <c r="I19" s="408"/>
+      <c r="I19" s="404"/>
       <c r="K19" s="60" t="s">
         <v>63</v>
       </c>
@@ -7582,17 +7613,17 @@
       <c r="R19" s="74"/>
     </row>
     <row r="20" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="411" t="s">
+      <c r="A20" s="407" t="s">
         <v>65</v>
       </c>
-      <c r="B20" s="411"/>
-      <c r="C20" s="411"/>
+      <c r="B20" s="407"/>
+      <c r="C20" s="407"/>
       <c r="D20" s="17"/>
-      <c r="E20" s="415" t="s">
+      <c r="E20" s="411" t="s">
         <v>66</v>
       </c>
-      <c r="F20" s="415"/>
-      <c r="G20" s="415"/>
+      <c r="F20" s="411"/>
+      <c r="G20" s="411"/>
       <c r="H20" s="60" t="s">
         <v>67</v>
       </c>
@@ -7617,15 +7648,15 @@
       <c r="R20" s="74"/>
     </row>
     <row r="21" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="411"/>
-      <c r="B21" s="411"/>
-      <c r="C21" s="411"/>
+      <c r="A21" s="407"/>
+      <c r="B21" s="407"/>
+      <c r="C21" s="407"/>
       <c r="D21" s="17"/>
-      <c r="E21" s="416" t="s">
+      <c r="E21" s="412" t="s">
         <v>70</v>
       </c>
-      <c r="F21" s="416"/>
-      <c r="G21" s="416"/>
+      <c r="F21" s="412"/>
+      <c r="G21" s="412"/>
       <c r="H21" s="58" t="s">
         <v>71</v>
       </c>
@@ -7650,15 +7681,15 @@
       <c r="R21" s="78"/>
     </row>
     <row r="22" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="411"/>
-      <c r="B22" s="411"/>
-      <c r="C22" s="411"/>
+      <c r="A22" s="407"/>
+      <c r="B22" s="407"/>
+      <c r="C22" s="407"/>
       <c r="D22" s="17"/>
-      <c r="E22" s="414" t="s">
+      <c r="E22" s="410" t="s">
         <v>74</v>
       </c>
-      <c r="F22" s="414"/>
-      <c r="G22" s="414"/>
+      <c r="F22" s="410"/>
+      <c r="G22" s="410"/>
       <c r="H22" s="58" t="s">
         <v>75</v>
       </c>
@@ -7683,15 +7714,15 @@
       <c r="R22" s="71"/>
     </row>
     <row r="23" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="411"/>
-      <c r="B23" s="411"/>
-      <c r="C23" s="411"/>
+      <c r="A23" s="407"/>
+      <c r="B23" s="407"/>
+      <c r="C23" s="407"/>
       <c r="D23" s="17"/>
-      <c r="E23" s="417" t="s">
+      <c r="E23" s="413" t="s">
         <v>78</v>
       </c>
-      <c r="F23" s="417"/>
-      <c r="G23" s="417"/>
+      <c r="F23" s="413"/>
+      <c r="G23" s="413"/>
       <c r="H23" s="58" t="s">
         <v>79</v>
       </c>
@@ -7716,17 +7747,17 @@
       <c r="R23" s="74"/>
     </row>
     <row r="24" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="408" t="s">
+      <c r="A24" s="404" t="s">
         <v>82</v>
       </c>
-      <c r="B24" s="408"/>
-      <c r="C24" s="408"/>
+      <c r="B24" s="404"/>
+      <c r="C24" s="404"/>
       <c r="D24" s="17"/>
-      <c r="E24" s="415" t="s">
+      <c r="E24" s="411" t="s">
         <v>66</v>
       </c>
-      <c r="F24" s="415"/>
-      <c r="G24" s="415"/>
+      <c r="F24" s="411"/>
+      <c r="G24" s="411"/>
       <c r="H24" s="58" t="s">
         <v>83</v>
       </c>
@@ -7754,16 +7785,16 @@
       <c r="A25" s="79" t="s">
         <v>86</v>
       </c>
-      <c r="B25" s="420" t="s">
+      <c r="B25" s="416" t="s">
         <v>87</v>
       </c>
-      <c r="C25" s="420"/>
+      <c r="C25" s="416"/>
       <c r="D25" s="17"/>
-      <c r="E25" s="416" t="s">
+      <c r="E25" s="412" t="s">
         <v>70</v>
       </c>
-      <c r="F25" s="416"/>
-      <c r="G25" s="416"/>
+      <c r="F25" s="412"/>
+      <c r="G25" s="412"/>
       <c r="H25" s="58" t="s">
         <v>88</v>
       </c>
@@ -7773,29 +7804,29 @@
       <c r="A26" s="79" t="s">
         <v>89</v>
       </c>
-      <c r="B26" s="421" t="s">
+      <c r="B26" s="417" t="s">
         <v>90</v>
       </c>
-      <c r="C26" s="421"/>
+      <c r="C26" s="417"/>
       <c r="D26" s="17"/>
-      <c r="E26" s="416" t="s">
+      <c r="E26" s="412" t="s">
         <v>74</v>
       </c>
-      <c r="F26" s="416"/>
-      <c r="G26" s="416"/>
+      <c r="F26" s="412"/>
+      <c r="G26" s="412"/>
       <c r="H26" s="58"/>
       <c r="I26" s="59"/>
     </row>
     <row r="27" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="418" t="s">
+      <c r="A27" s="414" t="s">
         <v>91</v>
       </c>
-      <c r="B27" s="418"/>
-      <c r="C27" s="418"/>
-      <c r="D27" s="418"/>
-      <c r="E27" s="418"/>
-      <c r="F27" s="418"/>
-      <c r="G27" s="418"/>
+      <c r="B27" s="414"/>
+      <c r="C27" s="414"/>
+      <c r="D27" s="414"/>
+      <c r="E27" s="414"/>
+      <c r="F27" s="414"/>
+      <c r="G27" s="414"/>
       <c r="H27" s="65"/>
       <c r="I27" s="54"/>
     </row>
@@ -7807,15 +7838,15 @@
       <c r="E28" s="81"/>
       <c r="F28" s="81"/>
       <c r="G28" s="83"/>
-      <c r="H28" s="408" t="s">
+      <c r="H28" s="404" t="s">
         <v>92</v>
       </c>
-      <c r="I28" s="408"/>
-      <c r="K28" s="408" t="s">
+      <c r="I28" s="404"/>
+      <c r="K28" s="404" t="s">
         <v>93</v>
       </c>
-      <c r="L28" s="408"/>
-      <c r="M28" s="408"/>
+      <c r="L28" s="404"/>
+      <c r="M28" s="404"/>
     </row>
     <row r="29" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="80"/>
@@ -7920,14 +7951,14 @@
       <c r="E33" s="81"/>
       <c r="F33" s="81"/>
       <c r="G33" s="83"/>
-      <c r="H33" s="419" t="s">
+      <c r="H33" s="415" t="s">
         <v>102</v>
       </c>
-      <c r="I33" s="419"/>
-      <c r="J33" s="419"/>
-      <c r="K33" s="419"/>
-      <c r="L33" s="419"/>
-      <c r="M33" s="419"/>
+      <c r="I33" s="415"/>
+      <c r="J33" s="415"/>
+      <c r="K33" s="415"/>
+      <c r="L33" s="415"/>
+      <c r="M33" s="415"/>
     </row>
     <row r="34" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="80"/>
@@ -8678,15 +8709,15 @@
       </c>
       <c r="E19" s="155">
         <f>'WACC calculation'!$D$13*'Detail Data'!E34</f>
-        <v>0</v>
+        <v>253.8382</v>
       </c>
       <c r="F19" s="155">
         <f>'WACC calculation'!$D$13*'Detail Data'!F34</f>
-        <v>0</v>
+        <v>231.33439999999999</v>
       </c>
       <c r="G19" s="155">
         <f>'WACC calculation'!$D$13*'Detail Data'!G34</f>
-        <v>0</v>
+        <v>202.41759999999999</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -8714,21 +8745,21 @@
         <v>134</v>
       </c>
       <c r="B21" s="158"/>
-      <c r="C21" s="388">
+      <c r="C21" s="384">
         <f>C16+C38</f>
         <v>3353.5</v>
       </c>
-      <c r="D21" s="388">
+      <c r="D21" s="384">
         <f>D16+D38</f>
         <v>1945.2</v>
       </c>
-      <c r="E21" s="388">
+      <c r="E21" s="384">
         <v>3035.1</v>
       </c>
-      <c r="F21" s="388">
+      <c r="F21" s="384">
         <v>3393.8</v>
       </c>
-      <c r="G21" s="389">
+      <c r="G21" s="385">
         <v>3554.2</v>
       </c>
     </row>
@@ -8939,19 +8970,19 @@
         <v>143</v>
       </c>
       <c r="B30" s="144"/>
-      <c r="C30" s="390">
+      <c r="C30" s="386">
         <v>12946.9</v>
       </c>
-      <c r="D30" s="390">
+      <c r="D30" s="386">
         <v>13741.3</v>
       </c>
-      <c r="E30" s="390">
+      <c r="E30" s="386">
         <v>13983.3</v>
       </c>
-      <c r="F30" s="390">
+      <c r="F30" s="386">
         <v>14093.3</v>
       </c>
-      <c r="G30" s="391">
+      <c r="G30" s="387">
         <v>14406</v>
       </c>
     </row>
@@ -9033,13 +9064,13 @@
       <c r="D34" s="154">
         <v>4681</v>
       </c>
-      <c r="E34" s="390">
+      <c r="E34" s="386">
         <v>4354</v>
       </c>
-      <c r="F34" s="390">
+      <c r="F34" s="386">
         <v>3968</v>
       </c>
-      <c r="G34" s="391">
+      <c r="G34" s="387">
         <v>3472</v>
       </c>
     </row>
@@ -9054,13 +9085,13 @@
       <c r="D35" s="172">
         <v>4636.8</v>
       </c>
-      <c r="E35" s="388">
+      <c r="E35" s="384">
         <v>4780</v>
       </c>
-      <c r="F35" s="388">
+      <c r="F35" s="384">
         <v>5092</v>
       </c>
-      <c r="G35" s="389">
+      <c r="G35" s="385">
         <v>5461</v>
       </c>
     </row>
@@ -9172,13 +9203,13 @@
       <c r="D40" s="154">
         <v>454.6</v>
       </c>
-      <c r="E40" s="390">
+      <c r="E40" s="386">
         <v>440.8</v>
       </c>
-      <c r="F40" s="390">
+      <c r="F40" s="386">
         <v>503.9</v>
       </c>
-      <c r="G40" s="390">
+      <c r="G40" s="386">
         <v>513.5</v>
       </c>
     </row>
@@ -9219,15 +9250,15 @@
       </c>
       <c r="E42" s="155">
         <f>E41+E19*(1-'DCF 1-Pager'!E25)+'Detail Data'!E34-'Detail Data'!D34</f>
-        <v>1385.1000000000004</v>
+        <v>1566.5943129999996</v>
       </c>
       <c r="F42" s="155">
         <f>F41+F19*(1-'DCF 1-Pager'!F25)+'Detail Data'!F34-'Detail Data'!E34</f>
-        <v>1626.1000000000004</v>
+        <v>1792.6607679999997</v>
       </c>
       <c r="G42" s="155">
         <f>G41+G19*(1-'DCF 1-Pager'!G25)+'Detail Data'!G34-'Detail Data'!F34</f>
-        <v>1540.8999999999996</v>
+        <v>1687.652759999999</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -9520,20 +9551,20 @@
       <c r="B3" s="194" t="s">
         <v>157</v>
       </c>
-      <c r="L3" s="425" t="s">
+      <c r="L3" s="421" t="s">
         <v>344</v>
       </c>
-      <c r="M3" s="426"/>
-      <c r="N3" s="427"/>
-      <c r="R3" s="428" t="s">
+      <c r="M3" s="422"/>
+      <c r="N3" s="423"/>
+      <c r="R3" s="424" t="s">
         <v>372</v>
       </c>
-      <c r="S3" s="429"/>
-      <c r="T3" s="429"/>
-      <c r="U3" s="429"/>
-      <c r="V3" s="429"/>
-      <c r="W3" s="429"/>
-      <c r="X3" s="430"/>
+      <c r="S3" s="425"/>
+      <c r="T3" s="425"/>
+      <c r="U3" s="425"/>
+      <c r="V3" s="425"/>
+      <c r="W3" s="425"/>
+      <c r="X3" s="426"/>
     </row>
     <row r="4" spans="2:24" ht="21" x14ac:dyDescent="0.35">
       <c r="B4" s="191" t="s">
@@ -9544,25 +9575,25 @@
         <v>Hershey Company</v>
       </c>
       <c r="L4" s="367"/>
-      <c r="M4" s="423" t="s">
+      <c r="M4" s="419" t="s">
         <v>348</v>
       </c>
-      <c r="N4" s="424"/>
-      <c r="R4" s="394"/>
-      <c r="S4" s="395"/>
-      <c r="T4" s="395" t="s">
+      <c r="N4" s="420"/>
+      <c r="R4" s="390"/>
+      <c r="S4" s="391"/>
+      <c r="T4" s="391" t="s">
         <v>373</v>
       </c>
-      <c r="U4" s="395" t="s">
+      <c r="U4" s="391" t="s">
         <v>374</v>
       </c>
-      <c r="V4" s="395" t="s">
+      <c r="V4" s="391" t="s">
         <v>375</v>
       </c>
-      <c r="W4" s="395" t="s">
+      <c r="W4" s="391" t="s">
         <v>376</v>
       </c>
-      <c r="X4" s="396" t="s">
+      <c r="X4" s="392" t="s">
         <v>377</v>
       </c>
     </row>
@@ -9581,21 +9612,21 @@
       <c r="N5" s="375" t="s">
         <v>347</v>
       </c>
-      <c r="R5" s="394" t="s">
+      <c r="R5" s="390" t="s">
         <v>378</v>
       </c>
-      <c r="S5" s="395" t="e">
+      <c r="S5" s="391" t="e">
         <f>AVERAGE('Relative Valuation'!D3:D6)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="T5" s="395">
+      <c r="T5" s="391">
         <f>AD21-AD24</f>
         <v>0</v>
       </c>
-      <c r="U5" s="395"/>
-      <c r="V5" s="395"/>
-      <c r="W5" s="395"/>
-      <c r="X5" s="397"/>
+      <c r="U5" s="391"/>
+      <c r="V5" s="391"/>
+      <c r="W5" s="391"/>
+      <c r="X5" s="393"/>
     </row>
     <row r="6" spans="2:24" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="191" t="s">
@@ -9609,26 +9640,26 @@
       </c>
       <c r="H6" s="196">
         <f>'WACC calculation'!D16</f>
-        <v>0</v>
+        <v>6.7806502134778832E-2</v>
       </c>
       <c r="L6" s="368"/>
       <c r="M6" s="365"/>
       <c r="N6" s="369"/>
-      <c r="R6" s="394" t="s">
+      <c r="R6" s="390" t="s">
         <v>128</v>
       </c>
-      <c r="S6" s="395" t="e">
+      <c r="S6" s="391" t="e">
         <f>AVERAGE('Relative Valuation'!C3:C6)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="T6" s="395">
+      <c r="T6" s="391">
         <f>AD19</f>
         <v>0</v>
       </c>
-      <c r="U6" s="395"/>
-      <c r="V6" s="395"/>
-      <c r="W6" s="395"/>
-      <c r="X6" s="397"/>
+      <c r="U6" s="391"/>
+      <c r="V6" s="391"/>
+      <c r="W6" s="391"/>
+      <c r="X6" s="393"/>
     </row>
     <row r="7" spans="2:24" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B7" s="191" t="s">
@@ -9656,21 +9687,21 @@
         <f>D77</f>
         <v>0</v>
       </c>
-      <c r="R7" s="398" t="s">
+      <c r="R7" s="394" t="s">
         <v>371</v>
       </c>
-      <c r="S7" s="395" t="e">
+      <c r="S7" s="391" t="e">
         <f>AVERAGE('Relative Valuation'!E3:E6)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="T7" s="399">
+      <c r="T7" s="395">
         <f>AD17</f>
         <v>0</v>
       </c>
-      <c r="U7" s="399"/>
-      <c r="V7" s="399"/>
-      <c r="W7" s="399"/>
-      <c r="X7" s="400"/>
+      <c r="U7" s="395"/>
+      <c r="V7" s="395"/>
+      <c r="W7" s="395"/>
+      <c r="X7" s="396"/>
     </row>
     <row r="8" spans="2:24" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B8" s="191" t="s">
@@ -9748,11 +9779,11 @@
       <c r="D14" s="205" t="s">
         <v>169</v>
       </c>
-      <c r="E14" s="422" t="s">
+      <c r="E14" s="418" t="s">
         <v>170</v>
       </c>
-      <c r="F14" s="422"/>
-      <c r="G14" s="422"/>
+      <c r="F14" s="418"/>
+      <c r="G14" s="418"/>
       <c r="H14" s="205"/>
       <c r="I14" s="205"/>
       <c r="J14" s="283"/>
@@ -10326,15 +10357,15 @@
       <c r="C43" s="280"/>
       <c r="E43" s="281">
         <f>E42/(1+$H$6)^((E41-$D$41)/365)</f>
-        <v>378.39837754191723</v>
+        <v>372.52711411569157</v>
       </c>
       <c r="F43" s="281">
         <f t="shared" ref="F43:G43" si="10">F42/(1+$H$6)^((F41-$D$41)/365)</f>
-        <v>1907.9669291685</v>
+        <v>1759.0853193860364</v>
       </c>
       <c r="G43" s="281">
         <f t="shared" si="10"/>
-        <v>1923.7594440167177</v>
+        <v>1660.7191873349771</v>
       </c>
       <c r="H43" s="281"/>
       <c r="I43" s="281"/>
@@ -10964,11 +10995,11 @@
       </c>
       <c r="F89" s="210">
         <f>'Detail Data'!E42</f>
-        <v>1385.1000000000004</v>
+        <v>1566.5943129999996</v>
       </c>
       <c r="G89" s="210">
         <f>'Detail Data'!F42</f>
-        <v>1626.1000000000004</v>
+        <v>1792.6607679999997</v>
       </c>
       <c r="H89" s="210"/>
       <c r="I89" s="279"/>
@@ -10984,11 +11015,11 @@
       </c>
       <c r="F90" s="281">
         <f>F89/(1+'WACC calculation'!G11)^((F88-$D$41)/365)</f>
-        <v>1385.1000000000004</v>
+        <v>1566.5943129999996</v>
       </c>
       <c r="G90" s="281">
         <f>G89/(1+'WACC calculation'!H11)^((G88-$D$41)/365)</f>
-        <v>1626.1000000000004</v>
+        <v>1792.6607679999997</v>
       </c>
       <c r="H90" s="281"/>
       <c r="I90" s="282"/>
@@ -11743,10 +11774,10 @@
       <c r="Q124" s="380" t="e">
         <v>#DIV/0!</v>
       </c>
-      <c r="AP124" s="401" t="e">
+      <c r="AP124" s="397" t="e">
         <v>#DIV/0!</v>
       </c>
-      <c r="AQ124" s="401" t="e">
+      <c r="AQ124" s="397" t="e">
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -11791,10 +11822,10 @@
       <c r="Q125" s="380" t="e">
         <v>#DIV/0!</v>
       </c>
-      <c r="AP125" s="401" t="e">
+      <c r="AP125" s="397" t="e">
         <v>#DIV/0!</v>
       </c>
-      <c r="AQ125" s="401" t="e">
+      <c r="AQ125" s="397" t="e">
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -11843,10 +11874,10 @@
       <c r="Q126" s="380" t="e">
         <v>#DIV/0!</v>
       </c>
-      <c r="AP126" s="401" t="e">
+      <c r="AP126" s="397" t="e">
         <v>#DIV/0!</v>
       </c>
-      <c r="AQ126" s="401" t="e">
+      <c r="AQ126" s="397" t="e">
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -11891,10 +11922,10 @@
       <c r="Q127" s="380" t="e">
         <v>#DIV/0!</v>
       </c>
-      <c r="AP127" s="401" t="e">
+      <c r="AP127" s="397" t="e">
         <v>#DIV/0!</v>
       </c>
-      <c r="AQ127" s="401" t="e">
+      <c r="AQ127" s="397" t="e">
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -11939,10 +11970,10 @@
       <c r="Q128" s="380" t="e">
         <v>#DIV/0!</v>
       </c>
-      <c r="AP128" s="401" t="e">
+      <c r="AP128" s="397" t="e">
         <v>#DIV/0!</v>
       </c>
-      <c r="AQ128" s="401" t="e">
+      <c r="AQ128" s="397" t="e">
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -12225,7 +12256,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19EC1B7B-724F-4C3D-BB7E-936BBF56ABA0}">
-  <dimension ref="B2:H29"/>
+  <dimension ref="B2:H31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" style="260"/>
@@ -12315,48 +12346,75 @@
       <c r="D7" s="382" t="s">
         <v>366</v>
       </c>
-      <c r="E7" s="431" t="s">
+      <c r="E7" s="434" t="s">
         <v>369</v>
       </c>
-      <c r="F7" s="431"/>
-      <c r="G7" s="431"/>
-      <c r="H7" s="431"/>
+      <c r="F7" s="427" t="s">
+        <v>381</v>
+      </c>
+      <c r="G7" s="435" t="s">
+        <v>385</v>
+      </c>
+      <c r="H7" s="434"/>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C8" s="260" t="s">
         <v>256</v>
       </c>
-      <c r="D8" s="264"/>
+      <c r="D8" s="264">
+        <v>4.4600000000000001E-2</v>
+      </c>
       <c r="E8" s="264"/>
       <c r="F8" s="264"/>
       <c r="G8" s="264"/>
-      <c r="H8" s="264"/>
+      <c r="H8" s="264" t="s">
+        <v>379</v>
+      </c>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C9" s="260" t="s">
         <v>257</v>
       </c>
-      <c r="D9" s="264"/>
+      <c r="D9" s="264">
+        <v>5.28E-2</v>
+      </c>
       <c r="E9" s="264"/>
       <c r="F9" s="264"/>
       <c r="G9" s="264"/>
-      <c r="H9" s="264"/>
+      <c r="H9" s="264" t="s">
+        <v>380</v>
+      </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C10" s="260" t="s">
         <v>258</v>
       </c>
-      <c r="D10" s="378"/>
-      <c r="E10" s="378"/>
-      <c r="F10" s="378"/>
-      <c r="G10" s="378"/>
-      <c r="H10" s="378"/>
+      <c r="D10" s="436">
+        <f>(2/3)*G10+1/3</f>
+        <v>0.41020000000000001</v>
+      </c>
+      <c r="E10" s="378">
+        <f>C29</f>
+        <v>0.34661866709107808</v>
+      </c>
+      <c r="F10" s="260">
+        <v>0.34</v>
+      </c>
+      <c r="G10" s="378">
+        <v>0.1153</v>
+      </c>
+      <c r="H10" s="433" t="s">
+        <v>384</v>
+      </c>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C11" s="260" t="s">
         <v>259</v>
       </c>
-      <c r="D11" s="264"/>
+      <c r="D11" s="264">
+        <f>D10*D8+D9</f>
+        <v>7.1094920000000006E-2</v>
+      </c>
       <c r="E11" s="264"/>
       <c r="F11" s="264"/>
       <c r="G11" s="264"/>
@@ -12369,17 +12427,25 @@
       <c r="C13" s="260" t="s">
         <v>260</v>
       </c>
-      <c r="D13" s="264"/>
+      <c r="D13" s="264">
+        <f>0.55%+D9</f>
+        <v>5.8299999999999998E-2</v>
+      </c>
       <c r="E13" s="264"/>
       <c r="F13" s="264"/>
       <c r="G13" s="264"/>
-      <c r="H13" s="264"/>
+      <c r="H13" s="264" t="s">
+        <v>387</v>
+      </c>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C14" s="260" t="s">
         <v>177</v>
       </c>
-      <c r="D14" s="264"/>
+      <c r="D14" s="264">
+        <f>'Detail Data'!D20/'Detail Data'!D16</f>
+        <v>0.2295525494276795</v>
+      </c>
       <c r="E14" s="264"/>
       <c r="F14" s="264"/>
       <c r="G14" s="264"/>
@@ -12396,73 +12462,106 @@
       <c r="C16" s="260" t="s">
         <v>261</v>
       </c>
-      <c r="D16" s="264"/>
+      <c r="D16" s="264">
+        <f>D13*(1-D14)*D4+D11*D3</f>
+        <v>6.7806502134778832E-2</v>
+      </c>
       <c r="E16" s="264"/>
       <c r="F16" s="264"/>
       <c r="G16" s="264"/>
       <c r="H16" s="264"/>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B20" s="382" t="s">
         <v>354</v>
       </c>
-      <c r="C20" s="261"/>
-    </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C20" s="428"/>
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B21" s="382" t="s">
         <v>363</v>
       </c>
-      <c r="C21" s="384"/>
-    </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C21" s="429">
+        <v>0.61</v>
+      </c>
+      <c r="D21" s="260" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B22" s="382" t="s">
         <v>364</v>
       </c>
-      <c r="C22" s="385"/>
-    </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C22" s="430">
+        <v>0.43730000000000002</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B23" s="382" t="s">
         <v>355</v>
       </c>
-      <c r="C23" s="385"/>
-    </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C23" s="430">
+        <v>0.1037</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B24" s="382" t="s">
         <v>365</v>
       </c>
-      <c r="C24" s="386"/>
-    </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C25" s="384"/>
-    </row>
-    <row r="26" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C24" s="431">
+        <f>C21/(1+(1-C23*C22))</f>
+        <v>0.31207601308097815</v>
+      </c>
+    </row>
+    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C25" s="429"/>
+    </row>
+    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B26" s="382" t="s">
         <v>367</v>
       </c>
-      <c r="C26" s="387"/>
-    </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C26" s="432"/>
+    </row>
+    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B27" s="382" t="s">
         <v>368</v>
       </c>
-      <c r="C27" s="385"/>
-    </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C27" s="430">
+        <f>C4/C3</f>
+        <v>0.14366543466113832</v>
+      </c>
+    </row>
+    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B28" s="382" t="s">
         <v>355</v>
       </c>
-      <c r="C28" s="385"/>
-    </row>
-    <row r="29" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B29" s="382" t="s">
-        <v>365</v>
-      </c>
-      <c r="C29" s="386"/>
+      <c r="C28" s="430">
+        <f>'Detail Data'!D20/'Detail Data'!D16</f>
+        <v>0.2295525494276795</v>
+      </c>
+    </row>
+    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B29" s="433" t="s">
+        <v>383</v>
+      </c>
+      <c r="C29" s="431">
+        <f>C24*(1+(1-C28)*C27)</f>
+        <v>0.34661866709107808</v>
+      </c>
+    </row>
+    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C30" s="429"/>
+    </row>
+    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B31" s="433" t="s">
+        <v>386</v>
+      </c>
+      <c r="C31" s="429">
+        <f>'Detail Data'!D16/'Detail Data'!D19</f>
+        <v>7.5788643533123032</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="E7:H7"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -12478,42 +12577,42 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B2" s="392" t="s">
+      <c r="B2" s="388" t="s">
         <v>370</v>
       </c>
-      <c r="C2" s="392" t="s">
+      <c r="C2" s="388" t="s">
         <v>128</v>
       </c>
-      <c r="D2" s="392" t="s">
+      <c r="D2" s="388" t="s">
         <v>127</v>
       </c>
-      <c r="E2" s="392" t="s">
+      <c r="E2" s="388" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B3" s="393"/>
-      <c r="C3" s="393"/>
-      <c r="D3" s="393"/>
-      <c r="E3" s="393"/>
+      <c r="B3" s="389"/>
+      <c r="C3" s="389"/>
+      <c r="D3" s="389"/>
+      <c r="E3" s="389"/>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B4" s="393"/>
-      <c r="C4" s="393"/>
-      <c r="D4" s="393"/>
-      <c r="E4" s="393"/>
+      <c r="B4" s="389"/>
+      <c r="C4" s="389"/>
+      <c r="D4" s="389"/>
+      <c r="E4" s="389"/>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B5" s="393"/>
-      <c r="C5" s="393"/>
-      <c r="D5" s="393"/>
-      <c r="E5" s="393"/>
+      <c r="B5" s="389"/>
+      <c r="C5" s="389"/>
+      <c r="D5" s="389"/>
+      <c r="E5" s="389"/>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B6" s="393"/>
-      <c r="C6" s="393"/>
-      <c r="D6" s="393"/>
-      <c r="E6" s="393"/>
+      <c r="B6" s="389"/>
+      <c r="C6" s="389"/>
+      <c r="D6" s="389"/>
+      <c r="E6" s="389"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Workbook is Dr. Payne's completed Module 4 Hershey workbook (DCF $218.59 perpetuity, $193.02 at a 13.02x exit multiple) with the FrontPage Capital Allocation and #REF! fixes carried over
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/workbook/QD-HSY.xlsx
+++ b/workbook/QD-HSY.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chrislester/Documents/GitHub/HSY-valuation/workbook/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D54BAC2-FB28-2A4B-892C-3C4A9D521137}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87BD3D59-ADD7-4C49-ABD7-1D7E8AEC1A9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15720" tabRatio="500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -212,7 +212,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="389">
   <si>
     <t>Hershey Company</t>
   </si>
@@ -1385,9 +1385,6 @@
   </si>
   <si>
     <t>short term and gross fixed assets, over and above debt already outstanding.</t>
-  </si>
-  <si>
-    <t>Midyear adjustment?</t>
   </si>
 </sst>
 </file>
@@ -3199,65 +3196,65 @@
     <xf numFmtId="195" fontId="47" fillId="13" borderId="45" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="14" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="17" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="15" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="15" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="10">
@@ -4150,7 +4147,7 @@
                   <c:v>218.58988139319837</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>205.78865016103435</c:v>
+                  <c:v>204.50280102213321</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4265,10 +4262,10 @@
                 <c:formatCode>"$"#,##0.00_);\("$"#,##0.00\);@_)</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>200.13228565680652</c:v>
+                  <c:v>193.02286141537462</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>245.16759035878044</c:v>
+                  <c:v>228.14877997561089</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6894,21 +6891,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="425" t="s">
+      <c r="A1" s="410" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="425"/>
-      <c r="C1" s="425"/>
-      <c r="D1" s="425"/>
-      <c r="E1" s="425"/>
-      <c r="F1" s="425"/>
-      <c r="G1" s="425"/>
-      <c r="H1" s="426"/>
-      <c r="I1" s="426"/>
-      <c r="J1" s="426"/>
-      <c r="K1" s="426"/>
-      <c r="L1" s="426"/>
-      <c r="M1" s="426"/>
+      <c r="B1" s="410"/>
+      <c r="C1" s="410"/>
+      <c r="D1" s="410"/>
+      <c r="E1" s="410"/>
+      <c r="F1" s="410"/>
+      <c r="G1" s="410"/>
+      <c r="H1" s="411"/>
+      <c r="I1" s="411"/>
+      <c r="J1" s="411"/>
+      <c r="K1" s="411"/>
+      <c r="L1" s="411"/>
+      <c r="M1" s="411"/>
     </row>
     <row r="2" spans="1:18" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
@@ -6922,18 +6919,18 @@
       <c r="E2" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="427" t="s">
+      <c r="F2" s="412" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="427"/>
-      <c r="H2" s="428" t="s">
+      <c r="G2" s="412"/>
+      <c r="H2" s="413" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="428"/>
-      <c r="J2" s="428"/>
-      <c r="K2" s="428"/>
-      <c r="L2" s="428"/>
-      <c r="M2" s="428"/>
+      <c r="I2" s="413"/>
+      <c r="J2" s="413"/>
+      <c r="K2" s="413"/>
+      <c r="L2" s="413"/>
+      <c r="M2" s="413"/>
     </row>
     <row r="3" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
@@ -6947,8 +6944,8 @@
       <c r="E3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="429"/>
-      <c r="G3" s="429"/>
+      <c r="F3" s="414"/>
+      <c r="G3" s="414"/>
       <c r="H3" s="11" t="s">
         <v>8</v>
       </c>
@@ -6975,8 +6972,8 @@
       <c r="E4" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="424"/>
-      <c r="G4" s="424"/>
+      <c r="F4" s="415"/>
+      <c r="G4" s="415"/>
       <c r="H4" s="19" t="s">
         <v>13</v>
       </c>
@@ -7008,15 +7005,15 @@
       <c r="G5" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="H5" s="411" t="s">
+      <c r="H5" s="416" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="411"/>
-      <c r="K5" s="422" t="s">
+      <c r="I5" s="416"/>
+      <c r="K5" s="417" t="s">
         <v>20</v>
       </c>
-      <c r="L5" s="422"/>
-      <c r="M5" s="422"/>
+      <c r="L5" s="417"/>
+      <c r="M5" s="417"/>
     </row>
     <row r="6" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="30" t="s">
@@ -7153,17 +7150,17 @@
       </c>
     </row>
     <row r="10" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="421" t="s">
+      <c r="A10" s="418" t="s">
         <v>33</v>
       </c>
-      <c r="B10" s="421"/>
-      <c r="C10" s="421"/>
+      <c r="B10" s="418"/>
+      <c r="C10" s="418"/>
       <c r="D10" s="17"/>
-      <c r="E10" s="411" t="s">
+      <c r="E10" s="416" t="s">
         <v>34</v>
       </c>
-      <c r="F10" s="411"/>
-      <c r="G10" s="411"/>
+      <c r="F10" s="416"/>
+      <c r="G10" s="416"/>
       <c r="H10" s="35" t="s">
         <v>35</v>
       </c>
@@ -7181,15 +7178,15 @@
       </c>
     </row>
     <row r="11" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="417"/>
-      <c r="B11" s="417"/>
-      <c r="C11" s="417"/>
+      <c r="A11" s="419"/>
+      <c r="B11" s="419"/>
+      <c r="C11" s="419"/>
       <c r="D11" s="17"/>
-      <c r="E11" s="423" t="s">
+      <c r="E11" s="420" t="s">
         <v>37</v>
       </c>
-      <c r="F11" s="423"/>
-      <c r="G11" s="423"/>
+      <c r="F11" s="420"/>
+      <c r="G11" s="420"/>
       <c r="H11" s="51" t="s">
         <v>38</v>
       </c>
@@ -7207,17 +7204,17 @@
       </c>
     </row>
     <row r="12" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="417"/>
-      <c r="B12" s="417"/>
-      <c r="C12" s="417"/>
+      <c r="A12" s="419"/>
+      <c r="B12" s="419"/>
+      <c r="C12" s="419"/>
       <c r="D12" s="17"/>
-      <c r="E12" s="423"/>
-      <c r="F12" s="423"/>
-      <c r="G12" s="423"/>
-      <c r="H12" s="411" t="s">
+      <c r="E12" s="420"/>
+      <c r="F12" s="420"/>
+      <c r="G12" s="420"/>
+      <c r="H12" s="416" t="s">
         <v>40</v>
       </c>
-      <c r="I12" s="411"/>
+      <c r="I12" s="416"/>
       <c r="K12" s="55" t="s">
         <v>41</v>
       </c>
@@ -7229,13 +7226,13 @@
       </c>
     </row>
     <row r="13" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="417"/>
-      <c r="B13" s="417"/>
-      <c r="C13" s="417"/>
+      <c r="A13" s="419"/>
+      <c r="B13" s="419"/>
+      <c r="C13" s="419"/>
       <c r="D13" s="17"/>
-      <c r="E13" s="423"/>
-      <c r="F13" s="423"/>
-      <c r="G13" s="423"/>
+      <c r="E13" s="420"/>
+      <c r="F13" s="420"/>
+      <c r="G13" s="420"/>
       <c r="H13" s="58" t="s">
         <v>43</v>
       </c>
@@ -7256,13 +7253,13 @@
       </c>
     </row>
     <row r="14" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="417"/>
-      <c r="B14" s="417"/>
-      <c r="C14" s="417"/>
+      <c r="A14" s="419"/>
+      <c r="B14" s="419"/>
+      <c r="C14" s="419"/>
       <c r="D14" s="17"/>
-      <c r="E14" s="423"/>
-      <c r="F14" s="423"/>
-      <c r="G14" s="423"/>
+      <c r="E14" s="420"/>
+      <c r="F14" s="420"/>
+      <c r="G14" s="420"/>
       <c r="H14" s="58" t="s">
         <v>45</v>
       </c>
@@ -7283,17 +7280,17 @@
       </c>
     </row>
     <row r="15" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="411" t="s">
+      <c r="A15" s="416" t="s">
         <v>47</v>
       </c>
-      <c r="B15" s="411"/>
-      <c r="C15" s="411"/>
+      <c r="B15" s="416"/>
+      <c r="C15" s="416"/>
       <c r="D15" s="17"/>
-      <c r="E15" s="411" t="s">
+      <c r="E15" s="416" t="s">
         <v>48</v>
       </c>
-      <c r="F15" s="411"/>
-      <c r="G15" s="411"/>
+      <c r="F15" s="416"/>
+      <c r="G15" s="416"/>
       <c r="H15" s="58" t="s">
         <v>49</v>
       </c>
@@ -7314,15 +7311,15 @@
       </c>
     </row>
     <row r="16" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="420"/>
-      <c r="B16" s="420"/>
-      <c r="C16" s="420"/>
+      <c r="A16" s="421"/>
+      <c r="B16" s="421"/>
+      <c r="C16" s="421"/>
       <c r="D16" s="17"/>
-      <c r="E16" s="418" t="s">
+      <c r="E16" s="422" t="s">
         <v>51</v>
       </c>
-      <c r="F16" s="418"/>
-      <c r="G16" s="418"/>
+      <c r="F16" s="422"/>
+      <c r="G16" s="422"/>
       <c r="H16" s="58" t="s">
         <v>52</v>
       </c>
@@ -7350,13 +7347,13 @@
       <c r="R16" s="72"/>
     </row>
     <row r="17" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="420"/>
-      <c r="B17" s="420"/>
-      <c r="C17" s="420"/>
+      <c r="A17" s="421"/>
+      <c r="B17" s="421"/>
+      <c r="C17" s="421"/>
       <c r="D17" s="17"/>
-      <c r="E17" s="418"/>
-      <c r="F17" s="418"/>
-      <c r="G17" s="418"/>
+      <c r="E17" s="422"/>
+      <c r="F17" s="422"/>
+      <c r="G17" s="422"/>
       <c r="H17" s="58" t="s">
         <v>55</v>
       </c>
@@ -7384,13 +7381,13 @@
       <c r="R17" s="72"/>
     </row>
     <row r="18" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="420"/>
-      <c r="B18" s="420"/>
-      <c r="C18" s="420"/>
+      <c r="A18" s="421"/>
+      <c r="B18" s="421"/>
+      <c r="C18" s="421"/>
       <c r="D18" s="17"/>
-      <c r="E18" s="418"/>
-      <c r="F18" s="418"/>
-      <c r="G18" s="418"/>
+      <c r="E18" s="422"/>
+      <c r="F18" s="422"/>
+      <c r="G18" s="422"/>
       <c r="H18" s="65" t="s">
         <v>58</v>
       </c>
@@ -7418,21 +7415,21 @@
       <c r="R18" s="71"/>
     </row>
     <row r="19" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="421" t="s">
+      <c r="A19" s="418" t="s">
         <v>61</v>
       </c>
-      <c r="B19" s="421"/>
-      <c r="C19" s="421"/>
+      <c r="B19" s="418"/>
+      <c r="C19" s="418"/>
       <c r="D19" s="17"/>
-      <c r="E19" s="422" t="s">
+      <c r="E19" s="417" t="s">
         <v>62</v>
       </c>
-      <c r="F19" s="422"/>
-      <c r="G19" s="422"/>
-      <c r="H19" s="411" t="s">
+      <c r="F19" s="417"/>
+      <c r="G19" s="417"/>
+      <c r="H19" s="416" t="s">
         <v>63</v>
       </c>
-      <c r="I19" s="411"/>
+      <c r="I19" s="416"/>
       <c r="K19" s="60" t="s">
         <v>64</v>
       </c>
@@ -7453,17 +7450,17 @@
       <c r="R19" s="74"/>
     </row>
     <row r="20" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="417" t="s">
+      <c r="A20" s="419" t="s">
         <v>66</v>
       </c>
-      <c r="B20" s="417"/>
-      <c r="C20" s="417"/>
+      <c r="B20" s="419"/>
+      <c r="C20" s="419"/>
       <c r="D20" s="17"/>
-      <c r="E20" s="413" t="s">
+      <c r="E20" s="423" t="s">
         <v>67</v>
       </c>
-      <c r="F20" s="413"/>
-      <c r="G20" s="413"/>
+      <c r="F20" s="423"/>
+      <c r="G20" s="423"/>
       <c r="H20" s="60" t="s">
         <v>68</v>
       </c>
@@ -7491,15 +7488,15 @@
       <c r="R20" s="74"/>
     </row>
     <row r="21" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="417"/>
-      <c r="B21" s="417"/>
-      <c r="C21" s="417"/>
+      <c r="A21" s="419"/>
+      <c r="B21" s="419"/>
+      <c r="C21" s="419"/>
       <c r="D21" s="17"/>
-      <c r="E21" s="415" t="s">
+      <c r="E21" s="424" t="s">
         <v>71</v>
       </c>
-      <c r="F21" s="415"/>
-      <c r="G21" s="415"/>
+      <c r="F21" s="424"/>
+      <c r="G21" s="424"/>
       <c r="H21" s="58" t="s">
         <v>72</v>
       </c>
@@ -7527,15 +7524,15 @@
       <c r="R21" s="78"/>
     </row>
     <row r="22" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="417"/>
-      <c r="B22" s="417"/>
-      <c r="C22" s="417"/>
+      <c r="A22" s="419"/>
+      <c r="B22" s="419"/>
+      <c r="C22" s="419"/>
       <c r="D22" s="17"/>
-      <c r="E22" s="418" t="s">
+      <c r="E22" s="422" t="s">
         <v>75</v>
       </c>
-      <c r="F22" s="418"/>
-      <c r="G22" s="418"/>
+      <c r="F22" s="422"/>
+      <c r="G22" s="422"/>
       <c r="H22" s="58" t="s">
         <v>76</v>
       </c>
@@ -7563,15 +7560,15 @@
       <c r="R22" s="71"/>
     </row>
     <row r="23" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="417"/>
-      <c r="B23" s="417"/>
-      <c r="C23" s="417"/>
+      <c r="A23" s="419"/>
+      <c r="B23" s="419"/>
+      <c r="C23" s="419"/>
       <c r="D23" s="17"/>
-      <c r="E23" s="419" t="s">
+      <c r="E23" s="425" t="s">
         <v>79</v>
       </c>
-      <c r="F23" s="419"/>
-      <c r="G23" s="419"/>
+      <c r="F23" s="425"/>
+      <c r="G23" s="425"/>
       <c r="H23" s="58" t="s">
         <v>80</v>
       </c>
@@ -7599,17 +7596,17 @@
       <c r="R23" s="74"/>
     </row>
     <row r="24" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="411" t="s">
+      <c r="A24" s="416" t="s">
         <v>83</v>
       </c>
-      <c r="B24" s="411"/>
-      <c r="C24" s="411"/>
+      <c r="B24" s="416"/>
+      <c r="C24" s="416"/>
       <c r="D24" s="17"/>
-      <c r="E24" s="413" t="s">
+      <c r="E24" s="423" t="s">
         <v>67</v>
       </c>
-      <c r="F24" s="413"/>
-      <c r="G24" s="413"/>
+      <c r="F24" s="423"/>
+      <c r="G24" s="423"/>
       <c r="H24" s="58" t="s">
         <v>84</v>
       </c>
@@ -7640,16 +7637,16 @@
       <c r="A25" s="79" t="s">
         <v>87</v>
       </c>
-      <c r="B25" s="414" t="s">
+      <c r="B25" s="428" t="s">
         <v>88</v>
       </c>
-      <c r="C25" s="414"/>
+      <c r="C25" s="428"/>
       <c r="D25" s="17"/>
-      <c r="E25" s="415" t="s">
+      <c r="E25" s="424" t="s">
         <v>71</v>
       </c>
-      <c r="F25" s="415"/>
-      <c r="G25" s="415"/>
+      <c r="F25" s="424"/>
+      <c r="G25" s="424"/>
       <c r="H25" s="58" t="s">
         <v>89</v>
       </c>
@@ -7662,29 +7659,29 @@
       <c r="A26" s="79" t="s">
         <v>90</v>
       </c>
-      <c r="B26" s="416" t="s">
+      <c r="B26" s="429" t="s">
         <v>91</v>
       </c>
-      <c r="C26" s="416"/>
+      <c r="C26" s="429"/>
       <c r="D26" s="17"/>
-      <c r="E26" s="415" t="s">
+      <c r="E26" s="424" t="s">
         <v>75</v>
       </c>
-      <c r="F26" s="415"/>
-      <c r="G26" s="415"/>
+      <c r="F26" s="424"/>
+      <c r="G26" s="424"/>
       <c r="H26" s="58"/>
       <c r="I26" s="59"/>
     </row>
     <row r="27" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="410" t="s">
+      <c r="A27" s="426" t="s">
         <v>92</v>
       </c>
-      <c r="B27" s="410"/>
-      <c r="C27" s="410"/>
-      <c r="D27" s="410"/>
-      <c r="E27" s="410"/>
-      <c r="F27" s="410"/>
-      <c r="G27" s="410"/>
+      <c r="B27" s="426"/>
+      <c r="C27" s="426"/>
+      <c r="D27" s="426"/>
+      <c r="E27" s="426"/>
+      <c r="F27" s="426"/>
+      <c r="G27" s="426"/>
       <c r="H27" s="65"/>
       <c r="I27" s="54"/>
     </row>
@@ -7696,15 +7693,15 @@
       <c r="E28" s="81"/>
       <c r="F28" s="81"/>
       <c r="G28" s="83"/>
-      <c r="H28" s="411" t="s">
+      <c r="H28" s="416" t="s">
         <v>93</v>
       </c>
-      <c r="I28" s="411"/>
-      <c r="K28" s="411" t="s">
+      <c r="I28" s="416"/>
+      <c r="K28" s="416" t="s">
         <v>94</v>
       </c>
-      <c r="L28" s="411"/>
-      <c r="M28" s="411"/>
+      <c r="L28" s="416"/>
+      <c r="M28" s="416"/>
     </row>
     <row r="29" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="80"/>
@@ -7809,14 +7806,14 @@
       <c r="E33" s="81"/>
       <c r="F33" s="81"/>
       <c r="G33" s="83"/>
-      <c r="H33" s="412" t="s">
+      <c r="H33" s="427" t="s">
         <v>103</v>
       </c>
-      <c r="I33" s="412"/>
-      <c r="J33" s="412"/>
-      <c r="K33" s="412"/>
-      <c r="L33" s="412"/>
-      <c r="M33" s="412"/>
+      <c r="I33" s="427"/>
+      <c r="J33" s="427"/>
+      <c r="K33" s="427"/>
+      <c r="L33" s="427"/>
+      <c r="M33" s="427"/>
     </row>
     <row r="34" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="80"/>
@@ -8069,31 +8066,6 @@
     <row r="69" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="35">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="H1:M1"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="H2:M2"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="K5:M5"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="A11:C14"/>
-    <mergeCell ref="E11:G14"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="E15:G15"/>
-    <mergeCell ref="A16:C18"/>
-    <mergeCell ref="E16:G18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="A20:C23"/>
-    <mergeCell ref="E20:G20"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="E22:G22"/>
-    <mergeCell ref="E23:G23"/>
     <mergeCell ref="A27:G27"/>
     <mergeCell ref="H28:I28"/>
     <mergeCell ref="K28:M28"/>
@@ -8104,6 +8076,31 @@
     <mergeCell ref="E25:G25"/>
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="E26:G26"/>
+    <mergeCell ref="A20:C23"/>
+    <mergeCell ref="E20:G20"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="E23:G23"/>
+    <mergeCell ref="A16:C18"/>
+    <mergeCell ref="E16:G18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="A11:C14"/>
+    <mergeCell ref="E11:G14"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="K5:M5"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="H1:M1"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="H2:M2"/>
+    <mergeCell ref="F3:G3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.45" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
@@ -9543,7 +9540,7 @@
       </c>
       <c r="N7" s="365">
         <f>D77</f>
-        <v>200.13228565680652</v>
+        <v>193.02286141537462</v>
       </c>
       <c r="R7" s="383" t="s">
         <v>188</v>
@@ -9581,11 +9578,11 @@
       </c>
       <c r="M8" s="367">
         <f>C108</f>
-        <v>205.78865016103435</v>
+        <v>204.50280102213321</v>
       </c>
       <c r="N8" s="368">
         <f>D108</f>
-        <v>245.16759035878044</v>
+        <v>228.14877997561089</v>
       </c>
     </row>
     <row r="9" spans="2:24" x14ac:dyDescent="0.2">
@@ -9596,12 +9593,7 @@
         <f>FrontPage!C4</f>
         <v>46300</v>
       </c>
-      <c r="F9" s="191" t="s">
-        <v>389</v>
-      </c>
-      <c r="H9">
-        <v>0</v>
-      </c>
+      <c r="H9"/>
       <c r="I9" s="200"/>
       <c r="J9" s="200"/>
     </row>
@@ -10277,7 +10269,7 @@
         <v>225</v>
       </c>
       <c r="I47" s="330">
-        <v>13.5</v>
+        <v>13.02</v>
       </c>
       <c r="J47" s="287"/>
     </row>
@@ -10287,7 +10279,7 @@
         <v>Terminal value in 2028</v>
       </c>
       <c r="C48" s="207">
-        <f>C47/(H6-C46)</f>
+        <f>(C47/(H6-C46))</f>
         <v>52410.884780436478</v>
       </c>
       <c r="E48" s="191" t="str">
@@ -10296,7 +10288,7 @@
       </c>
       <c r="I48" s="207">
         <f>I46*I47</f>
-        <v>47981.7</v>
+        <v>46275.683999999994</v>
       </c>
       <c r="J48" s="285"/>
     </row>
@@ -10305,15 +10297,15 @@
         <v>226</v>
       </c>
       <c r="C49" s="207">
-        <f>C48/(1+$H$6)^(($G$41-$D$41)/365)</f>
+        <f>C48/(1+H6)^((G41-D41)/365)</f>
         <v>45244.618421905558</v>
       </c>
       <c r="E49" s="191" t="s">
         <v>226</v>
       </c>
       <c r="I49" s="207">
-        <f>I48/(1+$H$6)^(($G$41-$D$41)/365)</f>
-        <v>41421.046731588234</v>
+        <f>I48/(1+H6)^((G41-D41)/365)</f>
+        <v>39948.298403353983</v>
       </c>
       <c r="J49" s="285"/>
     </row>
@@ -10329,7 +10321,7 @@
         <v>227</v>
       </c>
       <c r="I50" s="207">
-        <f>SUM(E43:I43)</f>
+        <f>SUM(E43:G43)</f>
         <v>3792.331620836705</v>
       </c>
       <c r="J50" s="285"/>
@@ -10348,7 +10340,7 @@
       </c>
       <c r="I51" s="289">
         <f>I49+I50</f>
-        <v>45213.378352424937</v>
+        <v>43740.630024190687</v>
       </c>
       <c r="J51" s="291"/>
     </row>
@@ -10370,7 +10362,7 @@
       </c>
       <c r="I53" s="294">
         <f>I49/$I$51</f>
-        <v>0.91612368376287656</v>
+        <v>0.91329956567293702</v>
       </c>
       <c r="J53" s="296"/>
     </row>
@@ -10388,7 +10380,7 @@
       <c r="G54" s="297"/>
       <c r="I54" s="294">
         <f t="shared" ref="I54" si="11">I50/$I$51</f>
-        <v>8.3876316237123438E-2</v>
+        <v>8.6700434327063008E-2</v>
       </c>
       <c r="J54" s="331"/>
     </row>
@@ -10405,7 +10397,7 @@
       </c>
       <c r="I55" s="332">
         <f>(H6-G42/I48)/(1+G42/I48)</f>
-        <v>2.6644615925342851E-2</v>
+        <v>2.518769378172846E-2</v>
       </c>
       <c r="J55" s="299"/>
     </row>
@@ -10500,9 +10492,7 @@
       <c r="B62" s="308" t="s">
         <v>246</v>
       </c>
-      <c r="C62" s="339">
-        <v>0</v>
-      </c>
+      <c r="C62" s="339"/>
       <c r="E62" s="211" t="s">
         <v>247</v>
       </c>
@@ -10520,9 +10510,7 @@
       <c r="B63" s="308" t="s">
         <v>249</v>
       </c>
-      <c r="C63" s="339">
-        <v>0</v>
-      </c>
+      <c r="C63" s="339"/>
       <c r="E63" s="191" t="s">
         <v>246</v>
       </c>
@@ -10540,9 +10528,7 @@
       <c r="B64" s="311" t="s">
         <v>251</v>
       </c>
-      <c r="C64" s="327">
-        <v>0</v>
-      </c>
+      <c r="C64" s="327"/>
       <c r="E64" s="191" t="s">
         <v>252</v>
       </c>
@@ -10589,9 +10575,7 @@
       <c r="B67" s="312" t="s">
         <v>257</v>
       </c>
-      <c r="C67" s="327">
-        <v>0</v>
-      </c>
+      <c r="C67" s="327"/>
       <c r="G67" s="206"/>
       <c r="I67" s="355"/>
       <c r="J67" s="359"/>
@@ -10664,7 +10648,7 @@
       </c>
       <c r="D73" s="345">
         <f>I51</f>
-        <v>45213.378352424937</v>
+        <v>43740.630024190687</v>
       </c>
       <c r="H73" s="284"/>
       <c r="J73" s="282"/>
@@ -10697,7 +10681,7 @@
       </c>
       <c r="D75" s="301">
         <f>D73-D74</f>
-        <v>41458.278352424939</v>
+        <v>39985.530024190688</v>
       </c>
       <c r="H75" s="207"/>
       <c r="J75" s="282"/>
@@ -10729,7 +10713,7 @@
       </c>
       <c r="D77" s="347">
         <f t="shared" ref="D77" si="12">D75/D76</f>
-        <v>200.13228565680652</v>
+        <v>193.02286141537462</v>
       </c>
       <c r="H77" s="288"/>
       <c r="J77" s="282"/>
@@ -10770,7 +10754,7 @@
       </c>
       <c r="D80" s="350">
         <f>D73/$E$17</f>
-        <v>3.6769306999898292</v>
+        <v>3.557160982734167</v>
       </c>
       <c r="E80" s="349"/>
       <c r="F80" s="349"/>
@@ -10789,7 +10773,7 @@
       </c>
       <c r="D81" s="349">
         <f>D73/$E$19</f>
-        <v>14.89683316939308</v>
+        <v>14.411594354120355</v>
       </c>
       <c r="E81" s="349"/>
       <c r="F81" s="349"/>
@@ -10809,7 +10793,7 @@
       </c>
       <c r="D82" s="316">
         <f>D73/$E$21</f>
-        <v>17.753778247963247</v>
+        <v>17.175479342034951</v>
       </c>
       <c r="E82" s="316"/>
       <c r="F82" s="317"/>
@@ -10980,7 +10964,7 @@
         <v>270</v>
       </c>
       <c r="I94" s="287">
-        <v>25.3</v>
+        <v>23.4</v>
       </c>
     </row>
     <row r="95" spans="2:14" x14ac:dyDescent="0.2">
@@ -10989,7 +10973,7 @@
         <v>Terminal value in 2028</v>
       </c>
       <c r="C95" s="207">
-        <f>C94/('WACC calculation'!D11-C93)</f>
+        <f>C94/('WACC calculation'!D11-'DCF 1-Pager'!C93)</f>
         <v>44931.115355377246</v>
       </c>
       <c r="E95" s="191" t="str">
@@ -10997,8 +10981,8 @@
         <v>Terminal value in 2028</v>
       </c>
       <c r="I95" s="285">
-        <f>I93*I94</f>
-        <v>54756.735084084903</v>
+        <f>I94*I93</f>
+        <v>50644.569208205008</v>
       </c>
     </row>
     <row r="96" spans="2:14" x14ac:dyDescent="0.2">
@@ -11006,15 +10990,15 @@
         <v>226</v>
       </c>
       <c r="C96" s="207">
-        <f>C95/(1+$H$6)^(($G$41-$D$41)/365)</f>
-        <v>38787.575864078652</v>
+        <f>C95/(1+'WACC calculation'!D11)^(('DCF 1-Pager'!G88-'DCF 1-Pager'!D88)/365)</f>
+        <v>38521.206590651149</v>
       </c>
       <c r="E96" s="191" t="s">
         <v>226</v>
       </c>
       <c r="I96" s="207">
-        <f>I95/(1+'WACC calculation'!D11)^(($G$41-$D$41)/365)</f>
-        <v>46945.09556952618</v>
+        <f>I95/(1+'WACC calculation'!D11)^((G88-D88)/365)</f>
+        <v>43419.574558375993</v>
       </c>
     </row>
     <row r="97" spans="2:43" x14ac:dyDescent="0.2">
@@ -11029,7 +11013,7 @@
         <v>227</v>
       </c>
       <c r="I97" s="285">
-        <f>SUM(E90:I90)</f>
+        <f>SUM(E90:G90)</f>
         <v>3842.4431363354206</v>
       </c>
     </row>
@@ -11039,7 +11023,7 @@
       </c>
       <c r="C98" s="289">
         <f>C96+C97</f>
-        <v>42630.019000414075</v>
+        <v>42363.649726986572</v>
       </c>
       <c r="D98" s="290"/>
       <c r="E98" s="206" t="s">
@@ -11047,7 +11031,7 @@
       </c>
       <c r="I98" s="291">
         <f>I96+I97</f>
-        <v>50787.538705861603</v>
+        <v>47262.017694711416</v>
       </c>
     </row>
     <row r="99" spans="2:43" x14ac:dyDescent="0.2">
@@ -11061,14 +11045,14 @@
       </c>
       <c r="C100" s="294">
         <f>C96/C98</f>
-        <v>0.90986531964017892</v>
+        <v>0.90929858118698159</v>
       </c>
       <c r="E100" s="295" t="s">
         <v>230</v>
       </c>
       <c r="I100" s="296">
         <f>I96/I98</f>
-        <v>0.9243427967913721</v>
+        <v>0.9186991304274047</v>
       </c>
     </row>
     <row r="101" spans="2:43" x14ac:dyDescent="0.2">
@@ -11077,7 +11061,7 @@
       </c>
       <c r="C101" s="294">
         <f>1-C100</f>
-        <v>9.0134680359821084E-2</v>
+        <v>9.0701418813018408E-2</v>
       </c>
       <c r="E101" s="295" t="s">
         <v>231</v>
@@ -11085,7 +11069,7 @@
       <c r="G101" s="297"/>
       <c r="I101" s="296">
         <f>1-I100</f>
-        <v>7.5657203208627899E-2</v>
+        <v>8.1300869572595302E-2</v>
       </c>
     </row>
     <row r="102" spans="2:43" x14ac:dyDescent="0.2">
@@ -11101,7 +11085,7 @@
       </c>
       <c r="I102" s="332">
         <f>('WACC calculation'!D11-G89/I95)/(1+G89/I95)</f>
-        <v>3.7140360221669388E-2</v>
+        <v>3.4477618842799158E-2</v>
       </c>
     </row>
     <row r="103" spans="2:43" x14ac:dyDescent="0.2">
@@ -11140,11 +11124,11 @@
       </c>
       <c r="C106" s="301">
         <f>C98</f>
-        <v>42630.019000414075</v>
+        <v>42363.649726986572</v>
       </c>
       <c r="D106" s="301">
         <f>I98</f>
-        <v>50787.538705861603</v>
+        <v>47262.017694711416</v>
       </c>
       <c r="H106" s="207"/>
       <c r="I106" s="282"/>
@@ -11172,11 +11156,11 @@
       </c>
       <c r="C108" s="303">
         <f>C106/C107</f>
-        <v>205.78865016103435</v>
+        <v>204.50280102213321</v>
       </c>
       <c r="D108" s="303">
         <f t="shared" ref="D108" si="13">D106/D107</f>
-        <v>245.16759035878044</v>
+        <v>228.14877997561089</v>
       </c>
       <c r="E108" s="304"/>
       <c r="F108" s="304"/>
@@ -11622,7 +11606,7 @@
       <c r="B123" s="213"/>
       <c r="D123" s="234">
         <f>D77</f>
-        <v>200.13228565680652</v>
+        <v>193.02286141537462</v>
       </c>
       <c r="E123" s="235">
         <f t="shared" ref="E123" si="21">F123-0.5</f>
@@ -11646,7 +11630,7 @@
       <c r="J123" s="237"/>
       <c r="L123" s="299">
         <f>I55</f>
-        <v>2.6644615925342851E-2</v>
+        <v>2.518769378172846E-2</v>
       </c>
       <c r="M123" s="235">
         <f t="shared" ref="M123" si="23">N123-0.5</f>

</xml_diff>

<commit_message>
Workbook is Dr. Payne's final Hershey workbook (Module 5: Relative Valuation tab and the DCF tab's multiples block filled) with the FrontPage Capital Allocation and #REF! fixes carried over
Detail Data, DCF valuation, WACC, and Key Defns unchanged from Module 4; site data unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/workbook/QD-HSY.xlsx
+++ b/workbook/QD-HSY.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chrislester/Documents/GitHub/HSY-valuation/workbook/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87BD3D59-ADD7-4C49-ABD7-1D7E8AEC1A9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21BFE91B-72D0-734F-853F-64047DFF48D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15720" tabRatio="500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FrontPage" sheetId="1" r:id="rId1"/>
@@ -212,7 +212,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="389">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="394">
   <si>
     <t>Hershey Company</t>
   </si>
@@ -1177,6 +1177,21 @@
     <t>Company</t>
   </si>
   <si>
+    <t>Hershey</t>
+  </si>
+  <si>
+    <t>Mondelez</t>
+  </si>
+  <si>
+    <t>Lindt</t>
+  </si>
+  <si>
+    <t>Tootsie Roll</t>
+  </si>
+  <si>
+    <t>Average</t>
+  </si>
+  <si>
     <t>The score is calculated based on 9 criteria divided into 3 groups.[1]</t>
   </si>
   <si>
@@ -1391,7 +1406,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="35">
+  <numFmts count="36">
     <numFmt numFmtId="7" formatCode="&quot;$&quot;#,##0.00_);\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
@@ -1427,6 +1442,7 @@
     <numFmt numFmtId="193" formatCode="0.000"/>
     <numFmt numFmtId="194" formatCode="0.0000"/>
     <numFmt numFmtId="195" formatCode="&quot;$&quot;#,##0_);\(&quot;$&quot;#,##0\);@_)"/>
+    <numFmt numFmtId="196" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="48" x14ac:knownFonts="1">
     <font>
@@ -1495,7 +1511,7 @@
       <sz val="10"/>
       <color theme="10"/>
       <name val="Courier New"/>
-      <family val="1"/>
+      <charset val="1"/>
     </font>
     <font>
       <b/>
@@ -1571,7 +1587,7 @@
     <font>
       <sz val="10"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <b/>
@@ -1628,7 +1644,7 @@
     <font>
       <sz val="10"/>
       <name val="Courier New"/>
-      <family val="1"/>
+      <charset val="1"/>
     </font>
     <font>
       <b/>
@@ -1853,7 +1869,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="46">
+  <borders count="47">
     <border>
       <left/>
       <right/>
@@ -2350,6 +2366,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0"/>
@@ -2363,7 +2390,7 @@
     <xf numFmtId="44" fontId="29" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="29" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="430">
+  <cellXfs count="432">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3146,12 +3173,8 @@
     <xf numFmtId="164" fontId="18" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="195" fontId="47" fillId="13" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="195" fontId="47" fillId="13" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="195" fontId="47" fillId="13" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="187" fontId="47" fillId="13" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="195" fontId="47" fillId="13" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="195" fontId="47" fillId="13" borderId="12" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="187" fontId="47" fillId="13" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="193" fontId="45" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="4" applyFont="1"/>
@@ -3160,6 +3183,12 @@
     <xf numFmtId="43" fontId="45" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="4" applyFont="1"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" xfId="4" applyNumberFormat="1"/>
+    <xf numFmtId="195" fontId="47" fillId="13" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="195" fontId="47" fillId="13" borderId="46" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="195" fontId="47" fillId="13" borderId="42" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="47" fillId="13" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="196" fontId="47" fillId="13" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="47" fillId="13" borderId="42" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -3169,6 +3198,66 @@
     </xf>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" xfId="8" applyFont="1"/>
     <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3195,66 +3284,6 @@
     </xf>
     <xf numFmtId="195" fontId="47" fillId="13" borderId="45" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="10">
@@ -6207,8 +6236,8 @@
     <xdr:to>
       <xdr:col>26</xdr:col>
       <xdr:colOff>552960</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>171360</xdr:rowOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>190410</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -6891,21 +6920,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="410" t="s">
+      <c r="A1" s="403" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="410"/>
-      <c r="C1" s="410"/>
-      <c r="D1" s="410"/>
-      <c r="E1" s="410"/>
-      <c r="F1" s="410"/>
-      <c r="G1" s="410"/>
-      <c r="H1" s="411"/>
-      <c r="I1" s="411"/>
-      <c r="J1" s="411"/>
-      <c r="K1" s="411"/>
-      <c r="L1" s="411"/>
-      <c r="M1" s="411"/>
+      <c r="B1" s="403"/>
+      <c r="C1" s="403"/>
+      <c r="D1" s="403"/>
+      <c r="E1" s="403"/>
+      <c r="F1" s="403"/>
+      <c r="G1" s="403"/>
+      <c r="H1" s="404"/>
+      <c r="I1" s="404"/>
+      <c r="J1" s="404"/>
+      <c r="K1" s="404"/>
+      <c r="L1" s="404"/>
+      <c r="M1" s="404"/>
     </row>
     <row r="2" spans="1:18" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
@@ -6919,18 +6948,18 @@
       <c r="E2" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="412" t="s">
+      <c r="F2" s="405" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="412"/>
-      <c r="H2" s="413" t="s">
+      <c r="G2" s="405"/>
+      <c r="H2" s="406" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="413"/>
-      <c r="J2" s="413"/>
-      <c r="K2" s="413"/>
-      <c r="L2" s="413"/>
-      <c r="M2" s="413"/>
+      <c r="I2" s="406"/>
+      <c r="J2" s="406"/>
+      <c r="K2" s="406"/>
+      <c r="L2" s="406"/>
+      <c r="M2" s="406"/>
     </row>
     <row r="3" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
@@ -6944,8 +6973,8 @@
       <c r="E3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="414"/>
-      <c r="G3" s="414"/>
+      <c r="F3" s="407"/>
+      <c r="G3" s="407"/>
       <c r="H3" s="11" t="s">
         <v>8</v>
       </c>
@@ -6972,8 +7001,8 @@
       <c r="E4" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="415"/>
-      <c r="G4" s="415"/>
+      <c r="F4" s="408"/>
+      <c r="G4" s="408"/>
       <c r="H4" s="19" t="s">
         <v>13</v>
       </c>
@@ -7005,15 +7034,15 @@
       <c r="G5" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="H5" s="416" t="s">
+      <c r="H5" s="409" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="416"/>
-      <c r="K5" s="417" t="s">
+      <c r="I5" s="409"/>
+      <c r="K5" s="410" t="s">
         <v>20</v>
       </c>
-      <c r="L5" s="417"/>
-      <c r="M5" s="417"/>
+      <c r="L5" s="410"/>
+      <c r="M5" s="410"/>
     </row>
     <row r="6" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="30" t="s">
@@ -7043,7 +7072,7 @@
         <v>1451.5</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:18" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="30" t="s">
         <v>24</v>
       </c>
@@ -7079,7 +7108,7 @@
         <v>7.1361848574237952</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:18" ht="28" x14ac:dyDescent="0.2">
       <c r="A8" s="30" t="s">
         <v>27</v>
       </c>
@@ -7150,17 +7179,17 @@
       </c>
     </row>
     <row r="10" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="418" t="s">
+      <c r="A10" s="411" t="s">
         <v>33</v>
       </c>
-      <c r="B10" s="418"/>
-      <c r="C10" s="418"/>
+      <c r="B10" s="411"/>
+      <c r="C10" s="411"/>
       <c r="D10" s="17"/>
-      <c r="E10" s="416" t="s">
+      <c r="E10" s="409" t="s">
         <v>34</v>
       </c>
-      <c r="F10" s="416"/>
-      <c r="G10" s="416"/>
+      <c r="F10" s="409"/>
+      <c r="G10" s="409"/>
       <c r="H10" s="35" t="s">
         <v>35</v>
       </c>
@@ -7178,15 +7207,15 @@
       </c>
     </row>
     <row r="11" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="419"/>
-      <c r="B11" s="419"/>
-      <c r="C11" s="419"/>
+      <c r="A11" s="412"/>
+      <c r="B11" s="412"/>
+      <c r="C11" s="412"/>
       <c r="D11" s="17"/>
-      <c r="E11" s="420" t="s">
+      <c r="E11" s="413" t="s">
         <v>37</v>
       </c>
-      <c r="F11" s="420"/>
-      <c r="G11" s="420"/>
+      <c r="F11" s="413"/>
+      <c r="G11" s="413"/>
       <c r="H11" s="51" t="s">
         <v>38</v>
       </c>
@@ -7204,17 +7233,17 @@
       </c>
     </row>
     <row r="12" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="419"/>
-      <c r="B12" s="419"/>
-      <c r="C12" s="419"/>
+      <c r="A12" s="412"/>
+      <c r="B12" s="412"/>
+      <c r="C12" s="412"/>
       <c r="D12" s="17"/>
-      <c r="E12" s="420"/>
-      <c r="F12" s="420"/>
-      <c r="G12" s="420"/>
-      <c r="H12" s="416" t="s">
+      <c r="E12" s="413"/>
+      <c r="F12" s="413"/>
+      <c r="G12" s="413"/>
+      <c r="H12" s="409" t="s">
         <v>40</v>
       </c>
-      <c r="I12" s="416"/>
+      <c r="I12" s="409"/>
       <c r="K12" s="55" t="s">
         <v>41</v>
       </c>
@@ -7226,13 +7255,13 @@
       </c>
     </row>
     <row r="13" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="419"/>
-      <c r="B13" s="419"/>
-      <c r="C13" s="419"/>
+      <c r="A13" s="412"/>
+      <c r="B13" s="412"/>
+      <c r="C13" s="412"/>
       <c r="D13" s="17"/>
-      <c r="E13" s="420"/>
-      <c r="F13" s="420"/>
-      <c r="G13" s="420"/>
+      <c r="E13" s="413"/>
+      <c r="F13" s="413"/>
+      <c r="G13" s="413"/>
       <c r="H13" s="58" t="s">
         <v>43</v>
       </c>
@@ -7253,13 +7282,13 @@
       </c>
     </row>
     <row r="14" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="419"/>
-      <c r="B14" s="419"/>
-      <c r="C14" s="419"/>
+      <c r="A14" s="412"/>
+      <c r="B14" s="412"/>
+      <c r="C14" s="412"/>
       <c r="D14" s="17"/>
-      <c r="E14" s="420"/>
-      <c r="F14" s="420"/>
-      <c r="G14" s="420"/>
+      <c r="E14" s="413"/>
+      <c r="F14" s="413"/>
+      <c r="G14" s="413"/>
       <c r="H14" s="58" t="s">
         <v>45</v>
       </c>
@@ -7280,17 +7309,17 @@
       </c>
     </row>
     <row r="15" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="416" t="s">
+      <c r="A15" s="409" t="s">
         <v>47</v>
       </c>
-      <c r="B15" s="416"/>
-      <c r="C15" s="416"/>
+      <c r="B15" s="409"/>
+      <c r="C15" s="409"/>
       <c r="D15" s="17"/>
-      <c r="E15" s="416" t="s">
+      <c r="E15" s="409" t="s">
         <v>48</v>
       </c>
-      <c r="F15" s="416"/>
-      <c r="G15" s="416"/>
+      <c r="F15" s="409"/>
+      <c r="G15" s="409"/>
       <c r="H15" s="58" t="s">
         <v>49</v>
       </c>
@@ -7311,15 +7340,15 @@
       </c>
     </row>
     <row r="16" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="421"/>
-      <c r="B16" s="421"/>
-      <c r="C16" s="421"/>
+      <c r="A16" s="414"/>
+      <c r="B16" s="414"/>
+      <c r="C16" s="414"/>
       <c r="D16" s="17"/>
-      <c r="E16" s="422" t="s">
+      <c r="E16" s="415" t="s">
         <v>51</v>
       </c>
-      <c r="F16" s="422"/>
-      <c r="G16" s="422"/>
+      <c r="F16" s="415"/>
+      <c r="G16" s="415"/>
       <c r="H16" s="58" t="s">
         <v>52</v>
       </c>
@@ -7347,13 +7376,13 @@
       <c r="R16" s="72"/>
     </row>
     <row r="17" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="421"/>
-      <c r="B17" s="421"/>
-      <c r="C17" s="421"/>
+      <c r="A17" s="414"/>
+      <c r="B17" s="414"/>
+      <c r="C17" s="414"/>
       <c r="D17" s="17"/>
-      <c r="E17" s="422"/>
-      <c r="F17" s="422"/>
-      <c r="G17" s="422"/>
+      <c r="E17" s="415"/>
+      <c r="F17" s="415"/>
+      <c r="G17" s="415"/>
       <c r="H17" s="58" t="s">
         <v>55</v>
       </c>
@@ -7381,13 +7410,13 @@
       <c r="R17" s="72"/>
     </row>
     <row r="18" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="421"/>
-      <c r="B18" s="421"/>
-      <c r="C18" s="421"/>
+      <c r="A18" s="414"/>
+      <c r="B18" s="414"/>
+      <c r="C18" s="414"/>
       <c r="D18" s="17"/>
-      <c r="E18" s="422"/>
-      <c r="F18" s="422"/>
-      <c r="G18" s="422"/>
+      <c r="E18" s="415"/>
+      <c r="F18" s="415"/>
+      <c r="G18" s="415"/>
       <c r="H18" s="65" t="s">
         <v>58</v>
       </c>
@@ -7415,21 +7444,21 @@
       <c r="R18" s="71"/>
     </row>
     <row r="19" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="418" t="s">
+      <c r="A19" s="411" t="s">
         <v>61</v>
       </c>
-      <c r="B19" s="418"/>
-      <c r="C19" s="418"/>
+      <c r="B19" s="411"/>
+      <c r="C19" s="411"/>
       <c r="D19" s="17"/>
-      <c r="E19" s="417" t="s">
+      <c r="E19" s="410" t="s">
         <v>62</v>
       </c>
-      <c r="F19" s="417"/>
-      <c r="G19" s="417"/>
-      <c r="H19" s="416" t="s">
+      <c r="F19" s="410"/>
+      <c r="G19" s="410"/>
+      <c r="H19" s="409" t="s">
         <v>63</v>
       </c>
-      <c r="I19" s="416"/>
+      <c r="I19" s="409"/>
       <c r="K19" s="60" t="s">
         <v>64</v>
       </c>
@@ -7450,17 +7479,17 @@
       <c r="R19" s="74"/>
     </row>
     <row r="20" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="419" t="s">
+      <c r="A20" s="412" t="s">
         <v>66</v>
       </c>
-      <c r="B20" s="419"/>
-      <c r="C20" s="419"/>
+      <c r="B20" s="412"/>
+      <c r="C20" s="412"/>
       <c r="D20" s="17"/>
-      <c r="E20" s="423" t="s">
+      <c r="E20" s="416" t="s">
         <v>67</v>
       </c>
-      <c r="F20" s="423"/>
-      <c r="G20" s="423"/>
+      <c r="F20" s="416"/>
+      <c r="G20" s="416"/>
       <c r="H20" s="60" t="s">
         <v>68</v>
       </c>
@@ -7488,15 +7517,15 @@
       <c r="R20" s="74"/>
     </row>
     <row r="21" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="419"/>
-      <c r="B21" s="419"/>
-      <c r="C21" s="419"/>
+      <c r="A21" s="412"/>
+      <c r="B21" s="412"/>
+      <c r="C21" s="412"/>
       <c r="D21" s="17"/>
-      <c r="E21" s="424" t="s">
+      <c r="E21" s="417" t="s">
         <v>71</v>
       </c>
-      <c r="F21" s="424"/>
-      <c r="G21" s="424"/>
+      <c r="F21" s="417"/>
+      <c r="G21" s="417"/>
       <c r="H21" s="58" t="s">
         <v>72</v>
       </c>
@@ -7524,15 +7553,15 @@
       <c r="R21" s="78"/>
     </row>
     <row r="22" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="419"/>
-      <c r="B22" s="419"/>
-      <c r="C22" s="419"/>
+      <c r="A22" s="412"/>
+      <c r="B22" s="412"/>
+      <c r="C22" s="412"/>
       <c r="D22" s="17"/>
-      <c r="E22" s="422" t="s">
+      <c r="E22" s="415" t="s">
         <v>75</v>
       </c>
-      <c r="F22" s="422"/>
-      <c r="G22" s="422"/>
+      <c r="F22" s="415"/>
+      <c r="G22" s="415"/>
       <c r="H22" s="58" t="s">
         <v>76</v>
       </c>
@@ -7560,15 +7589,15 @@
       <c r="R22" s="71"/>
     </row>
     <row r="23" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="419"/>
-      <c r="B23" s="419"/>
-      <c r="C23" s="419"/>
+      <c r="A23" s="412"/>
+      <c r="B23" s="412"/>
+      <c r="C23" s="412"/>
       <c r="D23" s="17"/>
-      <c r="E23" s="425" t="s">
+      <c r="E23" s="418" t="s">
         <v>79</v>
       </c>
-      <c r="F23" s="425"/>
-      <c r="G23" s="425"/>
+      <c r="F23" s="418"/>
+      <c r="G23" s="418"/>
       <c r="H23" s="58" t="s">
         <v>80</v>
       </c>
@@ -7596,17 +7625,17 @@
       <c r="R23" s="74"/>
     </row>
     <row r="24" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="416" t="s">
+      <c r="A24" s="409" t="s">
         <v>83</v>
       </c>
-      <c r="B24" s="416"/>
-      <c r="C24" s="416"/>
+      <c r="B24" s="409"/>
+      <c r="C24" s="409"/>
       <c r="D24" s="17"/>
-      <c r="E24" s="423" t="s">
+      <c r="E24" s="416" t="s">
         <v>67</v>
       </c>
-      <c r="F24" s="423"/>
-      <c r="G24" s="423"/>
+      <c r="F24" s="416"/>
+      <c r="G24" s="416"/>
       <c r="H24" s="58" t="s">
         <v>84</v>
       </c>
@@ -7637,16 +7666,16 @@
       <c r="A25" s="79" t="s">
         <v>87</v>
       </c>
-      <c r="B25" s="428" t="s">
+      <c r="B25" s="421" t="s">
         <v>88</v>
       </c>
-      <c r="C25" s="428"/>
+      <c r="C25" s="421"/>
       <c r="D25" s="17"/>
-      <c r="E25" s="424" t="s">
+      <c r="E25" s="417" t="s">
         <v>71</v>
       </c>
-      <c r="F25" s="424"/>
-      <c r="G25" s="424"/>
+      <c r="F25" s="417"/>
+      <c r="G25" s="417"/>
       <c r="H25" s="58" t="s">
         <v>89</v>
       </c>
@@ -7659,29 +7688,29 @@
       <c r="A26" s="79" t="s">
         <v>90</v>
       </c>
-      <c r="B26" s="429" t="s">
+      <c r="B26" s="422" t="s">
         <v>91</v>
       </c>
-      <c r="C26" s="429"/>
+      <c r="C26" s="422"/>
       <c r="D26" s="17"/>
-      <c r="E26" s="424" t="s">
+      <c r="E26" s="417" t="s">
         <v>75</v>
       </c>
-      <c r="F26" s="424"/>
-      <c r="G26" s="424"/>
+      <c r="F26" s="417"/>
+      <c r="G26" s="417"/>
       <c r="H26" s="58"/>
       <c r="I26" s="59"/>
     </row>
     <row r="27" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="426" t="s">
+      <c r="A27" s="419" t="s">
         <v>92</v>
       </c>
-      <c r="B27" s="426"/>
-      <c r="C27" s="426"/>
-      <c r="D27" s="426"/>
-      <c r="E27" s="426"/>
-      <c r="F27" s="426"/>
-      <c r="G27" s="426"/>
+      <c r="B27" s="419"/>
+      <c r="C27" s="419"/>
+      <c r="D27" s="419"/>
+      <c r="E27" s="419"/>
+      <c r="F27" s="419"/>
+      <c r="G27" s="419"/>
       <c r="H27" s="65"/>
       <c r="I27" s="54"/>
     </row>
@@ -7693,15 +7722,15 @@
       <c r="E28" s="81"/>
       <c r="F28" s="81"/>
       <c r="G28" s="83"/>
-      <c r="H28" s="416" t="s">
+      <c r="H28" s="409" t="s">
         <v>93</v>
       </c>
-      <c r="I28" s="416"/>
-      <c r="K28" s="416" t="s">
+      <c r="I28" s="409"/>
+      <c r="K28" s="409" t="s">
         <v>94</v>
       </c>
-      <c r="L28" s="416"/>
-      <c r="M28" s="416"/>
+      <c r="L28" s="409"/>
+      <c r="M28" s="409"/>
     </row>
     <row r="29" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="80"/>
@@ -7806,14 +7835,14 @@
       <c r="E33" s="81"/>
       <c r="F33" s="81"/>
       <c r="G33" s="83"/>
-      <c r="H33" s="427" t="s">
+      <c r="H33" s="420" t="s">
         <v>103</v>
       </c>
-      <c r="I33" s="427"/>
-      <c r="J33" s="427"/>
-      <c r="K33" s="427"/>
-      <c r="L33" s="427"/>
-      <c r="M33" s="427"/>
+      <c r="I33" s="420"/>
+      <c r="J33" s="420"/>
+      <c r="K33" s="420"/>
+      <c r="L33" s="420"/>
+      <c r="M33" s="420"/>
     </row>
     <row r="34" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="80"/>
@@ -9378,9 +9407,15 @@
     <col min="13" max="13" width="20" style="191" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="22.5" style="191" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="8.1640625" style="191" customWidth="1"/>
-    <col min="17" max="18" width="8" style="191"/>
+    <col min="17" max="17" width="8" style="191"/>
+    <col min="18" max="18" width="12.6640625" style="191" customWidth="1"/>
     <col min="19" max="19" width="9.33203125" style="191" bestFit="1" customWidth="1"/>
-    <col min="20" max="41" width="8" style="191"/>
+    <col min="20" max="20" width="10.6640625" style="191" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="17" style="191" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.1640625" style="191" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.6640625" style="191" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="18" style="191" bestFit="1" customWidth="1"/>
+    <col min="25" max="41" width="8" style="191"/>
     <col min="42" max="42" width="14.5" style="191" customWidth="1"/>
     <col min="43" max="43" width="12.1640625" style="191" bestFit="1" customWidth="1"/>
     <col min="44" max="46" width="22" style="191" bestFit="1" customWidth="1"/>
@@ -9406,20 +9441,20 @@
       <c r="B3" s="194" t="s">
         <v>169</v>
       </c>
-      <c r="L3" s="404" t="s">
+      <c r="L3" s="426" t="s">
         <v>170</v>
       </c>
-      <c r="M3" s="405"/>
-      <c r="N3" s="406"/>
-      <c r="R3" s="407" t="s">
+      <c r="M3" s="427"/>
+      <c r="N3" s="428"/>
+      <c r="R3" s="429" t="s">
         <v>171</v>
       </c>
-      <c r="S3" s="408"/>
-      <c r="T3" s="408"/>
-      <c r="U3" s="408"/>
-      <c r="V3" s="408"/>
-      <c r="W3" s="408"/>
-      <c r="X3" s="409"/>
+      <c r="S3" s="430"/>
+      <c r="T3" s="430"/>
+      <c r="U3" s="430"/>
+      <c r="V3" s="430"/>
+      <c r="W3" s="430"/>
+      <c r="X3" s="431"/>
     </row>
     <row r="4" spans="2:24" ht="21" x14ac:dyDescent="0.25">
       <c r="B4" s="191" t="s">
@@ -9430,25 +9465,25 @@
         <v>Hershey Company</v>
       </c>
       <c r="L4" s="362"/>
-      <c r="M4" s="402" t="s">
+      <c r="M4" s="424" t="s">
         <v>173</v>
       </c>
-      <c r="N4" s="403"/>
+      <c r="N4" s="425"/>
       <c r="R4" s="379"/>
-      <c r="S4" s="380"/>
-      <c r="T4" s="380" t="s">
+      <c r="S4" s="390"/>
+      <c r="T4" s="390" t="s">
         <v>174</v>
       </c>
-      <c r="U4" s="380" t="s">
+      <c r="U4" s="390" t="s">
         <v>175</v>
       </c>
-      <c r="V4" s="380" t="s">
+      <c r="V4" s="390" t="s">
         <v>176</v>
       </c>
-      <c r="W4" s="380" t="s">
+      <c r="W4" s="390" t="s">
         <v>177</v>
       </c>
-      <c r="X4" s="381" t="s">
+      <c r="X4" s="380" t="s">
         <v>178</v>
       </c>
     </row>
@@ -9470,20 +9505,29 @@
       <c r="R5" s="379" t="s">
         <v>182</v>
       </c>
-      <c r="S5" s="380" t="e">
-        <f>AVERAGE('Relative Valuation'!D3:D6)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="T5" s="380">
-        <f>AD21-AD24</f>
-        <v>0</v>
-      </c>
-      <c r="U5" s="380"/>
-      <c r="V5" s="380"/>
-      <c r="W5" s="380"/>
-      <c r="X5" s="382"/>
-    </row>
-    <row r="6" spans="2:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S5" s="394">
+        <f>'Relative Valuation'!D7</f>
+        <v>25</v>
+      </c>
+      <c r="T5" s="390">
+        <f>G26</f>
+        <v>2164.2978294104705</v>
+      </c>
+      <c r="U5" s="390">
+        <f>T5*S5</f>
+        <v>54107.445735261761</v>
+      </c>
+      <c r="V5" s="390"/>
+      <c r="W5" s="393">
+        <f>I65</f>
+        <v>207.15437400000002</v>
+      </c>
+      <c r="X5" s="381">
+        <f>U5/W5</f>
+        <v>261.19383670489987</v>
+      </c>
+    </row>
+    <row r="6" spans="2:24" ht="21" x14ac:dyDescent="0.25">
       <c r="B6" s="191" t="s">
         <v>183</v>
       </c>
@@ -9503,20 +9547,32 @@
       <c r="R6" s="379" t="s">
         <v>129</v>
       </c>
-      <c r="S6" s="380" t="e">
-        <f>AVERAGE('Relative Valuation'!C3:C6)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="T6" s="380">
-        <f>AD19</f>
-        <v>0</v>
-      </c>
-      <c r="U6" s="380"/>
-      <c r="V6" s="380"/>
-      <c r="W6" s="380"/>
-      <c r="X6" s="382"/>
-    </row>
-    <row r="7" spans="2:24" ht="22" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S6" s="394">
+        <f>'Relative Valuation'!C7</f>
+        <v>18.87</v>
+      </c>
+      <c r="T6" s="390">
+        <f>G19</f>
+        <v>3554.2</v>
+      </c>
+      <c r="U6" s="390">
+        <f>T6*S6</f>
+        <v>67067.754000000001</v>
+      </c>
+      <c r="V6" s="390">
+        <f>U6-C69</f>
+        <v>63312.654000000002</v>
+      </c>
+      <c r="W6" s="393">
+        <f>W5</f>
+        <v>207.15437400000002</v>
+      </c>
+      <c r="X6" s="381">
+        <f>U6/W6</f>
+        <v>323.75736367507255</v>
+      </c>
+    </row>
+    <row r="7" spans="2:24" ht="21" x14ac:dyDescent="0.25">
       <c r="B7" s="191" t="s">
         <v>185</v>
       </c>
@@ -9542,21 +9598,33 @@
         <f>D77</f>
         <v>193.02286141537462</v>
       </c>
-      <c r="R7" s="383" t="s">
+      <c r="R7" s="391" t="s">
         <v>188</v>
       </c>
-      <c r="S7" s="380" t="e">
-        <f>AVERAGE('Relative Valuation'!E3:E6)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="T7" s="384">
-        <f>AD17</f>
-        <v>0</v>
-      </c>
-      <c r="U7" s="384"/>
-      <c r="V7" s="384"/>
-      <c r="W7" s="384"/>
-      <c r="X7" s="385"/>
+      <c r="S7" s="394">
+        <f>'Relative Valuation'!E7</f>
+        <v>3.42</v>
+      </c>
+      <c r="T7" s="392">
+        <f>G17</f>
+        <v>12931.9</v>
+      </c>
+      <c r="U7" s="392">
+        <f>T7*S7</f>
+        <v>44227.097999999998</v>
+      </c>
+      <c r="V7" s="392">
+        <f>U7-C69</f>
+        <v>40471.998</v>
+      </c>
+      <c r="W7" s="395">
+        <f>W6</f>
+        <v>207.15437400000002</v>
+      </c>
+      <c r="X7" s="381">
+        <f>U7/W7</f>
+        <v>213.49825806719386</v>
+      </c>
     </row>
     <row r="8" spans="2:24" ht="22" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="191" t="s">
@@ -9634,11 +9702,11 @@
       <c r="D14" s="205" t="s">
         <v>196</v>
       </c>
-      <c r="E14" s="401" t="s">
+      <c r="E14" s="423" t="s">
         <v>197</v>
       </c>
-      <c r="F14" s="401"/>
-      <c r="G14" s="401"/>
+      <c r="F14" s="423"/>
+      <c r="G14" s="423"/>
       <c r="H14" s="205"/>
       <c r="I14" s="205"/>
       <c r="J14" s="282"/>
@@ -10026,7 +10094,7 @@
       <c r="M32" s="207"/>
     </row>
     <row r="33" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B33" s="394" t="s">
+      <c r="B33" s="396" t="s">
         <v>210</v>
       </c>
       <c r="D33" s="326"/>
@@ -10161,15 +10229,15 @@
         <f>D9</f>
         <v>46300</v>
       </c>
-      <c r="E41" s="395">
+      <c r="E41" s="397">
         <f>DATE(YEAR($D$6)+1,12,31)</f>
         <v>46387</v>
       </c>
-      <c r="F41" s="395">
+      <c r="F41" s="397">
         <f>DATE(YEAR($D$6)+2,12,31)</f>
         <v>46752</v>
       </c>
-      <c r="G41" s="395">
+      <c r="G41" s="397">
         <f>DATE(YEAR($D$6)+3,12,31)</f>
         <v>47118</v>
       </c>
@@ -10588,9 +10656,9 @@
       <c r="B68" s="273"/>
       <c r="H68" s="274"/>
       <c r="I68" s="275"/>
-      <c r="J68" s="396"/>
-      <c r="K68" s="395"/>
-      <c r="L68" s="395"/>
+      <c r="J68" s="398"/>
+      <c r="K68" s="397"/>
+      <c r="L68" s="397"/>
       <c r="M68" s="275"/>
       <c r="N68" s="275"/>
     </row>
@@ -10860,15 +10928,15 @@
         <f>D9</f>
         <v>46300</v>
       </c>
-      <c r="E88" s="395">
+      <c r="E88" s="397">
         <f>DATE(YEAR($D$6)+1,12,31)</f>
         <v>46387</v>
       </c>
-      <c r="F88" s="395">
+      <c r="F88" s="397">
         <f>DATE(YEAR($D$6)+2,12,31)</f>
         <v>46752</v>
       </c>
-      <c r="G88" s="395">
+      <c r="G88" s="397">
         <f>DATE(YEAR($D$6)+3,12,31)</f>
         <v>47118</v>
       </c>
@@ -10943,7 +11011,7 @@
       <c r="C93" s="284">
         <v>0.03</v>
       </c>
-      <c r="E93" s="397" t="s">
+      <c r="E93" s="399" t="s">
         <v>269</v>
       </c>
       <c r="I93" s="285">
@@ -10960,7 +11028,7 @@
         <f>G89*(1+C93)</f>
         <v>1846.4405910399998</v>
       </c>
-      <c r="E94" s="397" t="s">
+      <c r="E94" s="399" t="s">
         <v>270</v>
       </c>
       <c r="I94" s="287">
@@ -11687,26 +11755,26 @@
         <f t="shared" ref="L124" si="27">L125+0.005</f>
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="M124" s="398">
+      <c r="M124" s="400">
         <f t="dataTable" ref="M124:Q128" dt2D="1" dtr="1" r1="I47" r2="H6" ca="1"/>
         <v>2.3820270964768707E-2</v>
       </c>
-      <c r="N124" s="398">
+      <c r="N124" s="400">
         <v>2.5590794515862929E-2</v>
       </c>
-      <c r="O124" s="398">
+      <c r="O124" s="400">
         <v>2.7230567821613351E-2</v>
       </c>
-      <c r="P124" s="398">
+      <c r="P124" s="400">
         <v>2.8753558668125297E-2</v>
       </c>
-      <c r="Q124" s="398">
+      <c r="Q124" s="400">
         <v>3.0171813717399184E-2</v>
       </c>
-      <c r="AP124" s="398" t="e">
+      <c r="AP124" s="400" t="e">
         <v>#DIV/0!</v>
       </c>
-      <c r="AQ124" s="398" t="e">
+      <c r="AQ124" s="400" t="e">
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -11736,25 +11804,25 @@
         <f>L126+0.005</f>
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="M125" s="398">
+      <c r="M125" s="400">
         <v>1.9036064091101559E-2</v>
       </c>
-      <c r="N125" s="398">
+      <c r="N125" s="400">
         <v>2.0798314167657955E-2</v>
       </c>
-      <c r="O125" s="398">
+      <c r="O125" s="400">
         <v>2.2430424981325432E-2</v>
       </c>
-      <c r="P125" s="398">
+      <c r="P125" s="400">
         <v>2.3946299048180783E-2</v>
       </c>
-      <c r="Q125" s="398">
+      <c r="Q125" s="400">
         <v>2.5357926737411336E-2</v>
       </c>
-      <c r="AP125" s="398" t="e">
+      <c r="AP125" s="400" t="e">
         <v>#DIV/0!</v>
       </c>
-      <c r="AQ125" s="398" t="e">
+      <c r="AQ125" s="400" t="e">
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -11788,25 +11856,25 @@
       <c r="L126" s="229">
         <v>0.06</v>
       </c>
-      <c r="M126" s="398">
+      <c r="M126" s="400">
         <v>1.425185721743441E-2</v>
       </c>
-      <c r="N126" s="398">
+      <c r="N126" s="400">
         <v>1.6005833819452985E-2</v>
       </c>
-      <c r="O126" s="398">
+      <c r="O126" s="400">
         <v>1.7630282141037516E-2</v>
       </c>
-      <c r="P126" s="398">
+      <c r="P126" s="400">
         <v>1.9139039428236269E-2</v>
       </c>
-      <c r="Q126" s="398">
+      <c r="Q126" s="400">
         <v>2.0544039757423485E-2</v>
       </c>
-      <c r="AP126" s="398" t="e">
+      <c r="AP126" s="400" t="e">
         <v>#DIV/0!</v>
       </c>
-      <c r="AQ126" s="398" t="e">
+      <c r="AQ126" s="400" t="e">
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -11836,25 +11904,25 @@
         <f>L126-0.005</f>
         <v>5.5E-2</v>
       </c>
-      <c r="M127" s="398">
+      <c r="M127" s="400">
         <v>9.4676503437672692E-3</v>
       </c>
-      <c r="N127" s="398">
+      <c r="N127" s="400">
         <v>1.121335347124802E-2</v>
       </c>
-      <c r="O127" s="398">
+      <c r="O127" s="400">
         <v>1.2830139300749605E-2</v>
       </c>
-      <c r="P127" s="398">
+      <c r="P127" s="400">
         <v>1.4331779808291759E-2</v>
       </c>
-      <c r="Q127" s="398">
+      <c r="Q127" s="400">
         <v>1.5730152777435641E-2</v>
       </c>
-      <c r="AP127" s="398" t="e">
+      <c r="AP127" s="400" t="e">
         <v>#DIV/0!</v>
       </c>
-      <c r="AQ127" s="398" t="e">
+      <c r="AQ127" s="400" t="e">
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -11884,25 +11952,25 @@
         <f>L127-0.005</f>
         <v>0.05</v>
       </c>
-      <c r="M128" s="398">
+      <c r="M128" s="400">
         <v>4.6834434701001288E-3</v>
       </c>
-      <c r="N128" s="398">
+      <c r="N128" s="400">
         <v>6.4208731230430555E-3</v>
       </c>
-      <c r="O128" s="398">
+      <c r="O128" s="400">
         <v>8.0299964604616941E-3</v>
       </c>
-      <c r="P128" s="398">
+      <c r="P128" s="400">
         <v>9.5245201883472526E-3</v>
       </c>
-      <c r="Q128" s="398">
+      <c r="Q128" s="400">
         <v>1.0916265797447795E-2</v>
       </c>
-      <c r="AP128" s="398" t="e">
+      <c r="AP128" s="400" t="e">
         <v>#DIV/0!</v>
       </c>
-      <c r="AQ128" s="398" t="e">
+      <c r="AQ128" s="400" t="e">
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -12200,25 +12268,25 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="C2" s="392" t="s">
+      <c r="C2" s="388" t="s">
         <v>288</v>
       </c>
-      <c r="D2" s="392" t="s">
+      <c r="D2" s="388" t="s">
         <v>289</v>
       </c>
-      <c r="E2" s="392" t="str">
+      <c r="E2" s="388" t="str">
         <f>'Detail Data'!D2</f>
         <v>2025A</v>
       </c>
-      <c r="F2" s="392" t="str">
+      <c r="F2" s="388" t="str">
         <f>'Detail Data'!E2</f>
         <v>2026F</v>
       </c>
-      <c r="G2" s="392" t="str">
+      <c r="G2" s="388" t="str">
         <f>'Detail Data'!F2</f>
         <v>2027F</v>
       </c>
-      <c r="H2" s="392" t="str">
+      <c r="H2" s="388" t="str">
         <f>'Detail Data'!G2</f>
         <v>2028F</v>
       </c>
@@ -12227,7 +12295,7 @@
       <c r="B3" s="260" t="s">
         <v>290</v>
       </c>
-      <c r="C3" s="399">
+      <c r="C3" s="401">
         <f>'Detail Data'!D3</f>
         <v>32582.646000000001</v>
       </c>
@@ -12235,7 +12303,7 @@
         <f>C3/C5</f>
         <v>0.87438158896206775</v>
       </c>
-      <c r="E3" s="400"/>
+      <c r="E3" s="402"/>
       <c r="F3" s="372"/>
       <c r="G3" s="372"/>
       <c r="H3" s="372"/>
@@ -12244,7 +12312,7 @@
       <c r="B4" s="260" t="s">
         <v>291</v>
       </c>
-      <c r="C4" s="399">
+      <c r="C4" s="401">
         <f>'Detail Data'!D34</f>
         <v>4681</v>
       </c>
@@ -12252,16 +12320,16 @@
         <f>C4/C5</f>
         <v>0.12561841103793225</v>
       </c>
-      <c r="E4" s="400"/>
-      <c r="F4" s="400"/>
-      <c r="G4" s="400"/>
-      <c r="H4" s="400"/>
+      <c r="E4" s="402"/>
+      <c r="F4" s="402"/>
+      <c r="G4" s="402"/>
+      <c r="H4" s="402"/>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B5" s="260" t="s">
         <v>292</v>
       </c>
-      <c r="C5" s="399">
+      <c r="C5" s="401">
         <f>C3+C4</f>
         <v>37263.646000000001</v>
       </c>
@@ -12272,19 +12340,19 @@
       <c r="C7" s="260" t="s">
         <v>293</v>
       </c>
-      <c r="D7" s="392" t="s">
+      <c r="D7" s="388" t="s">
         <v>294</v>
       </c>
-      <c r="E7" s="392" t="s">
+      <c r="E7" s="388" t="s">
         <v>295</v>
       </c>
-      <c r="F7" s="386" t="s">
+      <c r="F7" s="382" t="s">
         <v>296</v>
       </c>
-      <c r="G7" s="392" t="s">
+      <c r="G7" s="388" t="s">
         <v>297</v>
       </c>
-      <c r="H7" s="392"/>
+      <c r="H7" s="388"/>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.2">
       <c r="C8" s="260" t="s">
@@ -12318,21 +12386,21 @@
       <c r="C10" s="260" t="s">
         <v>302</v>
       </c>
-      <c r="D10" s="393">
+      <c r="D10" s="389">
         <f>(2/3)*G10+1/3</f>
         <v>0.41020000000000001</v>
       </c>
-      <c r="E10" s="386">
+      <c r="E10" s="382">
         <f>C29</f>
         <v>0.34661866709107808</v>
       </c>
       <c r="F10" s="260">
         <v>0.34</v>
       </c>
-      <c r="G10" s="386">
+      <c r="G10" s="382">
         <v>0.1153</v>
       </c>
-      <c r="H10" s="392" t="s">
+      <c r="H10" s="388" t="s">
         <v>303</v>
       </c>
     </row>
@@ -12401,16 +12469,16 @@
       <c r="H16" s="264"/>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B20" s="392" t="s">
+      <c r="B20" s="388" t="s">
         <v>308</v>
       </c>
-      <c r="C20" s="387"/>
+      <c r="C20" s="383"/>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B21" s="392" t="s">
+      <c r="B21" s="388" t="s">
         <v>309</v>
       </c>
-      <c r="C21" s="388">
+      <c r="C21" s="384">
         <v>0.61</v>
       </c>
       <c r="D21" s="260" t="s">
@@ -12418,74 +12486,74 @@
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B22" s="392" t="s">
+      <c r="B22" s="388" t="s">
         <v>311</v>
       </c>
-      <c r="C22" s="389">
+      <c r="C22" s="385">
         <v>0.43730000000000002</v>
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B23" s="392" t="s">
+      <c r="B23" s="388" t="s">
         <v>312</v>
       </c>
-      <c r="C23" s="389">
+      <c r="C23" s="385">
         <v>0.1037</v>
       </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B24" s="392" t="s">
+      <c r="B24" s="388" t="s">
         <v>313</v>
       </c>
-      <c r="C24" s="390">
+      <c r="C24" s="386">
         <f>C21/(1+(1-C23*C22))</f>
         <v>0.31207601308097815</v>
       </c>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C25" s="388"/>
+      <c r="C25" s="384"/>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B26" s="392" t="s">
+      <c r="B26" s="388" t="s">
         <v>314</v>
       </c>
-      <c r="C26" s="391"/>
+      <c r="C26" s="387"/>
     </row>
     <row r="27" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B27" s="392" t="s">
+      <c r="B27" s="388" t="s">
         <v>315</v>
       </c>
-      <c r="C27" s="389">
+      <c r="C27" s="385">
         <f>C4/C3</f>
         <v>0.14366543466113832</v>
       </c>
     </row>
     <row r="28" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B28" s="392" t="s">
+      <c r="B28" s="388" t="s">
         <v>312</v>
       </c>
-      <c r="C28" s="389">
+      <c r="C28" s="385">
         <f>'Detail Data'!D20/'Detail Data'!D16</f>
         <v>0.2295525494276795</v>
       </c>
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B29" s="392" t="s">
+      <c r="B29" s="388" t="s">
         <v>316</v>
       </c>
-      <c r="C29" s="390">
+      <c r="C29" s="386">
         <f>C24*(1+(1-C28)*C27)</f>
         <v>0.34661866709107808</v>
       </c>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C30" s="388"/>
+      <c r="C30" s="384"/>
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B31" s="392" t="s">
+      <c r="B31" s="388" t="s">
         <v>317</v>
       </c>
-      <c r="C31" s="388">
+      <c r="C31" s="384">
         <f>'Detail Data'!D16/'Detail Data'!D19</f>
         <v>7.5788643533123032</v>
       </c>
@@ -12498,7 +12566,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CFA75F6-4D5D-48FC-B8C9-2750576B974E}">
-  <dimension ref="B2:E6"/>
+  <dimension ref="B2:E7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="18.1640625" bestFit="1" customWidth="1"/>
@@ -12520,28 +12588,77 @@
       </c>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B3" s="378"/>
-      <c r="C3" s="378"/>
-      <c r="D3" s="378"/>
-      <c r="E3" s="378"/>
+      <c r="B3" s="378" t="s">
+        <v>319</v>
+      </c>
+      <c r="C3" s="378">
+        <v>13.8</v>
+      </c>
+      <c r="D3" s="378">
+        <v>23.4</v>
+      </c>
+      <c r="E3" s="378">
+        <v>3.05</v>
+      </c>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B4" s="378"/>
-      <c r="C4" s="378"/>
-      <c r="D4" s="378"/>
-      <c r="E4" s="378"/>
+      <c r="B4" s="378" t="s">
+        <v>320</v>
+      </c>
+      <c r="C4" s="378">
+        <v>12.22</v>
+      </c>
+      <c r="D4" s="378">
+        <v>21.34</v>
+      </c>
+      <c r="E4" s="378">
+        <v>2.36</v>
+      </c>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B5" s="378"/>
-      <c r="C5" s="378"/>
-      <c r="D5" s="378"/>
-      <c r="E5" s="378"/>
+      <c r="B5" s="378" t="s">
+        <v>321</v>
+      </c>
+      <c r="C5" s="378">
+        <v>19.079999999999998</v>
+      </c>
+      <c r="D5" s="378">
+        <v>23.79</v>
+      </c>
+      <c r="E5" s="378">
+        <v>4.16</v>
+      </c>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B6" s="378"/>
-      <c r="C6" s="378"/>
-      <c r="D6" s="378"/>
-      <c r="E6" s="378"/>
+      <c r="B6" s="378" t="s">
+        <v>322</v>
+      </c>
+      <c r="C6" s="378">
+        <v>25.31</v>
+      </c>
+      <c r="D6" s="378">
+        <v>29.87</v>
+      </c>
+      <c r="E6" s="378">
+        <v>3.74</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B7" s="378" t="s">
+        <v>323</v>
+      </c>
+      <c r="C7" s="378">
+        <f>AVERAGE(C4:C6)</f>
+        <v>18.87</v>
+      </c>
+      <c r="D7" s="378">
+        <f t="shared" ref="D7:E7" si="0">AVERAGE(D4:D6)</f>
+        <v>25</v>
+      </c>
+      <c r="E7" s="378">
+        <f t="shared" si="0"/>
+        <v>3.42</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12559,7 +12676,7 @@
       <c r="B1" s="93"/>
       <c r="C1" s="93"/>
       <c r="D1" s="179" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="E1" s="93"/>
       <c r="F1" s="93"/>
@@ -12572,7 +12689,7 @@
     </row>
     <row r="2" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="93" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="B2" s="180">
         <f>'Detail Data'!E12</f>
@@ -12593,7 +12710,7 @@
     </row>
     <row r="3" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="93" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="B3" s="182">
         <f>'Detail Data'!G7</f>
@@ -12601,7 +12718,7 @@
       </c>
       <c r="C3" s="93"/>
       <c r="D3" s="183" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="E3" s="93"/>
       <c r="F3" s="93"/>
@@ -12614,7 +12731,7 @@
     </row>
     <row r="4" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="93" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="B4" s="182">
         <f>B2*B3</f>
@@ -12622,7 +12739,7 @@
       </c>
       <c r="C4" s="93"/>
       <c r="D4" s="183" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="E4" s="93"/>
       <c r="F4" s="93"/>
@@ -12677,7 +12794,7 @@
     </row>
     <row r="8" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="93" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="B8" s="177" t="e">
         <f>B4/#REF!-1</f>
@@ -12685,7 +12802,7 @@
       </c>
       <c r="C8" s="93"/>
       <c r="D8" s="183" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="E8" s="93"/>
       <c r="F8" s="93"/>
@@ -12701,7 +12818,7 @@
       <c r="B9" s="148"/>
       <c r="C9" s="148"/>
       <c r="D9" s="181" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="E9" s="148"/>
       <c r="F9" s="93"/>
@@ -12714,7 +12831,7 @@
     </row>
     <row r="10" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="93" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="B10" s="180">
         <f>'Detail Data'!E11</f>
@@ -12722,7 +12839,7 @@
       </c>
       <c r="C10" s="93"/>
       <c r="D10" s="183" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="E10" s="93"/>
       <c r="F10" s="93"/>
@@ -12735,7 +12852,7 @@
     </row>
     <row r="11" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="93" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="B11" s="127">
         <f>'Detail Data'!E3</f>
@@ -12743,7 +12860,7 @@
       </c>
       <c r="C11" s="93"/>
       <c r="D11" s="183" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="E11" s="93"/>
       <c r="F11" s="93"/>
@@ -12756,7 +12873,7 @@
     </row>
     <row r="12" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="93" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="B12" s="127">
         <f>'Detail Data'!G5*'Detail Data'!E11</f>
@@ -12764,7 +12881,7 @@
       </c>
       <c r="C12" s="93"/>
       <c r="D12" s="183" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="E12" s="93"/>
       <c r="F12" s="93"/>
@@ -12785,7 +12902,7 @@
       </c>
       <c r="C13" s="93"/>
       <c r="D13" s="181" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="E13" s="93"/>
       <c r="F13" s="93"/>
@@ -12798,7 +12915,7 @@
     </row>
     <row r="14" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="93" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="B14" s="182">
         <f>B11/B13</f>
@@ -12806,7 +12923,7 @@
       </c>
       <c r="C14" s="93"/>
       <c r="D14" s="183" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="E14" s="93"/>
       <c r="F14" s="93"/>
@@ -12819,7 +12936,7 @@
     </row>
     <row r="15" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="93" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="B15" s="177" t="e">
         <f>B14/#REF!-1</f>
@@ -12827,7 +12944,7 @@
       </c>
       <c r="C15" s="93"/>
       <c r="D15" s="183" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="E15" s="93"/>
       <c r="F15" s="93"/>
@@ -12857,7 +12974,7 @@
       <c r="B17" s="93"/>
       <c r="C17" s="93"/>
       <c r="D17" s="185" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="E17" s="93"/>
       <c r="F17" s="93"/>
@@ -12873,7 +12990,7 @@
       <c r="B18" s="93"/>
       <c r="C18" s="93"/>
       <c r="D18" s="186" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="E18" s="93"/>
       <c r="F18" s="93"/>
@@ -12892,7 +13009,7 @@
       <c r="B19" s="93"/>
       <c r="C19" s="93"/>
       <c r="D19" s="93" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="E19" s="93"/>
       <c r="F19" s="93"/>
@@ -12911,7 +13028,7 @@
       <c r="B20" s="93"/>
       <c r="C20" s="93"/>
       <c r="D20" s="93" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="E20" s="93"/>
       <c r="F20" s="93"/>
@@ -12927,7 +13044,7 @@
       <c r="B21" s="93"/>
       <c r="C21" s="93"/>
       <c r="D21" s="93" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="E21" s="93"/>
       <c r="F21" s="93"/>
@@ -12940,7 +13057,7 @@
     </row>
     <row r="22" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="93" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="B22" s="93"/>
       <c r="C22" s="93"/>
@@ -12956,7 +13073,7 @@
     </row>
     <row r="23" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="93" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B23" s="93"/>
       <c r="C23" s="93"/>
@@ -12989,7 +13106,7 @@
       <c r="B25" s="93"/>
       <c r="C25" s="93"/>
       <c r="D25" s="187" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="E25" s="188"/>
       <c r="F25" s="93"/>
@@ -13033,12 +13150,12 @@
       <c r="B28" s="93"/>
       <c r="C28" s="93"/>
       <c r="D28" s="187" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="E28" s="188"/>
       <c r="F28" s="93"/>
       <c r="G28" s="187" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="H28" s="93"/>
       <c r="I28" s="93"/>
@@ -13054,7 +13171,7 @@
       <c r="E29" s="188"/>
       <c r="F29" s="93"/>
       <c r="G29" s="187" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="H29" s="93"/>
       <c r="I29" s="93"/>
@@ -13070,7 +13187,7 @@
       <c r="E30" s="188"/>
       <c r="F30" s="93"/>
       <c r="G30" s="187" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="H30" s="93"/>
       <c r="I30" s="93"/>
@@ -13153,11 +13270,11 @@
       <c r="B36" s="93"/>
       <c r="C36" s="93"/>
       <c r="D36" s="93" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="E36" s="188"/>
       <c r="F36" s="186" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="G36" s="93"/>
       <c r="H36" s="93"/>
@@ -13171,11 +13288,11 @@
       <c r="B37" s="93"/>
       <c r="C37" s="93"/>
       <c r="D37" s="93" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="E37" s="188"/>
       <c r="F37" s="186" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="G37" s="93"/>
       <c r="H37" s="93"/>
@@ -13189,11 +13306,11 @@
       <c r="B38" s="93"/>
       <c r="C38" s="93"/>
       <c r="D38" s="93" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
       <c r="E38" s="93"/>
       <c r="F38" s="186" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="G38" s="93"/>
       <c r="H38" s="93"/>
@@ -13221,7 +13338,7 @@
       <c r="B40" s="93"/>
       <c r="C40" s="93"/>
       <c r="D40" s="189" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="E40" s="188"/>
       <c r="F40" s="93"/>
@@ -13265,12 +13382,12 @@
       <c r="B43" s="93"/>
       <c r="C43" s="93"/>
       <c r="D43" s="187" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="E43" s="188"/>
       <c r="F43" s="93"/>
       <c r="G43" s="187" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="H43" s="93"/>
       <c r="I43" s="93"/>
@@ -13286,7 +13403,7 @@
       <c r="E44" s="188"/>
       <c r="F44" s="93"/>
       <c r="G44" s="187" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="H44" s="93"/>
       <c r="I44" s="93"/>
@@ -13302,7 +13419,7 @@
       <c r="E45" s="188"/>
       <c r="F45" s="93"/>
       <c r="G45" s="187" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="H45" s="93"/>
       <c r="I45" s="93"/>
@@ -13318,7 +13435,7 @@
       <c r="E46" s="188"/>
       <c r="F46" s="93"/>
       <c r="G46" s="187" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="H46" s="93"/>
       <c r="I46" s="93"/>
@@ -13334,7 +13451,7 @@
       <c r="E47" s="188"/>
       <c r="F47" s="93"/>
       <c r="G47" s="187" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="H47" s="93"/>
       <c r="I47" s="93"/>
@@ -13347,12 +13464,12 @@
       <c r="B48" s="93"/>
       <c r="C48" s="93"/>
       <c r="D48" s="187" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="E48" s="188"/>
       <c r="F48" s="93"/>
       <c r="G48" s="187" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="H48" s="93"/>
       <c r="I48" s="93"/>
@@ -13368,7 +13485,7 @@
       <c r="E49" s="188"/>
       <c r="F49" s="93"/>
       <c r="G49" s="187" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="H49" s="93"/>
       <c r="I49" s="93"/>
@@ -13398,7 +13515,7 @@
       <c r="E51" s="188"/>
       <c r="F51" s="93"/>
       <c r="G51" s="187" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="H51" s="93"/>
       <c r="I51" s="93"/>
@@ -13414,7 +13531,7 @@
       <c r="E52" s="188"/>
       <c r="F52" s="93"/>
       <c r="G52" s="187" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
       <c r="H52" s="93"/>
       <c r="I52" s="93"/>
@@ -13430,7 +13547,7 @@
       <c r="E53" s="188"/>
       <c r="F53" s="93"/>
       <c r="G53" s="187" t="s">
-        <v>368</v>
+        <v>373</v>
       </c>
       <c r="H53" s="93"/>
       <c r="I53" s="93"/>
@@ -13457,12 +13574,12 @@
       <c r="B55" s="93"/>
       <c r="C55" s="93"/>
       <c r="D55" s="187" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="E55" s="188"/>
       <c r="F55" s="93"/>
       <c r="G55" s="187" t="s">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="H55" s="93"/>
       <c r="I55" s="93"/>
@@ -13489,12 +13606,12 @@
       <c r="B57" s="93"/>
       <c r="C57" s="93"/>
       <c r="D57" s="187" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
       <c r="E57" s="188"/>
       <c r="F57" s="93"/>
       <c r="G57" s="187" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
       <c r="H57" s="93"/>
       <c r="I57" s="93"/>
@@ -13526,7 +13643,7 @@
       <c r="E59" s="188"/>
       <c r="F59" s="93"/>
       <c r="G59" s="187" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="H59" s="93"/>
       <c r="I59" s="93"/>
@@ -13539,12 +13656,12 @@
       <c r="B60" s="93"/>
       <c r="C60" s="93"/>
       <c r="D60" s="187" t="s">
-        <v>374</v>
+        <v>379</v>
       </c>
       <c r="E60" s="188"/>
       <c r="F60" s="93"/>
       <c r="G60" s="187" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="H60" s="93"/>
       <c r="I60" s="93"/>
@@ -13560,7 +13677,7 @@
       <c r="E61" s="188"/>
       <c r="F61" s="93"/>
       <c r="G61" s="187" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="H61" s="93"/>
       <c r="I61" s="93"/>
@@ -13576,7 +13693,7 @@
       <c r="E62" s="188"/>
       <c r="F62" s="93"/>
       <c r="G62" s="187" t="s">
-        <v>377</v>
+        <v>382</v>
       </c>
       <c r="H62" s="93"/>
       <c r="I62" s="93"/>
@@ -13592,7 +13709,7 @@
       <c r="E63" s="188"/>
       <c r="F63" s="93"/>
       <c r="G63" s="187" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="H63" s="93"/>
       <c r="I63" s="93"/>
@@ -13608,7 +13725,7 @@
       <c r="E64" s="188"/>
       <c r="F64" s="93"/>
       <c r="G64" s="187" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="H64" s="93"/>
       <c r="I64" s="93"/>
@@ -13624,7 +13741,7 @@
       <c r="E65" s="188"/>
       <c r="F65" s="93"/>
       <c r="G65" s="187" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="H65" s="93"/>
       <c r="I65" s="93"/>
@@ -13651,12 +13768,12 @@
       <c r="B67" s="93"/>
       <c r="C67" s="93"/>
       <c r="D67" s="187" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="E67" s="188"/>
       <c r="F67" s="93"/>
       <c r="G67" s="187" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="H67" s="93"/>
       <c r="I67" s="93"/>
@@ -13672,7 +13789,7 @@
       <c r="E68" s="188"/>
       <c r="F68" s="93"/>
       <c r="G68" s="187" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
       <c r="H68" s="93"/>
       <c r="I68" s="93"/>
@@ -13688,7 +13805,7 @@
       <c r="E69" s="188"/>
       <c r="F69" s="93"/>
       <c r="G69" s="187" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="H69" s="93"/>
       <c r="I69" s="93"/>
@@ -13715,12 +13832,12 @@
       <c r="B71" s="93"/>
       <c r="C71" s="93"/>
       <c r="D71" s="187" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="E71" s="188"/>
       <c r="F71" s="93"/>
       <c r="G71" s="187" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
       <c r="H71" s="93"/>
       <c r="I71" s="93"/>
@@ -13733,12 +13850,12 @@
       <c r="B72" s="93"/>
       <c r="C72" s="93"/>
       <c r="D72" s="187" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="E72" s="188"/>
       <c r="F72" s="93"/>
       <c r="G72" s="187" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="H72" s="93"/>
       <c r="I72" s="93"/>

</xml_diff>

<commit_message>
Module 5: The Call section live (peer table, value range, weight sliders, Buy below $189 / avoid above $218 badge); Milestone 5 memo filed with 16 new notes; workbook saved from Excel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UPr5EffsAtQC31pN59zdbP
</commit_message>
<xml_diff>
--- a/workbook/QD-HSY.xlsx
+++ b/workbook/QD-HSY.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21BFE91B-72D0-734F-853F-64047DFF48D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15720" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FrontPage" sheetId="1" r:id="rId1"/>
@@ -1511,7 +1511,7 @@
       <sz val="10"/>
       <color theme="10"/>
       <name val="Courier New"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
@@ -1587,7 +1587,7 @@
     <font>
       <sz val="10"/>
       <name val="Calibri"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -1644,7 +1644,7 @@
     <font>
       <sz val="10"/>
       <name val="Courier New"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
@@ -3198,6 +3198,51 @@
     </xf>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" xfId="8" applyFont="1"/>
     <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="9" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3212,51 +3257,6 @@
     </xf>
     <xf numFmtId="165" fontId="9" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -6920,21 +6920,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="403" t="s">
+      <c r="A1" s="418" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="403"/>
-      <c r="C1" s="403"/>
-      <c r="D1" s="403"/>
-      <c r="E1" s="403"/>
-      <c r="F1" s="403"/>
-      <c r="G1" s="403"/>
-      <c r="H1" s="404"/>
-      <c r="I1" s="404"/>
-      <c r="J1" s="404"/>
-      <c r="K1" s="404"/>
-      <c r="L1" s="404"/>
-      <c r="M1" s="404"/>
+      <c r="B1" s="418"/>
+      <c r="C1" s="418"/>
+      <c r="D1" s="418"/>
+      <c r="E1" s="418"/>
+      <c r="F1" s="418"/>
+      <c r="G1" s="418"/>
+      <c r="H1" s="419"/>
+      <c r="I1" s="419"/>
+      <c r="J1" s="419"/>
+      <c r="K1" s="419"/>
+      <c r="L1" s="419"/>
+      <c r="M1" s="419"/>
     </row>
     <row r="2" spans="1:18" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
@@ -6948,18 +6948,18 @@
       <c r="E2" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="405" t="s">
+      <c r="F2" s="420" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="405"/>
-      <c r="H2" s="406" t="s">
+      <c r="G2" s="420"/>
+      <c r="H2" s="421" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="406"/>
-      <c r="J2" s="406"/>
-      <c r="K2" s="406"/>
-      <c r="L2" s="406"/>
-      <c r="M2" s="406"/>
+      <c r="I2" s="421"/>
+      <c r="J2" s="421"/>
+      <c r="K2" s="421"/>
+      <c r="L2" s="421"/>
+      <c r="M2" s="421"/>
     </row>
     <row r="3" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
@@ -6973,8 +6973,8 @@
       <c r="E3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="407"/>
-      <c r="G3" s="407"/>
+      <c r="F3" s="422"/>
+      <c r="G3" s="422"/>
       <c r="H3" s="11" t="s">
         <v>8</v>
       </c>
@@ -7001,8 +7001,8 @@
       <c r="E4" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="408"/>
-      <c r="G4" s="408"/>
+      <c r="F4" s="417"/>
+      <c r="G4" s="417"/>
       <c r="H4" s="19" t="s">
         <v>13</v>
       </c>
@@ -7034,15 +7034,15 @@
       <c r="G5" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="H5" s="409" t="s">
+      <c r="H5" s="404" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="409"/>
-      <c r="K5" s="410" t="s">
+      <c r="I5" s="404"/>
+      <c r="K5" s="415" t="s">
         <v>20</v>
       </c>
-      <c r="L5" s="410"/>
-      <c r="M5" s="410"/>
+      <c r="L5" s="415"/>
+      <c r="M5" s="415"/>
     </row>
     <row r="6" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="30" t="s">
@@ -7179,17 +7179,17 @@
       </c>
     </row>
     <row r="10" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="411" t="s">
+      <c r="A10" s="414" t="s">
         <v>33</v>
       </c>
-      <c r="B10" s="411"/>
-      <c r="C10" s="411"/>
+      <c r="B10" s="414"/>
+      <c r="C10" s="414"/>
       <c r="D10" s="17"/>
-      <c r="E10" s="409" t="s">
+      <c r="E10" s="404" t="s">
         <v>34</v>
       </c>
-      <c r="F10" s="409"/>
-      <c r="G10" s="409"/>
+      <c r="F10" s="404"/>
+      <c r="G10" s="404"/>
       <c r="H10" s="35" t="s">
         <v>35</v>
       </c>
@@ -7207,15 +7207,15 @@
       </c>
     </row>
     <row r="11" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="412"/>
-      <c r="B11" s="412"/>
-      <c r="C11" s="412"/>
+      <c r="A11" s="410"/>
+      <c r="B11" s="410"/>
+      <c r="C11" s="410"/>
       <c r="D11" s="17"/>
-      <c r="E11" s="413" t="s">
+      <c r="E11" s="416" t="s">
         <v>37</v>
       </c>
-      <c r="F11" s="413"/>
-      <c r="G11" s="413"/>
+      <c r="F11" s="416"/>
+      <c r="G11" s="416"/>
       <c r="H11" s="51" t="s">
         <v>38</v>
       </c>
@@ -7233,17 +7233,17 @@
       </c>
     </row>
     <row r="12" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="412"/>
-      <c r="B12" s="412"/>
-      <c r="C12" s="412"/>
+      <c r="A12" s="410"/>
+      <c r="B12" s="410"/>
+      <c r="C12" s="410"/>
       <c r="D12" s="17"/>
-      <c r="E12" s="413"/>
-      <c r="F12" s="413"/>
-      <c r="G12" s="413"/>
-      <c r="H12" s="409" t="s">
+      <c r="E12" s="416"/>
+      <c r="F12" s="416"/>
+      <c r="G12" s="416"/>
+      <c r="H12" s="404" t="s">
         <v>40</v>
       </c>
-      <c r="I12" s="409"/>
+      <c r="I12" s="404"/>
       <c r="K12" s="55" t="s">
         <v>41</v>
       </c>
@@ -7255,13 +7255,13 @@
       </c>
     </row>
     <row r="13" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="412"/>
-      <c r="B13" s="412"/>
-      <c r="C13" s="412"/>
+      <c r="A13" s="410"/>
+      <c r="B13" s="410"/>
+      <c r="C13" s="410"/>
       <c r="D13" s="17"/>
-      <c r="E13" s="413"/>
-      <c r="F13" s="413"/>
-      <c r="G13" s="413"/>
+      <c r="E13" s="416"/>
+      <c r="F13" s="416"/>
+      <c r="G13" s="416"/>
       <c r="H13" s="58" t="s">
         <v>43</v>
       </c>
@@ -7282,13 +7282,13 @@
       </c>
     </row>
     <row r="14" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="412"/>
-      <c r="B14" s="412"/>
-      <c r="C14" s="412"/>
+      <c r="A14" s="410"/>
+      <c r="B14" s="410"/>
+      <c r="C14" s="410"/>
       <c r="D14" s="17"/>
-      <c r="E14" s="413"/>
-      <c r="F14" s="413"/>
-      <c r="G14" s="413"/>
+      <c r="E14" s="416"/>
+      <c r="F14" s="416"/>
+      <c r="G14" s="416"/>
       <c r="H14" s="58" t="s">
         <v>45</v>
       </c>
@@ -7309,17 +7309,17 @@
       </c>
     </row>
     <row r="15" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="409" t="s">
+      <c r="A15" s="404" t="s">
         <v>47</v>
       </c>
-      <c r="B15" s="409"/>
-      <c r="C15" s="409"/>
+      <c r="B15" s="404"/>
+      <c r="C15" s="404"/>
       <c r="D15" s="17"/>
-      <c r="E15" s="409" t="s">
+      <c r="E15" s="404" t="s">
         <v>48</v>
       </c>
-      <c r="F15" s="409"/>
-      <c r="G15" s="409"/>
+      <c r="F15" s="404"/>
+      <c r="G15" s="404"/>
       <c r="H15" s="58" t="s">
         <v>49</v>
       </c>
@@ -7340,15 +7340,15 @@
       </c>
     </row>
     <row r="16" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="414"/>
-      <c r="B16" s="414"/>
-      <c r="C16" s="414"/>
+      <c r="A16" s="413"/>
+      <c r="B16" s="413"/>
+      <c r="C16" s="413"/>
       <c r="D16" s="17"/>
-      <c r="E16" s="415" t="s">
+      <c r="E16" s="411" t="s">
         <v>51</v>
       </c>
-      <c r="F16" s="415"/>
-      <c r="G16" s="415"/>
+      <c r="F16" s="411"/>
+      <c r="G16" s="411"/>
       <c r="H16" s="58" t="s">
         <v>52</v>
       </c>
@@ -7376,13 +7376,13 @@
       <c r="R16" s="72"/>
     </row>
     <row r="17" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="414"/>
-      <c r="B17" s="414"/>
-      <c r="C17" s="414"/>
+      <c r="A17" s="413"/>
+      <c r="B17" s="413"/>
+      <c r="C17" s="413"/>
       <c r="D17" s="17"/>
-      <c r="E17" s="415"/>
-      <c r="F17" s="415"/>
-      <c r="G17" s="415"/>
+      <c r="E17" s="411"/>
+      <c r="F17" s="411"/>
+      <c r="G17" s="411"/>
       <c r="H17" s="58" t="s">
         <v>55</v>
       </c>
@@ -7410,13 +7410,13 @@
       <c r="R17" s="72"/>
     </row>
     <row r="18" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="414"/>
-      <c r="B18" s="414"/>
-      <c r="C18" s="414"/>
+      <c r="A18" s="413"/>
+      <c r="B18" s="413"/>
+      <c r="C18" s="413"/>
       <c r="D18" s="17"/>
-      <c r="E18" s="415"/>
-      <c r="F18" s="415"/>
-      <c r="G18" s="415"/>
+      <c r="E18" s="411"/>
+      <c r="F18" s="411"/>
+      <c r="G18" s="411"/>
       <c r="H18" s="65" t="s">
         <v>58</v>
       </c>
@@ -7444,21 +7444,21 @@
       <c r="R18" s="71"/>
     </row>
     <row r="19" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="411" t="s">
+      <c r="A19" s="414" t="s">
         <v>61</v>
       </c>
-      <c r="B19" s="411"/>
-      <c r="C19" s="411"/>
+      <c r="B19" s="414"/>
+      <c r="C19" s="414"/>
       <c r="D19" s="17"/>
-      <c r="E19" s="410" t="s">
+      <c r="E19" s="415" t="s">
         <v>62</v>
       </c>
-      <c r="F19" s="410"/>
-      <c r="G19" s="410"/>
-      <c r="H19" s="409" t="s">
+      <c r="F19" s="415"/>
+      <c r="G19" s="415"/>
+      <c r="H19" s="404" t="s">
         <v>63</v>
       </c>
-      <c r="I19" s="409"/>
+      <c r="I19" s="404"/>
       <c r="K19" s="60" t="s">
         <v>64</v>
       </c>
@@ -7479,17 +7479,17 @@
       <c r="R19" s="74"/>
     </row>
     <row r="20" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="412" t="s">
+      <c r="A20" s="410" t="s">
         <v>66</v>
       </c>
-      <c r="B20" s="412"/>
-      <c r="C20" s="412"/>
+      <c r="B20" s="410"/>
+      <c r="C20" s="410"/>
       <c r="D20" s="17"/>
-      <c r="E20" s="416" t="s">
+      <c r="E20" s="406" t="s">
         <v>67</v>
       </c>
-      <c r="F20" s="416"/>
-      <c r="G20" s="416"/>
+      <c r="F20" s="406"/>
+      <c r="G20" s="406"/>
       <c r="H20" s="60" t="s">
         <v>68</v>
       </c>
@@ -7517,15 +7517,15 @@
       <c r="R20" s="74"/>
     </row>
     <row r="21" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="412"/>
-      <c r="B21" s="412"/>
-      <c r="C21" s="412"/>
+      <c r="A21" s="410"/>
+      <c r="B21" s="410"/>
+      <c r="C21" s="410"/>
       <c r="D21" s="17"/>
-      <c r="E21" s="417" t="s">
+      <c r="E21" s="408" t="s">
         <v>71</v>
       </c>
-      <c r="F21" s="417"/>
-      <c r="G21" s="417"/>
+      <c r="F21" s="408"/>
+      <c r="G21" s="408"/>
       <c r="H21" s="58" t="s">
         <v>72</v>
       </c>
@@ -7553,15 +7553,15 @@
       <c r="R21" s="78"/>
     </row>
     <row r="22" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="412"/>
-      <c r="B22" s="412"/>
-      <c r="C22" s="412"/>
+      <c r="A22" s="410"/>
+      <c r="B22" s="410"/>
+      <c r="C22" s="410"/>
       <c r="D22" s="17"/>
-      <c r="E22" s="415" t="s">
+      <c r="E22" s="411" t="s">
         <v>75</v>
       </c>
-      <c r="F22" s="415"/>
-      <c r="G22" s="415"/>
+      <c r="F22" s="411"/>
+      <c r="G22" s="411"/>
       <c r="H22" s="58" t="s">
         <v>76</v>
       </c>
@@ -7589,15 +7589,15 @@
       <c r="R22" s="71"/>
     </row>
     <row r="23" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="412"/>
-      <c r="B23" s="412"/>
-      <c r="C23" s="412"/>
+      <c r="A23" s="410"/>
+      <c r="B23" s="410"/>
+      <c r="C23" s="410"/>
       <c r="D23" s="17"/>
-      <c r="E23" s="418" t="s">
+      <c r="E23" s="412" t="s">
         <v>79</v>
       </c>
-      <c r="F23" s="418"/>
-      <c r="G23" s="418"/>
+      <c r="F23" s="412"/>
+      <c r="G23" s="412"/>
       <c r="H23" s="58" t="s">
         <v>80</v>
       </c>
@@ -7625,17 +7625,17 @@
       <c r="R23" s="74"/>
     </row>
     <row r="24" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="409" t="s">
+      <c r="A24" s="404" t="s">
         <v>83</v>
       </c>
-      <c r="B24" s="409"/>
-      <c r="C24" s="409"/>
+      <c r="B24" s="404"/>
+      <c r="C24" s="404"/>
       <c r="D24" s="17"/>
-      <c r="E24" s="416" t="s">
+      <c r="E24" s="406" t="s">
         <v>67</v>
       </c>
-      <c r="F24" s="416"/>
-      <c r="G24" s="416"/>
+      <c r="F24" s="406"/>
+      <c r="G24" s="406"/>
       <c r="H24" s="58" t="s">
         <v>84</v>
       </c>
@@ -7666,16 +7666,16 @@
       <c r="A25" s="79" t="s">
         <v>87</v>
       </c>
-      <c r="B25" s="421" t="s">
+      <c r="B25" s="407" t="s">
         <v>88</v>
       </c>
-      <c r="C25" s="421"/>
+      <c r="C25" s="407"/>
       <c r="D25" s="17"/>
-      <c r="E25" s="417" t="s">
+      <c r="E25" s="408" t="s">
         <v>71</v>
       </c>
-      <c r="F25" s="417"/>
-      <c r="G25" s="417"/>
+      <c r="F25" s="408"/>
+      <c r="G25" s="408"/>
       <c r="H25" s="58" t="s">
         <v>89</v>
       </c>
@@ -7688,29 +7688,29 @@
       <c r="A26" s="79" t="s">
         <v>90</v>
       </c>
-      <c r="B26" s="422" t="s">
+      <c r="B26" s="409" t="s">
         <v>91</v>
       </c>
-      <c r="C26" s="422"/>
+      <c r="C26" s="409"/>
       <c r="D26" s="17"/>
-      <c r="E26" s="417" t="s">
+      <c r="E26" s="408" t="s">
         <v>75</v>
       </c>
-      <c r="F26" s="417"/>
-      <c r="G26" s="417"/>
+      <c r="F26" s="408"/>
+      <c r="G26" s="408"/>
       <c r="H26" s="58"/>
       <c r="I26" s="59"/>
     </row>
     <row r="27" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="419" t="s">
+      <c r="A27" s="403" t="s">
         <v>92</v>
       </c>
-      <c r="B27" s="419"/>
-      <c r="C27" s="419"/>
-      <c r="D27" s="419"/>
-      <c r="E27" s="419"/>
-      <c r="F27" s="419"/>
-      <c r="G27" s="419"/>
+      <c r="B27" s="403"/>
+      <c r="C27" s="403"/>
+      <c r="D27" s="403"/>
+      <c r="E27" s="403"/>
+      <c r="F27" s="403"/>
+      <c r="G27" s="403"/>
       <c r="H27" s="65"/>
       <c r="I27" s="54"/>
     </row>
@@ -7722,15 +7722,15 @@
       <c r="E28" s="81"/>
       <c r="F28" s="81"/>
       <c r="G28" s="83"/>
-      <c r="H28" s="409" t="s">
+      <c r="H28" s="404" t="s">
         <v>93</v>
       </c>
-      <c r="I28" s="409"/>
-      <c r="K28" s="409" t="s">
+      <c r="I28" s="404"/>
+      <c r="K28" s="404" t="s">
         <v>94</v>
       </c>
-      <c r="L28" s="409"/>
-      <c r="M28" s="409"/>
+      <c r="L28" s="404"/>
+      <c r="M28" s="404"/>
     </row>
     <row r="29" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="80"/>
@@ -7835,14 +7835,14 @@
       <c r="E33" s="81"/>
       <c r="F33" s="81"/>
       <c r="G33" s="83"/>
-      <c r="H33" s="420" t="s">
+      <c r="H33" s="405" t="s">
         <v>103</v>
       </c>
-      <c r="I33" s="420"/>
-      <c r="J33" s="420"/>
-      <c r="K33" s="420"/>
-      <c r="L33" s="420"/>
-      <c r="M33" s="420"/>
+      <c r="I33" s="405"/>
+      <c r="J33" s="405"/>
+      <c r="K33" s="405"/>
+      <c r="L33" s="405"/>
+      <c r="M33" s="405"/>
     </row>
     <row r="34" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="80"/>
@@ -8095,6 +8095,31 @@
     <row r="69" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="35">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="H1:M1"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="H2:M2"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="K5:M5"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="A11:C14"/>
+    <mergeCell ref="E11:G14"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="A16:C18"/>
+    <mergeCell ref="E16:G18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="A20:C23"/>
+    <mergeCell ref="E20:G20"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="E23:G23"/>
     <mergeCell ref="A27:G27"/>
     <mergeCell ref="H28:I28"/>
     <mergeCell ref="K28:M28"/>
@@ -8105,31 +8130,6 @@
     <mergeCell ref="E25:G25"/>
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="E26:G26"/>
-    <mergeCell ref="A20:C23"/>
-    <mergeCell ref="E20:G20"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="E22:G22"/>
-    <mergeCell ref="E23:G23"/>
-    <mergeCell ref="A16:C18"/>
-    <mergeCell ref="E16:G18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="A11:C14"/>
-    <mergeCell ref="E11:G14"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="E15:G15"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="K5:M5"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="H1:M1"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="H2:M2"/>
-    <mergeCell ref="F3:G3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.45" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
@@ -11376,7 +11376,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="E115" s="226">
-        <f t="dataTable" ref="E115:I119" dt2D="1" dtr="1" r1="C46" r2="H6"/>
+        <f t="dataTable" ref="E115:I119" dt2D="1" dtr="1" r1="C46" r2="H6" ca="1"/>
         <v>162.91322629821829</v>
       </c>
       <c r="F115" s="226">
@@ -11397,7 +11397,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="M115" s="228">
-        <f t="dataTable" ref="M115:Q119" dt2D="1" dtr="1" r1="C46" r2="H6" ca="1"/>
+        <f t="dataTable" ref="M115:Q119" dt2D="1" dtr="1" r1="C46" r2="H6"/>
         <v>12.356524467110722</v>
       </c>
       <c r="N115" s="228">

</xml_diff>